<commit_message>
Add category 2: functional status
Molenaar 2023 (Cochrane, prehabilitation/functional capacity - native PubMed
syntax), McDonald 2023 (JCSM, physical function endpoints in cachexia trials),
Scheepers 2020 (Haematologica, geriatric assessment in older patients).

Records the cross-cutting finding that none of the three search on the outcome:
functional status is applied at screening, not retrieved on.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 OC treatment (general)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Functional status" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Functional status'!$A$2:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -972,4 +974,469 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>02. Functional status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1st author / year</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Impact factor</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Purpose of the study</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PICO</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - PubMed / MEDLINE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Embase</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Web of Science</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="713" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Prehabilitation versus no prehabilitation to improve functional capacity, reduce postoperative complications and improve quality of life in colorectal cancer surgery</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Molenaar CJ, 2023</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>To determine the effects of multimodal prehabilitation programmes on functional capacity, postoperative complications and quality of life in adults undergoing surgery for colorectal cancer. Functional capacity (6-minute walk test, VO2 peak, handgrip strength) is the lead outcome, yet no functional-capacity terms appear anywhere in the search - the strategy is population AND surgery AND (each of four intervention components), run as four separate intersections.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>P: Adults with non-metastatic colorectal cancer scheduled for surgery.
+I: Multimodal prehabilitation (&gt;= two preoperative components from exercise,
+   nutrition, psychological support, smoking cessation).
+C: No prehabilitation (usual preoperative care).
+O: Functional capacity (6-minute walk test, VO2 peak, handgrip strength);
+   postoperative complications and mortality; health-related quality of life;
+   hospital length of stay.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>[MEDLINE searched January 2021, reported in native PubMed syntax.
+Appendix 2, verbatim:]
+#1 Search ((("Colorectal Neoplasms"[Mesh] OR (("Neoplasms"[Mesh] OR carcinoma*[tiab]
+   OR neoplas*[tiab] OR tumour*[tiab] OR tumor*[tiab] OR cancer*[tiab] OR cancer[sb]
+   OR oncolog*[tiab] OR malignan*[tiab] OR carcinogen*[tiab] OR oncogen*[tiab]
+   AND (colorectal*[tiab] OR colon*[tiab] OR rectal*[tiab])))))
+#2 Search "surgery"[Subheading] OR "Surgical Procedures, Operative"[Mesh]
+   OR "Surgeons"[Mesh] OR "Perioperative Period"[Mesh] OR "Perioperative Care"[Mesh]
+   OR "Preoperative Care"[Mesh] OR "Perioperative Care"[Mesh:NoExp] OR surger*[tiab]
+   OR surgical*[tiab] OR surgeon*[tiab] OR operation*[tiab] OR operative*[tiab]
+   OR perioperati*[tiab] OR preoperati*[tiab] OR pre operati*[tiab]
+   OR peri operati*[tiab] OR anesthe*[tiab] OR anaesthe*[tiab] OR incisi*[tiab]
+   OR excisi*[tiab] OR invasive*[tiab] OR Prehab*[tiab]
+#3 Search (#1 AND #2)
+#4 Search "Exercise Therapy"[Mesh] OR "Exercise"[Mesh] OR "Physical Education and
+   Training"[Mesh] OR "Exercise Movement Techniques"[Mesh] OR remedial exercis*[tiab]
+   OR exercise therap*[tiab] OR rehabilitation exercis*[tiab] OR exercis*[tiab]
+   OR physical activit*[tiab] OR physical exercis*[tiab] OR aerobic exercis*[tiab]
+   OR exercise training*[tiab] OR isometric exercis*[tiab]
+   OR (Physical Education*[tiab] AND training) OR exercise movement Techni*[tiab]
+#5 Search (Psychosocial[tiab] OR psychologic*[tiab] OR "Cognitive Behavioral
+   Therapy"[Mesh] OR cognitive behav*[tiab] OR cognitive psychotherap*[tiab]
+   OR (cogniti*[tiab] AND therap*[tiab]) OR psychoeducation[tiab]
+   OR psycho-education[tiab])
+#6 Search "Nutrition Therapy"[Mesh] OR "Nutritional Status"[Mesh]
+   OR medical nutrition therap*[tiab] OR nutrition therap*[tiab] OR nutrition[tiab]
+#7 Search "Smoking Cessation"[Mesh] OR "Smoking"[Mesh] OR "Tobacco Use Cessation"[Mesh]
+   OR stopping smoking[tiab] OR smoking cessation*[tiab] OR giving up smoking*[tiab]
+   OR quitting smoking[tiab] smoking[tiab] OR smoking behav*[tiab]
+   OR smoking habit*[tiab] OR tobacco cessation[tiab]
+#8  Search #3 AND #4
+#9  Search #3 AND #5
+#10 Search #3 AND #6
+#11 Search #3 AND #7
+Note: no functional-capacity, physical-function or activities-of-daily-living terms
+appear in the strategy; the outcome was applied at screening.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>[Embase via Ovid, 1974 to 2021 week 4. Appendix 3, verbatim:]
+#1  exp colorectal tumor/
+#2  exp neoplasm/
+#3  (carcinoma* or neoplasm* or tumour* or tumor* or cancer* or oncolog* or malignan*
+    or carcinogen* or oncogen*).ab,ti.
+#4  2 or 3
+#5  (colorectal* or colon* or rectal*).ab,ti.
+#6  4 and 5
+#7  1 or 6
+#8  exp surgery/
+#9  exp surgeon/
+#10 exp perioperative period/
+#11 exp preoperative period/
+#12 (surger* or surgical* or surgeon* or operation* or operative* or perioperati*
+    or preoperati* or pre operati* or peri operati* or anesthe* or anaesthe*
+    or incisi* or excisi* or invasive* or Prehab*).ab,ti.
+#13 8 or 9 or 10 or 11 or 12
+#14 (remedial exercis* or exercise therap* or rehabilitation exercis* or exercis*
+    or physical activit* or physical exercis* or aerobic exercis* or exercise training*
+    or isometric exercis* or exercise movement techni*).ab,ti.
+#15 exp kinesiotherapy/
+#16 14 or 15
+#17 7 and 13 and 16
+#18 exp diet therapy/
+#19 exp nutritional status/
+#20 (medical nutrition therap* or nutrition therap* or nutrition).ab,ti.
+#21 18 or 19 or 20
+#22 7 and 13 and 21
+#23 exp cognitive behavioral therapy/
+#24 (Psychosocial or psychologic* or cognitive behav* or cognitive psychotherap*
+    or psychoeducation or psycho-education).ab,ti.
+#25 (cogniti* and therap*).ab,ti.
+#26 23 or 24 or 25
+#27 7 and 13 and 26
+#28 exp smoking cessation/
+#29 exp smoking/
+#30 (stopping smoking or smoking cessation* or giving up smoking* or quitting smoking
+    or smoking or smoking behav* or smoking habit* or tobacco cessation).ab,ti.
+#31 28 or 29 or 30
+#32 7 and 13 and 31</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were CENTRAL (Cochrane Library, 2021 week 4),
+MEDLINE (Ovid, 1950 to 2021 week 4), Embase (Ovid, 1974 to 2021 week 4) and PsycINFO
+(EBSCOhost, 1967 to 2021 week 4), plus ClinicalTrials.gov, Google Scholar, the
+Netherlands Trial Register and WHO ICTRP (to March 2021). Web of Science was not used.
+[PsycINFO strategy (Appendix 4) shows the same shape in EBSCOhost syntax:
+S1 DE "Neoplasms"; S2 TI colorectal cancer* OR AB colorectal cancer*; S3 DE "Surgery";
+S4 TI surger* OR AB surger*; S5 S1 OR S2; S6 S3 OR S4; S7 S5 AND S6;
+S8 DE "Psychosocial Rehabilitation"; ... S24 S7 AND S23]</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD013259.pub3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="760" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Physical function endpoints in cancer cachexia clinical trials: Systematic Review 1 of the cachexia endpoints series</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>McDonald J, 2023</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Cachexia, Sarcopenia and Muscle</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>9.4 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>To assess the frequency and diversity of physical function endpoints used in cancer cachexia clinical trials, and how often they change with intervention. Included as an exemplar of a librarian-built Ovid strategy in which physical function is the whole point of the review yet appears nowhere in the search: retrieval is population (cancer) AND condition (cachexia) AND study design, with physical function applied as an eligibility criterion.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>P: Adults (&gt;= 18 years) with cancer cachexia.
+I: Any cachexia intervention lasting more than 14 days (nutritional, pharmacological,
+   exercise, multimodal), in controlled trials with more than 40 participants.
+C: Control arm as defined by each trial.
+O: Physical function endpoints - handgrip strength, 6-minute walk test, timed
+   up-and-go, physical activity, patient-reported physical function.</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[Not searched as PubMed. Ovid MEDLINE(R) ALL 1946 to 1 July 2021; search run
+2 June 2021 by a research librarian, University of Oslo. Appendix S1, verbatim:]
+1  exp Neoplasms/ or (neoplasm* or cancer* or tumor* or tumour* or oncol* or malign*
+   or carcinom* or adenocarcinom* or adenoma or metasta*).ti,ab,kf.
+2  Cachexia/ or Emaciation/ or Malnutrition/ or Starvation/ or Wasting syndrome/
+   or Thinness/ or Sarcopenia/ or Anorexia/ or *Weight Loss/
+3  and/1-2
+4  ((cachexia or cachexic or anorexia or anorectic or emaciat* or malnutrition or
+   underweight or starvation* or thiness or leanness or sarcopenia or wasting syndrome*
+   or wasting disease* or weightloss* or ((appetite* or weight) adj2 (loss or loosing
+   or losing))) adj4 (neoplasm* or cancer* or tumor* or tumour* or oncol* or malign*
+   or carcinom* or adenocarcinom* or adenoma or metasta*)).ti,ab,kf.
+5  ((cachexia or cachexic or anorexia or ... [same term list as line 4] ...) and
+   (neoplasm* or cancer* or tumor* or tumour* or oncol* or malign* or carcinom*
+   or adenocarcinom* or adenoma or metasta*)).ti.
+6  or/3-5
+7  randomized controlled trial.pt.
+8  controlled clinical trial.pt.
+9  randomized.ab.
+10 placebo.ab.
+11 drug therapy.fs.
+12 randomly.ab.
+13 trial.ab.
+14 groups.ab.
+15 or/7-14
+16 exp animals/ not humans.sh.
+17 15 not 16
+18 6 and 17
+19 limit 18 to yr="1990 -Current"
+20 cohort studies/ or follow-up studies/ or longitudinal studies/ or "national
+   longitudinal study of adolescent health"/ or prospective studies/
+   or retrospective studies/
+21 (cohort* or longitudinal or prospective* or retrospective*).tw.
+22 or/20-21
+23 and/6,22
+24 limit 23 to yr="1990 -Current"
+25 24 not 19
+26 19 or 24
+Note: no physical-function terms appear in the strategy.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>[Embase Classic+Embase 1947 to 1 July 2021 via Ovid; run 2 June 2021.
+Appendix S1, verbatim (population/condition block; the design block is a long
+standard Embase RCT/observational filter, lines 7-45):]
+1  exp neoplasm/ or (neoplasm* or cancer* or tumor* or tumour* or oncol* or malign*
+   or carcinom* or adenocarcinom* or adenoma or metasta*).ti,ab,kw.
+2  cachexia/ or emaciation/ or *malnutrition/ or starvation/ or wasting syndrome/
+   or *anorexia/ or sarcopenia/ or *weight loss/
+3  and/1-2
+4  ((cachexia or cachexic or anorexia or anorectic or emaciat* or malnutrition or
+   underweight or starvation* or thiness or leanness or sarcopenia or wasting syndrome*
+   or wasting disease* or weightloss* or ((appetite* or weight) adj2 (loss or loosing
+   or losing))) adj3 (neoplasm* or cancer* or tumor* or tumour* or oncol* or malign*
+   or carcinom* or adenocarcinom* or adenoma or metasta*)).ti,ab,kw.
+5  ((cachexia or cachexic or anorexia or ... [same term list] ...) and (neoplasm*
+   or cancer* or tumor* or tumour* or oncol* or malign* or carcinom* or adenocarcinom*
+   or adenoma or metasta*)).ti.
+6  or/3-5
+7-25   [Embase RCT filter: Randomized controlled trial/; Controlled clinical trial/;
+       random$.ti,ab.; randomization/; intermethod comparison/; placebo.ti,ab.;
+       (compare or compared or comparison).ti.; ((evaluated or evaluate or evaluating
+       or assessed or assess) and (compare or compared or comparing or comparison)).ab.;
+       (open adj label).ti,ab.; ((double or single or doubly or singly) adj (blind or
+       blinded or blindly)).ti,ab.; double blind procedure/; parallel group$1.ti,ab.;
+       (crossover or cross over).ti,ab.; ((assign$ or match or matched or allocation)
+       adj5 (alternate or group$1 or intervention$1 or patient$1 or subject$1 or
+       participant$1)).ti,ab.; (assigned or allocated).ti,ab.; (controlled adj7 (study
+       or design or trial)).ti,ab.; (volunteer or volunteers).ti,ab.; human experiment/;
+       trial.ti.]
+26 or/7-25
+27-39  [exclusion filter for non-trial designs and animal studies]
+40 or/27-39
+41 26 not 40
+42 and/6,41
+43 limit 42 to yr="1990 -Current"
+44 limit 43 to conference abstracts
+45 43 not 44
+46 cohort analysis/ or follow up/ or longitudinal study/ or "national longitudinal
+   study of adolescent health"/ or prospective study/ or retrospective study/
+47 ((cohort adj (study or studies)) or cohort analy* or longitudinal).tw.
+48 or/46-47
+49 and/6,48
+50 limit 49 to yr="1990 -Current"
+51 limit 50 to conference abstracts
+52 50 not 51
+53 52 not 45</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were MEDLINE (Ovid), Embase (Ovid) and the Cochrane
+Central Register of Controlled Trials, 1990 to 2 June 2021. Web of Science was not used.
+[CENTRAL strategy, verbatim:
+#1 [mh Neoplasms]
+#2 ((neoplasm* or cancer* or tumor* or tumour* or oncol* or malign* or carcinom*
+   or adenocarcinom* or adenoma or metasta*)):ti,ab,kw
+#3 #1 or #2
+#4 [mh Cachexia] or [mh ^Emaciation] or [mh ^Malnutrition] or [mh Starvation]
+   or [mh ^"Wasting syndrome"] or [mh Thinness] or [mh Sarcopenia] or [mh Anorexia]
+#5 MeSH descriptor: [Weight Loss] this term only
+#6 #3 and (#4 or #5)
+#7 (((cachexia or cachexic or anorexia or anorectic or emaciat* or malnutrition or
+   underweight or starvation* or thiness or leanness or sarcopenia or "wasting syndrome"
+   or "wasting syndromes" or "wasting disease" or "wasting diseases" or weightloss*
+   or ((appetite* or weight) near/2 (loss or loosing or losing))) near/3 (neoplasm*
+   or cancer* or tumor* or tumour* or oncol* or malign* or carcinom* or adenocarcinom*
+   or adenoma or metasta*))):ti,ab,kw
+#8 [same term list combined with AND rather than near/3]:ti
+#9 #6 or #7 or #8 with Publication Year from 1990 to 2021, in Trials]</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jcsm.13321</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="368" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Geriatric assessment in older patients with a hematologic malignancy: a systematic review</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Scheepers ERM, 2020</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Haematologica</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>8.2 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>To summarise what geriatric assessment adds in older patients with a haematologic malignancy - the prevalence of geriatric impairments (including impaired activities of daily living) and their association with treatment decisions, chemotherapy toxicity, healthcare utilisation, physical functioning after treatment, quality of life and mortality. Included as the one review of the three restricted to older adults, and because it shows the common substitute for a functional-status block: retrieval on "frailty OR geriatric assessment", with functional status captured only downstream.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>P: Older patients with a haematologic malignancy (leukaemia, lymphoma, multiple
+   myeloma, myelodysplastic syndrome, myeloproliferative neoplasms).
+I: Geriatric assessment (any validated multidomain instrument), applied before or
+   during antineoplastic treatment.
+C: No geriatric assessment, or patients without the impairment identified.
+O: Prevalence of geriatric impairments; treatment decision-making; chemotherapy
+   toxicity; healthcare utilisation; physical functioning after treatment; quality of
+   life; mortality.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>[MEDLINE, searched 4 March 2019 and updated 20 January 2020; results limited to
+studies published after 1 January 2013. Reported in native PubMed syntax as a single
+string in the Methods, verbatim:]
+((("Hematologic Neoplasms"[Mesh] OR "Leukemia"[Mesh] OR "Lymphoma"[Mesh]
+OR "Multiple Myeloma"[Mesh] OR "Myelodysplastic Syndromes"[Mesh] OR leukemia[tiab]
+OR leukaemia[tiab] OR lymphoma*[tiab] OR hodgkin*[tiab] OR non-hodgkin*[tiab]
+OR (multiple myeloma[tiab]) OR myelodysplas*[tiab] OR (haematolog* AND malignan*[tiab])
+OR (hematolog* AND malignan*[tiab]) OR (myeloid[tiab] OR lymphoid[tiab]
+AND neoplas*[tiab]) OR myeloproliferative[tiab] OR (plasma cell neoplas*[tiab])
+OR plasma cell dyscrasia*[tiab] OR (myeloid[tiab] AND sarcoma*[tiab])
+OR waldenstrom[tiab] OR myelofibrosis[tiab] OR mastocystosis[tiab]
+OR (polycyth* AND vera[tiab]) OR (essential AND thrombocyt*[tiab])))
+AND (("frailty"[All Fields] OR "Geriatric Assessment"[Mesh] OR frail*[tiab]
+OR vulnerabl*[tiab] OR geriatric assessment*[tiab] OR geriatric*[tiab]))
+No age or language limitations were applied.
+Note: functional status enters only through "Geriatric Assessment"[Mesh] and
+frail*/vulnerabl*; there are no ADL, IADL or physical-function terms.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Searched, but no separate Embase string was published. The Methods state that "the
+following search was performed ... in both MEDLINE and EMBASE" and then give one
+strategy in PubMed syntax; the Emtree translation is not reported. Yield is reported
+by database (832 citations from MEDLINE, 3797 from EMBASE, 4629 total).</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were MEDLINE and EMBASE only, supplemented by
+cross-referencing the reference lists of included studies and by carrying forward
+eligible studies from the earlier 2013 review by Hamaker et al.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3324/haematol.2019.245803</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add category 3: cognition
Treanor 2016 (Cochrane, six-database cognition block incl. native PubMed),
Lawrie 2019 (Cochrane, cognit* embedded in a late-effects adjacency),
Jim 2012 (JCO, seven unstructured keyword pairings).

Flags two apparent typographical slips in Treanor's published PubMed appendix
(#19 combines with #17 not #18; #26 omits #25).
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 OC treatment (general)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Functional status" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Cognition" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Functional status'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 Cognition'!$A$2:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1439,4 +1441,521 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>03. Cognition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1st author / year</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Impact factor</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Purpose of the study</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PICO</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - PubMed / MEDLINE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Embase</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Web of Science</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="760" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Non-pharmacological interventions for cognitive impairment due to systemic cancer treatment</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Treanor CJ, 2016</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>To evaluate the cognitive effects, non-cognitive effects, duration and safety of non-pharmacological interventions aimed at maintaining cognitive function or ameliorating cognitive impairment resulting from cancer or systemic cancer treatment. The most complete cognition search block found in this exercise: one core adjacency statement generates the cross-product of nine cognition terms and ten impairment terms, sitting alongside five controlled-vocabulary terms and a chemo-fog/chemo-brain phrase. Reproduced in six database syntaxes, including a native PubMed version.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>P: Adults with cancer receiving or having received systemic cancer treatment
+   (chemotherapy or hormonal therapy, alone or with other treatments).
+I: Non-pharmacological interventions targeting cognitive function (compensatory
+   strategy training, cognitive rehabilitation/training, exercise, mind-body).
+C: Wait-list, usual care, attention control or an alternative non-pharmacological
+   intervention.
+O: Objective and subjective cognitive function; non-cognitive effects (quality of
+   life, physical and psychological well-being, fatigue, mood); duration of effect;
+   adverse events.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>[PubMed searched natively (via NCBI); 1980 to 29 September 2015. Appendix 6, verbatim:]
+#1  neoplasm*[MeSH Terms]
+#2  (cancer* or neoplas* or tumor* or tumour* or carcinoma* or adenocarcinoma*
+    or malignan* or leukemia* or leukaemia*)
+#3  #1 or #2
+#4  cognition disorders[MeSH Terms]
+#5  neurobehavioral manifestations[MeSH Terms]
+#6  mental processes[MeSH Terms]
+#7  neuropsychological tests[MeSH Terms]
+#8  attention[MeSH Terms]
+#9  "chemo* fog"
+#10 "chemo* brain"
+#11 (("cognit* deficit*") OR "cognit* declin*" OR "cognit* disorder*"
+    OR "cognit* function*" OR "cognit* dysfunction*" OR "cognit* impair*"
+    OR "cognit* decrement*" OR "cognit* problem*" OR "cognit* sequelae*")
+#12 (("memory deficit*") OR "memory declin*" OR "memory disorder*"
+    OR "memory function*" OR "memory dysfunction*" OR "memory impair*"
+    OR "memory decrement*" OR "memory problem*" OR "memory sequelae*")
+#13 [same nine-suffix pattern applied to neurobehavior*]
+#14 [same nine-suffix pattern applied to neurobehaviour*]
+#15 [same nine-suffix pattern applied to "problem solving"]
+#16 [same nine-suffix pattern applied to attention]
+#17 [same nine-suffix pattern applied to concentrat*]
+#18 #4 or #5 or #6 or #7 or #8 or #9 or #10 or #11 or #12 or #13 or #14 or #15
+    or #16 or #17
+#19 #3 and #17
+#20 randomized controlled trial[pt]
+#21 controlled clinical trial[pt]
+#22 randomized[tiab]
+#23 placebo[tiab]
+#24 clinical trials as topic[mesh:noexp]
+#25 randomly[tiab]
+#26 #20 or #21 or #22 or #23 or #24
+#27 animals [mh] NOT humans [mh]
+#28 #26 NOT #27
+#29 #19 AND #28
+Note as printed: line #19 combines #3 with #17 (concentrat* only) rather than with the
+full #18 union, and line #26 omits #25 - both appear to be typographical slips in the
+published appendix. Reproduce with care.
+[The Ovid MEDLINE version, Appendix 2, is the cleaner statement of the same concept:
+1  exp Neoplasms/
+2  (cancer* or neoplas* or tumor* or tumour* or carcinoma* or adenocarcinoma*
+   or malignan* or leukemia* or leukaemia*).mp
+3  1 or 2
+4  exp Cognition Disorders/
+5  exp Neurobehavioral Manifestations/
+6  exp Mental Processes/
+7  exp Neuropsychological Tests/
+8  Attention/
+9  (chemo* adj5 (fog or brain)).mp.
+10 ((cognit* or neurocognit* or neuropsycholog* or memory or neurobehavior*
+   or neurobehaviour* or problem solving or attention or concentrat*) adj5
+   (deficit* or declin* or disorder* or function* or dysfunction* or impair*
+   or decrement* or disturb* or problem* or sequelae*)).mp.
+11 4 or 5 or 6 or 7 or 8 or 9 or 10
+12 3 and 11
+13 randomized controlled trial.pt.
+14 controlled clinical trial.pt.
+15 randomized.ab.
+16 placebo.ab.
+17 clinical trials as topic.sh.
+18 randomly.ab.
+19 trial.ti.
+20 13 or 14 or 15 or 16 or 17 or 18 or 19
+21 12 and 20
+22 exp animals/ not humans.sh.
+23 21 not 22]</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>[Embase via OvidSP, 1980 to 29 September 2015. Appendix 3, verbatim:]
+1  exp neoplasm/
+2  (cancer* or neoplas* or tumor* or tumour* or carcinoma* or adenocarcinoma*
+   or malignan* or leukemia* or leukaemia*).mp.
+3  1 or 2
+4  exp cognitive defect/
+5  cognition/
+6  neuropsychological test/
+7  attention/
+8  (chemo* adj5 (fog or brain)).mp.
+9  ((cognit* or neurocognit* or neuropsycholog* or memory or neurobehavior*
+   or neurobehaviour* or problem solving or attention or concentrat*) adj5
+   (deficit* or declin* or disorder* or function* or dysfunction* or impair*
+   or decrement* or disturb* or problem* or sequelae*)).mp.
+10 4 or 5 or 6 or 7 or 8 or 9
+11 3 and 10
+12 crossover procedure/
+13 double-blind procedure/
+14 randomized controlled trial/
+15 single-blind procedure/
+16 random*.mp.
+17 factorial*.mp.
+18 (crossover* or cross over* or cross-over*).mp.
+19 placebo*.mp.
+20 (double* adj blind*).mp.
+21 (singl* adj blind*).mp.
+22 assign*.mp.
+23 allocat*.mp.
+24 volunteer*.mp.
+25 12 or 13 or 14 or 15 or 16 or 17 or 18 or 19 or 20 or 21 or 22 or 23 or 24
+26 11 and 25
+key: mp = title, abstract, subject headings, heading word, drug trade name, original
+title, device manufacturer, drug manufacturer, device trade name, keyword.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were CENTRAL, MEDLINE (OvidSP), Embase (OvidSP),
+PsycINFO (OvidSP), CINAHL (EBSCO) and PubMed, 1980 to 29 September 2015, plus trial
+registries and grey literature (theses, dissertations, conference proceedings).
+Web of Science was not used.
+[The CINAHL version (Appendix 5, EBSCOhost syntax) is the closest analogue to a
+Web of Science-style proximity search and may be the most useful template if you
+do add Web of Science:
+S13 (MH "Cognition Disorders+") S14 (MH "Neurobehavioral Manifestations+")
+S15 (MH "Mental Processes+") S16 (MH "Neuropsychological Tests+") S17 (MH "Attention+")
+S18 "chemo*" S19 "fog" S20 "brain" S21 (S19 or S20) S22 (S18 N2 S21)
+S23 "cognit*" S24 "neurocognit*" S25 "neuropsycholog*" S26 "memory"
+S27 "neurobehavior*" S28 "neurobehaviour*" S29 "problem solving" S30 "attention"
+S31 "concentrat*" S32 (S23 or S24 or S25 or S26 or S27 or S28 or S29 or S30)
+S33 "deficit*" S34 "declin*" S35 "disorder*" S36 "function*" S37 "dysfunction*"
+S38 "impair*" S39 "decrement*" S40 "disturb*" S41 "problem*" S42 "sequelae*"
+S43 (S33 or S34 or ... or S42) S44 (S32 N2 S43)
+S45 (S13 or S14 or S15 or S16 or S17 or S22 or S44) S46 (S12 and S45)
+S47 MH "Randomized controlled trials" S48 MH "Clinical trials" S49 MH "Placebos"
+S50 (S47 or S48 or S49) S51 (S44 and S50)]</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD011325.pub2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="655.5" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Long-term neurocognitive and other side effects of radiotherapy, with or without chemotherapy, for glioma</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Lawrie TA, 2019</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>To evaluate the long-term (at least two years after diagnosis) neurocognitive and other side effects of radiotherapy, with or without chemotherapy, in people with glioma, and to write a brief economic commentary. Included as an exemplar of the alternative structure: rather than a stand-alone cognition block, cognit* is one term inside a generic late-effects adjacency, so cognition is retrieved as a species of treatment harm.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>P: People with glioma (any grade), followed at least two years from diagnosis.
+I: Radiotherapy, with or without chemotherapy.
+C: No radiotherapy, or a different type/dose/schedule of radiotherapy.
+O: Long-term neurocognitive function (primary); other late side effects; quality of
+   life; survival; costs (brief economic commentary).</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[Not searched as PubMed. MEDLINE via Ovid, 1946 to October week 5 2018; searched
+16 February 2018 and updated 14 November 2018. Appendix 1, verbatim:]
+1  exp Glioma/
+2  (glioma* or astrocytoma* or medulloblastoma* or ependymoma* or craniophyrangioma*
+   or oligodendroglioma* or glioblastoma* or GBM*).ti,ab.
+3  1 or 2
+4  exp Radiotherapy/
+5  radiotherapy.fs.
+6  (radiotherap* or radiat* or irradiat*).ti,ab.
+7  exp Antineoplastic Agents/
+8  Antineoplastic Combined Chemotherapy Protocols/
+9  chemotherap*.mp.
+10 exp Chemoradiotherapy/
+11 (radiochemo* or chemoradio*).mp.
+12 4 or 5 or 6 or 7 or 8 or 9 or 10 or 11
+13 3 and 12
+14 Radiation Effects/
+15 exp Radiation Injuries/
+16 adverse effects.fs.
+17 ((late or adverse* or long term or side or long-term or chronic* or residual*
+   or delay* or undesirable or unexpected) adj5 (effect* or event* or outcome*
+   or reaction* or complication* or harm* or injur* or toxic* or cognit*)).ti,ab.
+18 (adrs or tolerab*).ti,ab.
+19 (radiation induced* or radiation-induced).ti,ab.
+20 14 or 15 or 16 or 17 or 18 or 19
+21 randomized controlled trial.pt.
+22 controlled clinical trial.pt.
+23 randomized.ab.
+24 placebo.ab.
+25 clinical trials as topic.sh.
+26 randomly.ab.
+27 trial.ti.
+28 exp Cohort Studies/
+29 cohort*.tw.
+30 longitudinal*.tw.
+31 prospective*.tw.
+32 21 or 22 or 23 or 24 or 25 or 26 or 27 or 28 or 29 or 30 or 31
+33 13 and 20 and 32
+34 exp animals/ not humans.sh.
+35 33 not 34
+key: mp = title, abstract, original title, name of substance word, subject heading
+word, keyword heading word, protocol supplementary concept word, rare disease
+supplementary concept word, unique identifier; ab = abstract; sh = subject heading;
+ti = title; pt = publication type.
+[A parallel MEDLINE run replaced the design filter (lines 21-32) with a health-economics
+filter for the economic commentary.]</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>[Embase via Ovid, 1980 to 2018 week 46. Appendix 1, verbatim:]
+1  exp Glioma/
+2  (glioma* or astrocytoma* or medulloblastoma* or ependymoma* or craniophyrangioma*
+   or oligodendroglioma* or glioblastoma* or GBM*).ti,ab.
+3  1 or 2
+4  exp radiotherapy/
+5  radiotherapy.fs.
+6  (radiotherap* or radiat* or irradiat*).ti,ab.
+7  exp chemotherapy/
+8  exp antineoplastic agent/
+9  chemotherap*.mp.
+10 exp chemoradiotherapy/
+11 (radiochemo* or chemoradio*).mp.
+12 4 or 5 or 6 or 7 or 8 or 9 or 10 or 11
+13 3 and 12
+14 radiation response/
+15 exp radiation injury/
+16 ae.fs.
+17 ((late or adverse* or long term or side or long-term or chronic* or residual*
+   or delay* or undesirable or unexpected) adj5 (effect* or event* or outcome*
+   or reaction* or complication* or harm* or injur* or toxic* or cognit*)).ti,ab.
+18 (adrs or tolerab*).ti,ab.
+19 (radiation induced* or radiation-induced).ti,ab.
+20 14 or 15 or 16 or 17 or 18 or 19
+21 crossover procedure/
+22 randomized controlled trial/
+23 single blind procedure/
+24 random*.mp.
+25 factorial*.mp.
+26 (crossover* or cross over* or cross-over).mp.
+27 placebo*.mp.
+28 (doubl* adj blind*).mp.
+29 (singl* adj blind*).mp.
+30 assign*.mp.
+31 allocat*.mp.
+32 volunteer*.mp.
+33 exp cohort analysis/
+34 cohort*.tw.
+35 longitudinal*.tw.
+36 prospective*.tw.
+37 21 or 22 or ... or 36
+38 13 and 20 and 37
+[A parallel Embase run substituted a health-economics filter for lines 21-37.]</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were CENTRAL (2018, Issue 11), MEDLINE via Ovid and
+Embase via Ovid, plus ClinicalTrials.gov and the WHO ICTRP for ongoing trials.
+No language restrictions. Web of Science was not used.
+[CENTRAL strategy, verbatim:
+#1 MeSH descriptor: [Glioma] explode all trees
+#2 glioma* or astrocytoma* or medulloblastoma* or ependymoma* or craniophyrangioma*
+   or oligodendroglioma* or glioblastoma* or GBM*
+#3 #1 or #2
+#4 MeSH descriptor: [Radiotherapy] explode all trees
+#5 radiotherap* or radiat* or irradiat*
+#6 MeSH descriptor: [Antineoplastic Agents] explode all trees
+#7 MeSH descriptor: [Antineoplastic Combined Chemotherapy Protocols] this term only
+#8 Any MeSH descriptor with qualifier(s): [Radiotherapy - RT]
+#9 Any MeSH descriptor with qualifier(s): [Drug therapy - DT]
+#10 Chemotherap*
+#11 MeSH descriptor: [Chemoradiotherapy] explode all trees
+#12 radiochemo* or chemoradio*
+#13 #4 or #5 or #6 or #7 or #8 or #9 or #10 or #11 or #12
+#14 #3 AND #13
+#15 MeSH descriptor: [Radiation Effects] this term only
+#16 MeSH descriptor: [Radiation Injuries] explode all trees
+#17 Any MeSH descriptor with qualifier(s): [Adverse effects - AE]
+#18 ((late or adverse* or long term or side or long-term or chronic* or residual*
+    or delay* or undesirable or unexpected) near/5 (effect* or event* or outcome*
+    or reaction* or complication* or harm* or injur* or toxic* or cognit*))
+#19 adrs or tolerab*
+#20 radiation induced* or radiation-induced
+#21 #15 or #16 or #17 or #18 or #19 or #20
+#22 #14 AND #21]</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD013047.pub2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="264.5" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Meta-analysis of cognitive functioning in breast cancer survivors previously treated with standard-dose chemotherapy</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Jim HSL, 2012</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Journal of Clinical Oncology</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>42.1 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>To quantify cognitive deficits in breast cancer survivors at least six months after completing standard-dose chemotherapy, and to examine demographic and clinical moderators (age, education, time since chemotherapy, endocrine therapy). Included deliberately as the counter-example: a meta-analysis in the highest-impact journal in this collection, whose entire search is seven short keyword pairings with no structured concept blocks, no truncation discipline and no design filter.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>P: Women who had completed standard-dose chemotherapy for breast cancer at least
+   six months previously.
+I: Standard-dose chemotherapy (past exposure).
+C: Healthy controls, patients not treated with chemotherapy, or the patient's own
+   pre-treatment/normative scores.
+O: Objective neuropsychological test performance across cognitive domains (verbal
+   ability, memory, executive function, processing speed, attention, visuospatial).</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>[PubMed searched natively; studies published 1937 to June 2011; English only.
+Seven search-term sets, verbatim from the Methods:]
+(1) cognitive effects AND cancer patients AND chemotherapy
+(2) cognition AND cancer AND chemotherapy
+(3) cognition disorders/chemically induced AND cancer AND chemotherapy
+(4) [cognition disorders/chemically induced OR cognition disorders]
+    AND [neoplasms/drug therapy OR neoplasms/radiotherapy OR neoplasms]
+(5) [cognition disorders or cognition or cognitive effects and cancer] AND chemotherapy
+(6) chemobrain AND cancer
+(7) cognitive impairment AND breast cancer
+Reference lists of retrieved publications and of relevant earlier systematic reviews
+and meta-analyses were also examined.
+Note: no field tags, no explicit MeSH explosion and no truncation are given, so these
+strings are not reproducible in the sense PRISMA-S requires. They are recorded here
+exactly as published.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were PubMed, PsycINFO, CINAHL and the Cochrane
+Library.
+[The terms used for PsycINFO, CINAHL and the Cochrane Library, verbatim:
+(1) cognitive disorders AND chemotherapy AND cancer
+(2) cognition AND chemotherapy AND cancer
+(3) chemobrain OR chemobrain OR chemo-brain
+(4) cognitive effects and chemotherapy and cancer
+Set (3) is printed with "chemobrain" twice; presumably one instance was intended to be
+a different spelling variant.]</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were PubMed, PsycINFO, CINAHL and the Cochrane
+Library only.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1200/JCO.2011.39.5640</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add category 4: depression
Soong 2025 (JAMA Netw Open, older adults with cancer - closest population match
in the collection), Vita 2023 (Cochrane, antidepressants), Kulchycki 2024
(JAMA Netw Open, librarian-built; includes a Scopus proximity strategy usable
as a Web of Science template).

Notes the ovarian-specific option (Watts 2015, BMJ Open) that failed the IF bar.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -10,11 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 OC treatment (general)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Functional status" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Cognition" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Depression" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Functional status'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 Cognition'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 Depression'!$A$2:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1958,4 +1960,498 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>04. Depression</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1st author / year</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Impact factor</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Purpose of the study</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PICO</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - PubMed / MEDLINE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Embase</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Web of Science</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="322" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Exercise Interventions for Depression, Anxiety, and Quality of Life in Older Adults With Cancer: A Systematic Review and Meta-Analysis</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Soong RY, 2025</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>JAMA Network Open</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>10.5 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>To determine whether exercise interventions are associated with improvements in psychological outcomes - depression, anxiety and health-related quality of life - among older adults with cancer. The closest match in this whole collection to the population of interest (older adults with cancer, patient-centred outcomes), and the only review here whose search carries an explicit older-adults block. The trade-off is sensitivity: the outcome block is four terms with no controlled vocabulary in PubMed.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>P: Older adults with cancer (mean age &gt;= 60 years), any cancer type, any comorbidity.
+I: Exercise interventions - aerobic, resistance and strength training, or mind-body
+   exercise (qigong, yoga, tai chi).
+C: Usual care.
+O: Depression severity; anxiety severity; health-related quality of life (HRQOL).</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>[PubMed searched natively, database inception to 5 November 2024.
+eTable 1 in Supplement 1, verbatim:]
+#1 "Geriatrics"[Mesh] OR "Aged"[Mesh] OR Aging OR Aged OR Centenarians
+   OR Nonagenarians OR Octogenarians OR Elder* OR Gerontology OR 'older adult*'
+#2 Neoplas*[title/abstract] OR Cancer[title/abstract] OR Malignan*[title/abstract]
+#3 Exercis*[title/abstract] OR Exerciz*[title/abstract]
+   OR (Physical*[title/abstract] AND Interven*[title/abstract])
+   OR (Physical*[title/abstract] AND Activit*[title/abstract])
+#4 depress* OR anxi* OR burden* OR Stress* OR 'quality of life'
+The four sets are combined with AND. Note the curly quotation marks as printed;
+PubMed will not parse 'older adult*' or 'quality of life' as phrases unless the
+quotes are replaced with straight double quotes.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>[Embase, database inception to 5 November 2024. eTable 1, verbatim:]
+#1 'geriatrics'/exp OR 'aged'/exp OR 'aging'/exp OR 'senescence'/exp
+   OR 'older adult*' OR 'aging' OR 'centenarians' OR 'nonagenarians'
+   OR 'octogenarians' OR 'gerontology' OR 'older people'/exp
+#2 'neoplas*'/exp OR 'cancer'/exp OR 'malignan*'/exp
+#3 'exercis*' OR 'exerciz*' OR (physical* NEAR/2 (intervent* OR activit*))
+#4 'depress*' OR 'depression'/exp OR 'anxi*' OR 'anxiety'/exp OR 'disease burden*'
+   OR 'physiological stress*' OR 'quality of life'
+Note: 'neoplas*'/exp and 'malignan*'/exp are printed with truncation inside an
+Emtree explosion, which Embase does not accept; these lines will need repair
+before reuse.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were PubMed, Embase, PsycINFO and the Cochrane
+Library, from inception to 5 November 2024.
+[Cochrane Library version, verbatim:
+#1 MeSH descriptor: [Geriatrics] explode all trees OR ((Aging OR Aged OR Centenarians
+   OR Nonagenarians OR Octogenarians OR Elder* OR Gerontology OR 'older adult*'):ti,ab,kw)
+#2 (neoplas*):ti,ab,kw OR (cancer):ti,ab,kw OR (malignan*):ti,ab,kw
+#3 MeSH descriptor: [Exercise] explode all trees OR (exercis*' OR 'exerciz*'
+   OR (physical* NEAR/2 (intervent* OR activit*)):ti,ab,kw)
+#4 MeSH descriptor: [Depression] explode all trees OR (anxi* OR burden* OR Stress*
+   OR 'quality of life'):ti,ab,kw)
+PsycINFO version, verbatim:
+#1 (Geriatrics OR Aged OR Aging OR Centenarians OR Nonagenarians OR Octogenarians
+   OR Elder* OR Gerontology OR 'Older Adult*').mp.
+#2 (neoplas* OR cancer OR malignan*).ti,ab.
+#3 exp Exercise/ OR exercis*.ti,ab. OR exerciz*.ti,ab.
+   OR (physical* adj2 (intervent*.ti,ab. or activit*.ti,ab.))
+#4 (depress* OR anxi* OR burden* OR stress* OR 'quality of life').ti,ab.]</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1001/jamanetworkopen.2024.57859</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="760" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Antidepressants for the treatment of depression in people with cancer</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Vita G, 2023</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>To evaluate the efficacy, tolerability and acceptability of antidepressants for treating depressive symptoms in adults (18 years or older) with cancer of any site and stage. Included as the reference-standard structure for this outcome: population AND depression AND antidepressant, where the depression block pairs three MeSH terms with one adjacency that catches adjustment, reactive and dysthymic disorders, and the drug block names roughly 70 individual agents alongside five exploded drug classes.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>P: Adults (&gt;= 18 years) with any primary cancer diagnosis and depression (major
+   depressive disorder, adjustment disorder, dysthymic disorder, or depressive
+   symptoms measured on a validated scale).
+I: Any antidepressant.
+C: Placebo, or another antidepressant.
+O: Efficacy (change in depressive symptoms, response, remission); tolerability
+   (adverse events, dropouts due to adverse events); acceptability (dropouts for any
+   reason).</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[Not searched as PubMed. MEDLINE via Ovid, 1946 to November 2022; latest search date
+24 November 2022. Appendix 2, verbatim:]
+1  exp Neoplasms/
+2  (cancer* or tumor* or tumour* or neoplas* or malignan* or carcinoma*
+   or adenocarcinoma* or choriocarcinoma* or lymphoma* or leukemia* or leukaemia*
+   or metastat* or sarcoma* or teratoma*).mp.
+3  1 or 2
+4  Depression/
+5  exp Depressive Disorder/
+6  Adjustment Disorders/
+7  (depress* or melanchol* or ((adjustment or reactive or dysthymic) adj5
+   disorder*)).mp.
+8  4 or 5 or 6 or 7
+9  drug therapy.fs.
+10 exp Antidepressive Agents/
+11 exp Heterocyclic Compounds/
+12 exp Serotonin Uptake Inhibitors/
+13 exp Adrenergic Uptake Inhibitors/
+14 exp Monoamine Oxidase Inhibitors/
+15 (anti-depress* or antidepress* or drug therap* or pharmacotherap* or trycyclic*
+   or TCA* or heterocyclic* or serotonin uptake or SSRI* or SNRI*
+   or monoamine oxidase inhibitor* or MAOI*).mp.
+16 (desipramine or imipramine or clomipramine or opipramol or trimipramine or
+   lofepramine or dibenzepin or amitriptyline or nortriptyline or protriptyline or
+   doxepin or iprindole or melitracen or butriptyline or dosulepin or amoxapine or
+   dimetacrine or amineptine or maprotiline or quinupramine or zimeldine or
+   fluoxetine or citalopram or paroxetine or sertraline or alaproclate or
+   fluvoxamine or etoperidone or escitalopram or isocarboxazid or nialamide or
+   phenelzine or tranylcypromine or iproniazide or iproclozide or moclobemide or
+   toloxatone or oxitriptan or tryptophan or mianserin or nomifensine or trazodone
+   or nefazodone or minaprine or bifemelane or viloxazine or oxaflozane or
+   mirtazapine or bupropion or medifoxamine or tianeptine or pivagabine or
+   venlafaxine or milnacipran or reboxetine or gepirone or duloxetine or
+   agomelatine or desvenlafaxine or vilazodone or hyperici herba or
+   hypericum perforatum or st john* wort* or saint john* wort*).mp.
+17 9 or 10 or 11 or 12 or 13 or 14 or 15 or 16
+18 3 and 8 and 17
+19 randomized controlled trial.pt.
+20 controlled clinical trial.pt.
+21 randomized.ab.
+22 placebo.ab.
+23 clinical trials as topic.sh.
+24 randomly.ab.
+25 trial.ti.
+26 19 or 20 or 21 or 22 or 23 or 24 or 25
+27 18 and 26
+28 exp animals/ not humans.sh.
+29 27 not 28
+key: mp = title, abstract, original title, name of substance word, subject heading
+word, keyword heading word, protocol supplementary concept, rare disease
+supplementary concept, unique identifier; pt = publication type; ab = abstract;
+sh = subject heading; ti = title.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>[Embase via Ovid, 1980 to November 2022. Appendix 3, verbatim:]
+1  exp neoplasm/
+2  (cancer* or tumor* or tumour* or neoplas* or malignan* or carcinoma*
+   or adenocarcinoma* or choriocrcinoma* or leukemia* or leukaemia* or metastat*
+   or sarcoma* or teratoma*).ti,ab.
+3  1 or 2
+4  exp depression/
+5  adjustment disorder/
+6  (depress* or melanchol* or ((adjustment or reactive or dysthymic) adj3
+   disorder*)).ti,ab.
+7  4 or 5 or 6
+8  exp antidepressant agent/
+9  exp heterocyclic compound/
+10 exp serotonin uptake inhibitor/
+11 exp adrenergic receptor affecting agent/
+12 exp monoamine oxidase inhibitor/
+13 (anti-depress* or antidepress* or drug therap* or pharmacotherap* or trycyclic*
+   or TCA* or heterocyclic* or serotonin uptake or SSRI* or SNRI*
+   or monoamine oxidase inhibitor* or MAOI*).ti,ab.
+14 [the same ~70-agent drug-name line as MEDLINE line 16].ti,ab.
+15 8 or 9 or 10 or 11 or 12 or 13 or 14
+16 3 and 7 and 15
+17 crossover procedure/
+18 double-blind procedure/
+19 randomized controlled trial/
+20 single-blind procedure/
+21 random*.mp.
+22 factorial*.mp.
+23 (crossover* or cross over* or cross-over*).mp.
+24 placebo*.mp.
+25 (double* adj blind*).mp.
+26 (singl* adj blind*).mp.
+27 assign*.mp.
+28 allocat*.mp.
+29 volunteer*.mp.
+30 17 or 18 or 19 or 20 or 21 or 22 or 23 or 24 or 25 or 26 or 27 or 28 or 29
+31 16 and 30
+32 (exp animal/ or nonhuman/ or exp animal experiment/) not human/
+33 31 not 32
+Note "choriocrcinoma*" is a typo for choriocarcinoma* in the published Embase and
+CENTRAL appendices; the MEDLINE appendix spells it correctly.</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were CENTRAL (2022, Issue 11), MEDLINE Ovid,
+Embase Ovid and PsycINFO Ovid, all to November 2022, supplemented by handsearching
+the trial databases of the FDA, MHRA, EMA and other drug-approving agencies.
+Web of Science was not used.
+[CENTRAL strategy (Appendix 1), verbatim:
+#1 MeSH descriptor: [Neoplasms] explode all trees
+#2 (cancer* or tumor* or tumour* or neoplas* or malignan* or carcinoma* or
+   adenocarcinoma* or choriocrcinoma* or leukemia* or leukaemia* or metastat*
+   or sarcoma* or teratoma*)
+#3 #1 or #2
+#4 MeSH descriptor: [Depression] explode all trees
+#5 MeSH descriptor: [Depressive Disorder] explode all trees
+#6 MeSH descriptor: [Adjustment Disorders] explode all trees
+#7 (depress* or melanchol* or ((adjustment or reactive or dysthymic) near/5 disorder*))
+#8 #4 or #5 or #6 or #7
+#9 Any MeSH descriptor with qualifier(s): [Drug therapy - DT]
+#10-#16 [antidepressant class MeSH explosions and the ~70-agent drug-name list]
+#17 #9 or #10 or #11 or #12 or #13 or #14 or #15 or #16
+#18 #3 and #8 and #17]</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD011006.pub4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="736" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Aerobic Physical Activity and Depression Among Patients With Cancer: A Systematic Review and Meta-Analysis</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Kulchycki M, 2024</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>JAMA Network Open</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>10.5 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>To determine whether aerobic physical activity is associated with reduced depression among patients with cancer, and to examine patient, cancer, intervention and methodological moderators. Included because the strategy was built by a named research librarian and is the most sensitive depression block in this collection - it is the one to copy if you want maximum recall on the outcome, including a Scopus/citation-index translation in proximity syntax.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>P: Patients with any cancer diagnosis, including haematopoietic stem cell transplant
+   recipients.
+I: Aerobic physical activity interventions (randomised controlled trials).
+C: Usual care or non-aerobic control.
+O: Severity of depression on validated self-reported scales (CES-D, HADS, BDI and
+   others), short- and long-term.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>[Not searched as PubMed. Ovid MEDLINE, publications 1 January 1980 to 5 July 2023;
+strategy built by a research librarian. eTable 1 in Supplement 1, verbatim
+(population and depression blocks; the exercise block is lines 8-19 and the design
+filter lines 20-32):]
+1  exp neoplasms/ or cancer survivors/ or psycho-oncology/ or exp hematopoietic stem
+   cell transplantation/ or stem cell transplantation/ or hematopoietic stem cell
+   mobilization/
+2  (cancer* or neoplas* or tumo?r* or malignan* or metasta* or oncogen* or oncolog*
+   or psychooncolog* or sarcoma* or leuk?emi* or lymphoma* or hodgkin* or nonhodgkin*
+   or carcino* or melanoma* or thymoma* or myeloma* or blastoma* or hepatoblastoma*
+   or mesenchymoma* or mesothelioma* or hepatoma* or adenocarcinoma*
+   or glioma*).ti,ab,kf
+3  (HSCT or ((h?ematopoietic or h?emato-poietic) adj3 (transplant* or sct or bct
+   or mobili#ation)) or pbsct or pbct or psct or ((peripheral or pbsc or pbscs) adj3
+   transplant*) or autohct or autopbsct or autopbsc or autopsc or cbsct or
+   ((autologous or auto-logous or auto or allogeneic or allo-geneic or homologous
+   or homo-logous) adj hct)).ti,ab,kf
+4  or/1-3
+5  depression/ or exp depressive disorder/ or sadness/ or demoralization/ or
+   mental health/ or happiness/ or hope/ or resilience, psychological/
+6  (depress* or dysthymi* or melanchol* or affective or mood or distress* or sadness
+   or sad or hopeless* or demorali* or mental health or psych* health or wellbeing
+   or wellness or contented or contentment or happiness or hope* or
+   resilien*).ti,ab,kf
+7  5 or 6
+8-19  [exercise block: exp exercise/ or exp exercise movement techniques/ or exp
+      exercise therapy/ or dancing/ or exp physical fitness/ or exp sports/ or
+      aquatic therapy/; plus 11 text-word lines covering modality, dose, sport and
+      exergaming terms]
+20-30 [design filter: randomized controlled trial/ or Random Allocation/ or Double
+      Blind Method/ or Single Blind Method/; trial publication types; exp Clinical
+      Trials as topic/; (clinical adj trial$).tw,kf; (RCT or RCTs).tw,kf;
+      ((singl$ or doubl$ or treb$ or tripl$) adj (blind$3 or dumm* or mask$3)).tw,kf;
+      PLACEBOS/; (placebo$ or sham).tw,kf;
+      (randomized or randomised or randomly).ab; trial.ti]
+31 exp animals/ not humans.sh
+32 30 not 31
+33 4 and 7 and 19 and 32
+   limit 33 to (english language and yr="1980 -Current")</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>[Embase via Ovid, 1 January 1980 to 5 July 2023. eTable 1, verbatim (population and
+depression blocks; exercise block lines 8-19, design filter lines 20-29):]
+1  exp neoplasm/ or exp cancer patient/ or psycho-oncology/ or exp hematopoietic stem
+   cell transplantation/ or stem cell transplantation/
+2  (cancer* or neoplas* or tumo?r* or malignan* or metasta* or oncogen* or oncolog*
+   or psychooncolog* or sarcoma* or leuk?emi* or lymphoma* or hodgkin* or nonhodgkin*
+   or carcino* or melanoma* or thymoma* or myeloma* or blastoma* or hepatoblastoma*
+   or mesenchymoma* or mesothelioma* or hepatoma* or adenocarcinoma*
+   or glioma*).ti,ab,kw
+3  [same HSCT line as MEDLINE, .ti,ab,kw]
+4  or/1-3
+5  exp depression/ or sadness/ or demoralization/ or mental health/ or psychological
+   well-being/ or happiness/ or hope/ or hopelessness/ or unhappiness/ or
+   psychological resilience/
+6  (depress* or dysthymi* or melanchol* or affective or mood or distress* or sadness
+   or sad or hopeless* or demorali* or mental health or psych* health or wellbeing
+   or wellness or contented or contentment or happiness or hope* or
+   resilien*).ti,ab,kw
+7  5 or 6
+8-19  [exercise block, Emtree equivalents plus the same 11 text-word lines]
+20-28 [Embase design filter]
+29 or/20-28
+30 (exp animal/ or nonhuman/) not exp human/
+31 29 not 30
+32 4 and 7 and 19 and 31
+33 limit 32 to (english language and yr="1980 -Current")</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Web of Science was not searched. Scopus was used as the citation-index equivalent,
+alongside MEDLINE, Embase, CENTRAL, CINAHL and PsycINFO (1 January 1980 to
+5 July 2023). The Scopus strategy is the closest available template for a Web of
+Science translation, since Scopus proximity syntax (W/n) maps onto Web of Science
+NEAR/n.
+[Scopus strategy, verbatim (population and depression sets; the exercise block is
+sets 5-15 and the design filter sets 16-24):
+1 TITLE-ABS-KEY(cancer* or neoplas* or tumo*r* or malignan* or metasta* or oncogen*
+  or oncolog* or psychooncolog* or sarcoma* or leuk*emi* or lymphoma* or hodgkin*
+  or nonhodgkin* or carcino* or melanoma* or thymoma* or myeloma* or blastoma*
+  or hepatoblastoma* or mesenchymoma* or mesothelioma* or hepatoma*
+  or adenocarcinoma* or glioma*)
+2 TITLE-ABS-KEY(HSCT or ((h*ematopoietic or h*emato-poietic) W/3 (transplant* or sct
+  or bct or mobili?ation)) or pbsct or pbct or psct or ((peripheral or pbsc or pbscs)
+  W/3 transplant*) or autohct or autopbsct or autopbsc or autopsc or cbsct or
+  ((autologous or auto-logous or auto or allogeneic or allo-geneic or homologous
+  or homo-logous) W/1 hct))
+3 #1 or #2
+4 TITLE-ABS-KEY(depress* or dysthymi* or melanchol* or affective or mood or distress*
+  or sadness or sad or hopeless* or demorali* or "mental health" or (psych* W/1 health)
+  or wellbeing or wellness or contented or contentment or happiness or hope*
+  or resilien*)
+...
+25 #3 AND #4 AND #15 AND #24
+26 #25 AND PUBYEAR AFT 1979 AND ( LIMIT-TO ( LANGUAGE , "English" ) )]</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1001/jamanetworkopen.2024.37964</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add category 5: nutritional status
Billson 2013 (Cochrane) is ovarian-cancer specific and above the IF bar - the
most directly reusable record so far. Takaoka 2024 (Adv Nutr) is the only review
in the collection publishing a full Web of Science TS= strategy. Lovell 2025
(BJC) lays the search out by PICO element with three parallel nutritional-status
sub-blocks.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -11,12 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Functional status" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Cognition" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Depression" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Nutritional status" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Functional status'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 Cognition'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 Depression'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5 Nutritional status'!$A$2:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2454,4 +2456,506 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>05. Nutritional status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1st author / year</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Impact factor</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Purpose of the study</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PICO</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - PubMed / MEDLINE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Embase</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Web of Science</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="736" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Perioperative nutrition interventions for women with ovarian cancer</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Billson HA, 2013</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>To assess the effects of nutrition interventions during the perioperative period for women with ovarian cancer. The single most directly reusable record in this collection: an ovarian-cancer population block intersected with a 17-line nutrition block that includes Nutritional Status/ and Nutrition Assessment/ as explicit MeSH and Emtree terms, in a journal above the threshold.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>P: Women with ovarian cancer undergoing surgery (perioperative period).
+I: Any nutrition intervention - enteral or parenteral nutrition, oral supplements,
+   immunonutrition, early feeding, dietary advice.
+C: Standard perioperative care or an alternative nutrition intervention.
+O: Postoperative complications and infection; length of hospital stay; nutritional
+   status; quality of life; gastrointestinal function; mortality.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>[Not searched as PubMed. Medline via Ovid, 1946 to July week 4 2012.
+Appendix 2, verbatim:]
+1  exp Perioperative Care/
+2  exp Perioperative Period/
+3  (peri-operative or perioperative).mp.
+4  exp Surgical Procedures, Operative/
+5  surgery.fs.
+6  (surg* or operat* or procedure*).mp.
+7  1 or 2 or 3 or 4 or 5 or 6
+8  exp Nutrition Therapy/
+9  exp Nutrition Disorders/
+10 Nutritional Status/
+11 Nutrition Assessment/
+12 Cachexia/
+13 (weight or underweight or cachexi* or malnutrition).mp.
+14 (nutrition* or nutrient* or macronutrient* or micronutrient* or immunonutrition
+   or immuno-nutrition).mp.
+15 exp Food/
+16 (food* or feed* or supplement* or vitamin* or mineral* or protein* or fat*
+   or carbohydrate* or calorie* or energy).mp.
+17 exp Diet/
+18 diet therapy.fs.
+19 diet*.mp.
+20 exp Fish Oils/
+21 exp Amino Acids/
+22 (amino acid* or fatty acid* or fish oil* or omega 3 or glutamin* or arginine
+   or novel substrate* or nitrogen).mp.
+23 exp Feeding Methods/
+24 (enteral or parenteral or TPN or naso-gastric or nasogastric or gastrostomy
+   or jejunostomy).mp.
+25 8 or 9 or 10 or 11 or 12 or 13 or 14 or 15 or 16 or 17 or 18 or 19 or 20 or 21
+   or 22 or 23 or 24
+26 exp Genital Neoplasms, Female/
+27 exp Ovarian Neoplasms/
+28 ((gynaecologic* or gynecologic* or ovar*) adj5 (cancer* or tumor* or tumour*
+   or malignan* or carcinoma* or adenocarcinoma*)).mp.
+29 26 or 27 or 28
+30 randomized controlled trial.pt.
+31 controlled clinical trial.pt.
+32 randomized.ab.
+33 placebo.ab.
+34 clinical trials as topic.sh.
+35 randomly.ab.
+36 trial.ti.
+37 30 or 31 or 32 or 33 or 34 or 35 or 36
+38 7 and 25 and 29 and 37
+39 exp animals/ not humans.sh.
+40 38 not 39
+key: mp = protocol supplementary concept, rare disease supplementary concept, title,
+original title, abstract, name of substance word, subject heading word, unique
+identifier; pt = publication type; ab = abstract; sh = subject heading;
+fs = floating subheading.
+(Line 38 is printed as "7 and 25 and 29 and 37~" with a stray tilde.)</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>[Embase via Ovid, 1980 to 2012 week 31. Appendix 3, verbatim:]
+1  perioperative period/
+2  (peri-operative or perioperative).mp.
+3  exp surgery/
+4  su.fs.
+5  (surg* or operat* or procedure*).mp.
+6  1 or 2 or 3 or 4 or 5
+7  exp diet therapy/
+8  exp nutritional disorder/
+9  exp nutritional status/
+10 nutritional assessment/
+11 cachexia/
+12 (weight or underweight or cachexi* or malnutrition).mp.
+13 (nutrition* or nutrient* or macronutrient* or micronutrient* or immunonutrition
+   or immuno-nutrition).mp.
+14 exp Food/
+15 (food* or feed* or supplement* or vitamin* or mineral* or protein* or fat*
+   or carbohydrate* or calorie* or energy).mp.
+16 exp diet/
+17 diet*.mp.
+18 fish oil/
+19 exp amino acid/
+20 (amino acid* or fatty acid* or fish oil* or omega 3 or glutamin* or arginine
+   or novel substrate* or nitrogen).mp.
+21 exp food intake/
+22 (enteral or parenteral or PN or TPN or naso-gastric or nasogastric or gastrostomy
+   or jejunostomy).mp.
+23 7 or 8 or 9 or 10 or 11 or 12 or 13 or 14 or 15 or 16 or 17 or 18 or 19 or 20
+   or 21 or 22
+24 exp female genital tract tumor/
+25 exp ovary tumor/
+26 ((gynaecologic* or gynecologic* or ovar*) adj5 (cancer* or tumor* or tumour*
+   or malignan* or carcinoma* or adenocarcinoma*)).mp.
+27 24 or 25 or 26
+28 crossover procedure/
+29 double-blind procedure/
+30 randomized controlled trial/
+31 single-blind procedure/
+32 random*.mp.
+33 factorial*.mp.
+34 (crossover* or cross over* or cross-over*).mp.
+35 placebo*.mp.
+36 (double* adj blind*).mp.
+37 (singl* adj blind*).mp.
+38 assign*.mp.
+39 allocat*.mp.
+40 volunteer*.mp.
+41 28 or 29 or 30 or 31 or 32 or 33 or 34 or 35 or 36 or 37 or 38 or 39 or 40
+42 6 and 23 and 27 and 41
+43 (exp Animal/ or Nonhuman/ or exp Animal Experiment/) not Human/
+44 42 not 43</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were the Cochrane Gynaecological Cancer Group
+Specialised Register, CENTRAL (2012, Issue 7), Medline (1946 to July week 4 2012),
+Embase (1980 to 2012 week 31), DARE (to 7 August 2012), AMED (1985 to April 2012),
+BNI (1992 to April 2012) and CINAHL. Web of Science was not used.
+[CENTRAL/DARE strategy (Appendix 1), verbatim - useful because it is the same
+three-block design in a proximity syntax:
+#1 MeSH descriptor Perioperative Care explode all trees
+#2 MeSH descriptor Perioperative Period explode all trees
+#3 peri-operative or perioperative
+#4 MeSH descriptor Surgical Procedures, Operative explode all trees
+#5 Any MeSH descriptor with qualifier: SU
+#6 surg* or operat* or procedure*
+#7 (#1 OR #2 OR #3 OR #4 OR #5 OR #6)
+#8 MeSH descriptor Nutrition Therapy explode all trees
+#9 MeSH descriptor Nutrition Disorders explode all trees
+#10 MeSH descriptor Nutritional Status, this term only
+#11 MeSH descriptor Nutrition Assessment, this term only
+#12 MeSH descriptor Cachexia, this term only
+#13 weight or underweight or cachexi* or malnutrition
+#14 nutrition* or nutrient* or macronutrient* or micronutrient* or immunonutrition
+#15 MeSH descriptor Food explode all trees
+#16 food* or feed* or supplement* or vitamin* or mineral* or protein* or fat*
+    or carbohydrate* or calorie* or energy
+#17 MeSH descriptor Diet explode all trees
+#18 Any MeSH descriptor with qualifier: DH
+#19 diet*
+#20 MeSH descriptor Fish Oils explode all trees
+#21 MeSH descriptor Amino Acids explode all trees
+#22 amino acid* or fatty acid* or fish oil* or omega 3 or glutamin* or arginine
+    or novel substrate* or nitrogen
+#23 MeSH descriptor Feeding Methods explode all trees
+#24 enteral or parenteral of PN or TPN or naso-gastric or nasogastric or gastrostomy
+    or jejunostomy
+#25 (#8 OR ... OR #24)
+#26 MeSH descriptor Genital Neoplasms, Female explode all trees
+#27 MeSH descriptor Ovarian Neoplasms explode all trees
+#28 (gynaecologic* or gynecologic* or ovar*) near/5 (cancer* or tumor* or tumour*
+    or malignan* or carcinoma* or adenocarcinoma*)
+#29 (#26 OR #27 OR #28)
+#30 (#7 AND #25 AND #29)
+Line #24 is printed with "of PN" where "or PN" is meant.]</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD009884.pub2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="494.5" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Prevalence of and Survival with Cachexia among Patients with Cancer: A Systematic Review and Meta-Analysis</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Takaoka T, 2024</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Advances in Nutrition</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>8.0 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>To quantify how the reported prevalence of cachexia in patients with cancer varies by diagnostic criterion, and to estimate the association between cachexia and overall survival. Included because it is the only review in this collection that publishes a complete Web of Science strategy, set out side by side with the PubMed version so the MeSH-to-TS= translation is visible line for line.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>P: Patients with cancer (any type, any stage).
+I/E: Presence of cachexia, diagnosed by any published definitive criterion
+   (Fearon, EPCRC, ASPEN/AND, Evans, GLIM and others).
+C: Patients with cancer without cachexia.
+O: Prevalence of cachexia by diagnostic criterion; overall survival.</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[PubMed searched natively, inception to 31 July 2023. Supplemental Table 2, verbatim
+(result counts as printed):]
+#1  Neoplasms [MeSH]                                    3,857,356
+#2  Cancer [TIAB]                                       2,173,946
+#3  Tumor [TIAB]                                        1,420,714
+#4  #1 OR #2 OR #3                                      4,767,145
+#5  Cachexia [MeSH]                                         6,238
+#6  Wasting Syndrome [MeSH]                                 1,985
+#7  Disease-related malnutrition [TIAB]                       251
+#8  #5 OR #6 OR #7                                          8,308
+#9  Diagnosis [MeSH]                                    9,374,402
+#10 Assessment [TIAB]                                   1,261,169
+#11 Screening [TIAB]                                      676,373
+#12 #9 OR #10 OR #11                                   10,513,314
+#13 #4 AND #8                                               4,381
+#14 #13 AND #12                                             1,680
+#15 Clinical Study [Publication Type]                   1,138,887
+#16 Epidemiologic Studies [MeSH]                        3,152,279
+#17 #15 OR #16                                          3,923,924
+#18 #14 AND #17                                               439
+Note the nutritional-status concept here is narrow - three terms - and there is no
+truncation on Cancer/Tumor. Sensitivity was traded for a manageable yield.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Not searched. Only PubMed and Web of Science were searched, from inception to
+31 July 2023, by a single researcher.</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>[Web of Science searched, inception to 31 July 2023. Supplemental Table 2, verbatim
+(result counts as printed):]
+#1  TS = Neoplasms                       230,171
+#2  TS = Cancer                        3,018,044
+#3  TS = Tumor                         2,042,632
+#4  #1 OR #2 OR #3                     4,034,303
+#5  TS = Cachexia                         12,778
+#6  TS = Wasting Syndrome                  6,221
+#7  TS = Disease-related malnutrition      4,463
+#8  #5 OR #6 OR #7                        22,512
+#9  TS = Diagnosis                     1,992,601
+#10 TS = Assessment                    2,079,264
+#11 TS = Screening                     1,145,410
+#12 #9 OR #10 OR #11                   4,803,898
+#13 #4 AND #8                             10,115
+#14 #13 AND #12                            2,171
+#15 TS = Clinical study                2,353,376
+#16 TS = Epidemiologic study              58,077
+#17 TS = Epidemiological study           142,973
+#18 #16 OR #17                           196,384
+#19 #15 OR #18                         2,490,979
+#20 #14 AND #19                              644
+TS = topic search (title, abstract, author keywords, Keywords Plus). Note that the
+study-design concept, which is a publication type in PubMed, has to be re-expressed
+as free text in Web of Science, and that British and American spellings of
+"epidemiologic(al)" must both be entered.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.advnut.2024.100282</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="760" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Nutritional status, body composition and chemotherapy dosing in children and young people with cancer: a systematic review</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Lovell AL, 2025</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>British Journal of Cancer</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>6.4 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>To determine whether nutritional status (undernutrition, overweight/obesity, altered body composition) alters the pharmacokinetics and pharmacodynamics of antineoplastic drugs in children and young people (&lt; 21 years) with cancer. Included as the clearest example of a search laid out explicitly by PICO element, with nutritional status broken into three parallel sub-blocks - undernutrition, overnutrition, and neutral body-composition measures - which is the structure most likely to transfer to an ovarian cancer review where both directions matter.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>P: Children and young people (&lt; 21 years) with cancer receiving antineoplastic
+   therapy.
+I/E: Antineoplastic drug therapy (chemotherapy, alkylating agents, combination
+   protocols).
+C: Nutritional status groups - undernutrition/sarcopenia versus normal nutrition
+   versus overweight/obesity/sarcopenic obesity, defined by body composition, BMI
+   or nutritional status measures.
+O: Pharmacokinetic and pharmacodynamic parameters; drug toxicity and adverse
+   reactions; survival (overall, disease-free, progression-free).</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>[MEDLINE (PubMed) searched to 30 September 2024; strategy developed with a library
+specialist and set out by PICO element. Supplementary 1, verbatim:]
+Population
+  Child/ [MeSH], Pediatrics/ [MeSH], Adolescent/ [MeSH], Infant/ [MeSH]
+  (child* or pediatric or pediatric or adolescen* or teen* or kids or preteen
+  or pre-teen or youth or infan* or "young adult*" or "school age*").mp.
+  Neoplasms [MeSH]
+  (neoplasm* or cancer or "p?ediatric oncology" or "p?ediatric cancer"
+  or "child* cancer").mp.
+Intervention
+  Drug Therapy/ [MeSH], Antineoplastic Agents/ [MeSH], Alkylating Agents/ [MeSH],
+  Antineoplastic Combined Chemotherapy Protocols/ [MeSH]
+  (chemotherap* or "drug therapy" or "antineoplastic agent*" or "alkylating agent*"
+  or cytotox* or antitumo?r or anti?cancer).mp.
+Comparison  [this is where nutritional status sits]
+  Malnutrition/ [MeSH], Thinness/ [MeSH], Protein-Energy Malnutrition/ [MeSH],
+  Severe Acute Malnutrition/ [MeSH], Sarcopenia/ [MeSH]
+  (malnutrition or thinness or "protein-energy malnutrition"
+  or "severe-acute malnutrition" or malnourish* or underweight or PEM
+  or "protein-calorie malnutrition" or "nutritional deficien*" or undernutrition
+  or sarcopeni*).mp.
+  Overnutrition/ [MeSH], Overweight/ [MeSH], Obesity/ [MeSH]
+  (overnutrition or overweight or obesity or obese or hypernutrition
+  or "sarcopenic obesity").mp.
+  Nutritional Status/ [MeSH], Body Composition/ [MeSH], Body Mass Index/ [MeSH],
+  Body Weight/ [MeSH]
+  ("nutrition* status" or "body composition" or "body mass index" or "body weight"
+  or BMI).mp.
+Outcome
+  Pharmacokinetics/ [MeSH], Toxicology/ [MeSH], Metabolism/ [MeSH],
+  Pharmacogenetics/ [MeSH]
+  (pharmacokinetic* or toxic* or metabolism or pharmacodynamic).mp.
+  "Drug-Related Side Effects and Adverse Reactions"/ [MeSH]
+  ("drug toxicity" or "drug side effect*" or toxicit*).mp.
+  Survival/ [MeSH], Disease-Free Survival/ [MeSH], Survival Rate/ [MeSH],
+  Progression-Free Survival/ [MeSH], Survival Analysis/ [MeSH]
+  (surviv* or "disease-free surviv*" or "survival rate"
+  or "progression-free surviv*" or "survival analysis").mp.
+Keyword search: mp = title, book title, abstract, original title, name of substance
+word, subject heading word, floating sub-heading word, keyword heading word, organism
+supplementary concept word, protocol supplementary concept word, rare disease
+supplementary concept word, unique identifier, synonyms, population supplementary
+concept word, anatomy supplementary concept word.
+Note the strategy mixes PubMed-style [MeSH] tags with Ovid-style .mp. and is titled
+"Proposed search terms prepared for MEDLINE database" - it is a term list to be
+translated, not a runnable line-numbered strategy.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Searched, but no Embase-specific string was published. The Methods state that
+"Medical Subject Headings, major topics, and multi-purpose terms were developed" and
+adapted across databases; only the MEDLINE term list is reproduced
+(Supplementary 1).</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Searched (Web of Science Core Collection), but no Web of Science-specific string was
+published. Databases searched were MEDLINE (PubMed), EMBASE, Web of Science Core
+Collection, Scopus, ProQuest Health, Cochrane Trials and Cochrane Reviews, all to
+30 September 2024. Only the MEDLINE term list is reproduced.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41416-025-03023-3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add category 6: health-related quality of life
Mishra 2012 (Cochrane) searches on instrument acronyms - QLQ-C30, FACIT, SF-36,
HADS, POMS, MSAS - which is the most transferable idea here. Osanto 2024
(eClinicalMedicine) has a full Web of Science TI=/AB=/TS= strategy and a 40-term
PRO block spanning anxiety, depression, functional status, fatigue and pain.
Cramer 2017 (Cochrane) is the contrast: HRQOL is the primary outcome and appears
nowhere in the search.

Flags line-numbering errors in Cramer's published PubMed appendix.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Cognition" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Depression" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Nutritional status" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 HRQOL" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
@@ -19,6 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 Cognition'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 Depression'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5 Nutritional status'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6 HRQOL'!$A$2:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2958,4 +2960,568 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>06. Health-related quality of life (HRQOL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1st author / year</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Impact factor</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Purpose of the study</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PICO</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - PubMed / MEDLINE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Embase</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Web of Science</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="760" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Exercise interventions on health-related quality of life for people with cancer during active treatment</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Mishra SI, 2012</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>To evaluate the effectiveness of exercise on overall HRQoL and on specific HRQoL domains among adults with cancer during active treatment. Included because its HRQoL block is the most complete in this collection: alongside the expected controlled vocabulary and free text it lists the named measurement instruments, so trials reporting only "FACT-G" or "QLQ-C30" are still retrieved.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>P: Adults with any cancer, during active treatment (surgery, chemotherapy,
+   radiotherapy, hormonal therapy).
+I: Exercise interventions (aerobic, resistance, combination, mind-body including
+   yoga, tai chi, qigong, hydrotherapy).
+C: Usual care, no exercise, or an alternative non-exercise intervention.
+O: Overall HRQoL and HRQoL domains - physical, psychological, social, spiritual
+   well-being, pain, fatigue, sleep, body image, vitality; adverse events.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>[MEDLINE searched via PubMed, inception to May 2010 (430 hits) and January 2010 to
+November 2011 (190 hits). Appendix 1, verbatim - lines 32-58 are the HRQoL block:]
+1-31   [exercise block: exp exercise/; exercise tolerance/; exp exertion/; Pliability/;
+       physical fitness/; "Physical Education and Training"/; exp physical endurance/;
+       exercise therapy/; exercising.mp.; physical condition$.mp.; stamina.mp.;
+       motor activity/; exercise test/; exp Sports/; tai chi.mp. or tai ji/; yoga/;
+       muscle stretching exercises/; exp "range of motion, articular"/; pilates.mp.;
+       qigong.mp.; chi kung.mp.; resistance training.mp.; mind body therap$.mp.;
+       exp complementary therapies/; Bad Ragaz.mp.; Ai Chi.mp.; Halliwick.mp.;
+       hippotherapy.mp.; Hydrotherapy/; balance exercise$.mp.; aquatic exercise$.mp.]
+32     1 or 2 or 3 or ... or 31
+33     "quality of life"/
+34     exp health status/
+35     "activities of daily living"/
+36     life qualit$.mp.
+37     exp self concept/
+38     health level.mp.
+39     level of health.mp.
+40     wellness.mp.
+41     well being.mp.
+42     (activities of daily life or daily living activities).mp.
+43     functional ability.mp.
+44     good health.mp.
+45     healthiness.mp.
+46     patient reported outcomes.mp.
+47     social adjustment/
+48     physical limitations.mp.
+49     psychiatric status.mp.
+50     pain measurement/
+51     functional assessment.mp.
+52     fact questionnaire.mp.
+53     fact survey.mp.
+54     qlc-c30.mp.
+55     facit.mp.
+56     toi.mp.
+57     (flic or sf-36 or ces-d or bdi or sta1 or bfi or hads or lasa or poms or qli
+       or rsci or pais or bpi or msas or mos or ptgi or panas).mp.
+58     sense of coherence.mp.
+59-65  [design filter: randomized.ab.; placebo.ab.; randomly.ab.; trial.ab.;
+       randomized controlled trial.pt.; controlled clinical trial.pt.; random$.ab]
+66-69  [population: exp neoplasms/; cancer.mp.;
+       (neoplasm$ or tumor$ or tumour or malignan$).mp.; active treatment.mp.]
+70     [union of lines 33-58 - the HRQoL set]
+71     [union of the design lines]
+72     [union of the cancer lines]
+73     32 and 70 and 71 and 72
+74-76  Survivors/ ; survivor.mp. ; 74 or 75   [used to exclude survivorship trials,
+       which are covered by the companion review]
+Note "qlc-c30" is a transposition of QLQ-C30, and "sta1" of STAI, in the published
+appendix. Repair both before reuse.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>[Embase, inception to May 2010 (713 hits) and January 2010 to November 2011 (349 hits).
+Appendix 3, verbatim - lines 33-58 are the HRQoL block:]
+1-31   [exercise block, Emtree equivalents: exp exercise/; exertion.mp.; pliability/;
+       fitness/; (physical education and training).mp.; physical endurance.mp. or
+       endurance/; kinesiotherapy/; exercising.mp.; "physical condition$".mp.;
+       stamina.mp.; exp motor activity/; exp sports/; exercise test/; tai chi.mp.;
+       tai ji.mp.; yoga/; stretching exercise/; "range of motion"/; pilates.mp.;
+       qigong.mp.; chi kung.mp.; muscle strength/ or muscle training/ or resistance
+       training.mp.; mind body therapy.mp.; alternative medicine/; bad ragaz.mp.;
+       ai chi.mp.; halliwick.mp.; hippotherapy.mp.; hydrotherapy/;
+       balance exercises.mp.; aquatic exercise/]
+32     1 or 2 or ... or 31
+33     "quality of life"/
+34     exp health status/
+35     daily life activity/
+36     life qualit$.mp.
+37     exp self concept/
+38     health level.mp.
+39     "level of health".mp.
+40     wellbeing/
+41     wellness.mp.
+42     good health.mp.
+43     functional ability.mp.
+44     healthiness.mp.
+45     "patient reported outcomes".mp.
+46     social adaptation/
+47     physical limitation$.mp.
+48     psychiatric status.mp.
+49     pain assessment/
+50     functional assessment/
+51     questionnaire/ or fact questionnaire.mp.
+52     fact survey.mp.
+53     health survey/
+54     qlc-c30.mp.
+55     facit.mp.
+56     toi.mp.
+57     sense of coherence.mp.
+58     (flic or sf-36 or ces-d or bdi or stal or bfi or hads or lasa or poms or qli
+       or rsci or pais or bpi or msas or mos or ptgi or panas).mp.
+59-64  [design filter]
+65     59 or 60 or 61 or 62 or 63 or 64
+66     [union of the HRQoL lines]
+67-70  exp neoplasm/; cancer.mp.;
+       (neoplasm$ or tumor$ or tumour or malignan$).mp.; active treatment
+71     (67 or 68 or 69 or 70)
+72-74  Survivors/; survivor$.mp.; 72 or 73
+75     32 and 65 and 66 and 71
+76     75 not 74
+(Line 69 is printed as ".mp3" - a typo for .mp.; "stal" in line 58 is STAI.)</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Web of Science was used, but for citation searching of key authors rather than with a
+subject strategy, so no Web of Science string exists. As reported: "We also searched
+citations of key authors through Web of Science and Scopus, and searched PubMed's
+related article feature."
+Databases searched with a strategy: CENTRAL, PubMed MEDLINE (Appendix 1),
+MEDLINE In-Process (Appendix 2), EMBASE (Appendix 3), CINAHL (Appendix 4),
+PsycINFO (Appendix 5), and PEDRO, LILACS, SIGLE, SportDiscus, OTSeeker and
+Sociological Abstracts (Appendix 6), all from inception to November 2011, with no
+language or date restriction. Trial registries (WHO ICTRP, Current Controlled Trials,
+CenterWatch, ClinicalTrials.gov), reference lists and expert contact were also used.
+[The CINAHL version (Appendix 4) is the same HRQoL set in EBSCOhost syntax and
+includes (MH "Functional Status") and (MH "Pain Measurement") as controlled terms.]</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD008465.pub2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="724.5" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Health-related quality of life outcomes in randomized controlled trials in metastatic hormone-sensitive prostate cancer: a systematic review</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Osanto S, 2024</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>eClinicalMedicine</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>9.6 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>To review how HRQoL was assessed and reported in phase III randomised trials comparing treatment arms in metastatic hormone-sensitive prostate cancer. Included for two reasons: it is one of only two records in this collection with a published Web of Science strategy, and its HRQoL/PRO block is the broadest - it treats anxiety, depression, functional status, fatigue, pain, symptom burden, sexual and social functioning as facets of the same concept, which is exactly the union your review needs across categories 2, 3, 4, 6 and 7.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>P: Patients with metastatic hormone-sensitive prostate cancer (mHSPC).
+I: Systemic treatment arms of phase III RCTs (androgen deprivation therapy alone or
+   in combination with docetaxel, abiraterone, apalutamide, enzalutamide, darolutamide
+   or radiotherapy).
+C: The comparator arm of each trial (usually ADT alone).
+O: Health-related quality of life and patient-reported outcomes - instrument used,
+   domains, timing, compliance, statistical handling, and the direction of any
+   between-arm difference.</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[PubMed searched natively; restricted to publications from 1 January 2015.
+Supplementary Table 2, verbatim - the HRQoL/PRO block reproduced in full, the
+population and treatment blocks abbreviated:]
+Block 1 (population): ("Metastatic Hormone sensitive Prostate Cancer"[tw] OR
+  "mHSPC"[tw] OR "metastatic castration naive prostate cancer"[tw] OR ... [14 phrase
+  variants] ... OR (("Prostatic Neoplasms"[mesh] OR "prostate cancer"[tw] OR ...
+  [28 prostate-cancer phrase variants] ...) AND ("metastatic"[tw] OR "metasta*"[tw]
+  OR "oligometastatic"[tw] OR "oligometasta*"[tw])))
+AND
+Block 2 (treatment): ("androgen deprivation therapy"[tw] OR "androgen depriv*"[tw]
+  OR "androgen block*"[tw] OR "ADT"[tiab] OR "Androgen Antagonists"[Mesh]
+  OR "Androgen Antagonists"[Pharmacological Action])
+AND
+Block 3 (HRQoL / patient-reported outcomes) - verbatim:
+  ("Quality of Life"[mesh] OR "Quality of Life"[tw] OR "Life Quality"[tw]
+  OR "HR-QoL"[tw] OR "HRQoL"[tw] OR "QoL"[tw] OR "PROs"[tw]
+  OR "Patient Reported Outcome Measures"[Mesh] OR "Patient Reported Outcome"[tw]
+  OR "Patient Reported Outcomes"[tw] OR "Patient Reported"[tw] OR "Anxiety"[mesh]
+  OR "anxiety"[tw] OR "Depression"[mesh] OR "depression"[tw]
+  OR "Psychological Distress"[mesh] OR "distress"[tw] OR "emotional"[tw]
+  OR "Functional Status"[Mesh] OR "functional status"[tw] OR "health outcomes"[tw]
+  OR "health related quality of life"[tw] OR "Health Status"[Mesh]
+  OR "health status"[tw] OR "HRQL"[tw] OR "patient outcomes"[tw] OR "PRO"[tw]
+  OR "psychological"[tw] OR "psychosocial"[tw] OR "sexual functioning"[tw]
+  OR "Sexuality"[Mesh] OR "Sexual Behavior"[Mesh] OR "Social Interaction"[Mesh]
+  OR "social functioning"[tw] OR "social wellbeing"[tw] OR "social"[tw]
+  OR "Symptom Assessment"[Mesh] OR "symptom assessment"[tw]
+  OR "symptom burden"[tw] OR "symptom distress"[tw] OR "Fatigue"[mesh]
+  OR "fatigue"[tw] OR "Pain"[mesh] OR "pain"[tw])
+AND
+Block 4 (design): ("randomized controlled trial"[pt] OR "randomized"[ti]
+  OR "randomised"[ti] OR "RCT"[ti] OR "trial"[ti] OR "Clinical Trial, Phase III"[pt]
+  OR "phase iii"[tw] OR "phase three"[tw] OR "phase 3"[tw] OR "phaseiii"[tw]
+  OR "phasethree"[tw] OR "phase3"[tw])
+NOT "review"[pt] AND english[la] AND ("2015/01/01"[PDAT] : "3000/12/31"[PDAT])
+NOT (phase II publication types and title terms, unless also phase III)</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>[Embase (OVID version), same date limits. Supplementary Table 2, verbatim - structure
+reproduced, population block abbreviated:]
+(("Metastatic Hormone sensitive Prostate Cancer".ti,ab OR "mHSPC".ti,ab OR ...
+[same phrase variants] ... OR ((exp *"Prostatic Cancer"/ OR "prostate cancer".ti,ab
+OR ... ) ADJ4 ("metastatic".ti,ab OR "metasta*".ti,ab OR "oligometastatic".ti,ab
+OR "oligometasta*".ti,ab)))
+AND ("androgen deprivation therapy".ti,ab OR "androgen depriv*".ti,ab
+OR "androgen block*".ti,ab OR "ADT".ti,ab OR "Androgen deprivation therapy"/
+OR exp *"antiandrogen"/)
+AND (exp *"Quality of Life"/ OR "Quality of Life".ti,ab OR ... [the same
+40-term PRO list, expressed as Emtree explosions plus .ti,ab text words] ...)
+AND [phase III / randomised design filter] NOT review NOT meeting abstract,
+English, 2015 onwards.
+Note the population block uses ADJ4 in Embase where PubMed used a plain AND, so the
+Embase run is the more specific of the two.</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>[Web of Science searched. Supplementary Table 2, verbatim - the topic block
+reproduced in full, population block abbreviated:]
+((TI=("Metastatic Hormone sensitive Prostate Cancer" OR "mHSPC" OR ... [phrase
+variants] ... OR (("Prostatic Cancer" OR "prostate cancer" OR ...) AND "metastatic"))
+OR AB=(... same phrase variants ... OR (("Prostatic Cancer" OR "prostate cancer"
+OR ...) NEAR/5 ("metastatic" OR "metasta*" OR "oligometastatic" OR "oligometasta*"))))
+AND (TI=("androgen deprivation therapy" OR "androgen depriv*" OR "androgen block*"
+OR "ADT" OR "Androgen deprivation therapy" OR "antiandrogen")
+OR AB=("androgen deprivation therapy" OR "androgen depriv*" OR "androgen block*"
+OR "ADT" OR "Androgen deprivation therapy" OR "antiandrogen"))
+AND TS=("Quality of Life" OR "Quality of Life" OR "Life Quality" OR "HR-QoL"
+OR "HRQoL" OR "QoL" OR "PROs" OR "Patient-Reported Outcome"
+OR "Patient Reported Outcome" OR "Patient Reported Outcomes" OR "Patient Reported"
+OR "Anxiety" OR "anxiety" OR "Depression" OR "depression" OR "Distress Syndrome"
+OR "distress" OR "emotional" OR "Functional Status" OR "functional status"
+OR "health outcomes" OR "health related quality of life" OR "Health Status"
+OR "health status" OR "HRQL" OR "patient outcomes" OR "PRO" OR "psychological"
+OR "psychosocial" OR "sexual functioning" OR "Sexuality" OR "Sexual behavior"
+OR "Social Interaction" OR "social functioning" OR "social wellbeing" OR "social"
+OR "Symptom Assessment" OR "symptom assessment" OR "symptom burden"
+OR "symptom distress" OR "Fatigue" OR "fatigue" OR "Pain" OR "pain")
+AND TI=("randomized controlled trial" OR "controlled clinical trial" OR "randomized"
+OR "randomised" OR "RCT" OR "trial" OR "phase 3 clinical trial" OR "phase iii"
+OR "phase three" OR "phase 3" OR "phaseiii" OR "phasethree" OR "phase3")
+NOT DT=review AND la=english
+AND py=(2015 OR 2016 OR 2017 OR 2018 OR 2019 OR 2020 OR 2021 OR 2022 OR 2023)
+NOT dt=(meeting abstract)
+NOT (TI=("phase 2 clinical trial" OR "phase ii" OR "phase two" OR "phase 2"
+OR "phaseii" OR "phasetwo" OR "phase2") NOT TS=("phase 3 clinical trial" OR ...))
+This is the most complete Web of Science template in the collection: note TI=/AB=
+used separately where PubMed uses [tw], TS= for the topic block, NEAR/5 replacing
+ADJ4, DT= for document type, la= for language and py= for an explicit year list.
+Google Scholar and the Cochrane Library were also searched.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.eclinm.2024.102922</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="760" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Yoga for improving health-related quality of life, mental health and cancer-related symptoms in women diagnosed with breast cancer</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Cramer H, 2017</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>To assess the effects of yoga on health-related quality of life, mental health and cancer-related symptoms among women diagnosed with breast cancer, during or after active treatment. Included as the contrast case, and because it is restricted to women: HRQoL is the first-named outcome in the title and the primary outcome of the review, yet no quality-of-life, mental-health or symptom term appears anywhere in any of the six search strategies.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>P: Women with a diagnosis of breast cancer, receiving active treatment or having
+   completed treatment.
+I: Yoga (including asana, pranayama, dhyana, dharana, meditation).
+C: No therapy, or another active intervention (psychosocial/educational, exercise).
+O: Health-related quality of life; mental health (depression, anxiety); cancer-related
+   symptoms (fatigue, sleep disturbance); adverse events.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>[MEDLINE searched via PubMed on 29 January 2016. Appendix 1, verbatim:]
+#1  yoga [mh]
+#2  yoga* [tiab]
+#3  yogic [tiab]
+#4  meditation [tiab]
+#5  asana* [tiab]
+#6  pranayama [tiab]
+#7  dharana [tiab]
+#8  dhyana [tiab]
+#9  #1 OR #2 OR #3 OR #4 OR #5 OR #6 OR #7 OR #8
+#10 breast neoplasms [mh]
+#11 breast neoplasm* [tiab]
+#12 breast cancer [tiab]
+#13 breast carcinoma* [tiab]
+#14 breast tumor* [tiab]
+#15 mamma carcinoma* [tiab]
+#16 mammary neoplasm* [tiab]
+#17 mammary carcinoma* [tiab]
+#18 mammary gland carcinoma* [tiab]
+#19 #10 OR #11 OR #12 OR #13 OR #14 OR #15 OR #16 OR #17 OR #18
+#20 randomized controlled trial [pt]
+#21 controlled clinical trial [pt]
+#22 randomized [tiab]
+#23 placebo [tiab]
+#24 clinical trials as topic [mesh: noexp]
+#25 randomly [tiab]
+#26 trial [ti]
+#27 #19 OR #20 OR #21 OR #22 OR #23 OR #24 OR #25 OR #26
+#28 Search #7 AND #17 AND #25
+#29 Search animals[mh] NOT humans[mh]
+#30 Search #26 NOT #27
+Three problems in the published appendix, all worth noting before reuse: line #27
+unions the population set (#19) with the design terms instead of unioning the design
+terms alone; line #28 combines single line numbers (#7 = dharana, #17 = mammary
+carcinoma*, #25 = randomly) rather than the three set unions #9, #19 and #27; and
+line #30 subtracts #27 from #26 rather than #29 from #28. What was run was almost
+certainly #9 AND #19 AND (design union) NOT (animals not humans).
+There is no HRQoL, mental-health or symptom block.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>[Embase searched 29 January 2016. Appendix 2 gives two versions.
+Embase.com syntax, verbatim:]
+#1  random* OR factorial* OR crossover* OR cross NEXT/1 over* OR placebo*
+    OR (doubl* AND blind*) OR (singl* AND blind*) OR assign* OR allocat*
+    OR volunteer* OR 'crossover procedure'/exp OR 'double blind procedure'/exp
+    OR 'randomized controlled trial'/exp OR 'single blind procedure'/exp
+#2  'breast neoplasm'
+#3  'breast cancer'/exp OR 'breast cancer'
+#4  'breast tumour'
+#5  'breast tumor'/exp OR 'breast tumor'
+#6  'breast carcinoma'/exp OR 'breast carcinoma'
+#7  'mamma carcinoma'/exp OR 'mamma carcinoma'
+#8  'mammary neoplasm'
+#9  'mammary carcinoma'/exp OR 'mammary carcinoma'
+#10 'mammary gland carcinoma'
+#11 #2 OR #3 OR #4 OR #5 OR #6 OR #7 OR #8 OR #9 OR #10
+#12 'breast cancer survivor'
+#13 'breast cancer survivors'
+#14 #12 OR #13
+#15 #11 OR #14
+#16 'yoga'/exp OR yoga
+#17 yogic
+#18 asana
+#19 pranayama
+#20 dhyana
+#21 dharana
+#22 'meditation'/exp OR meditation
+#23 #16 OR #17 OR #18 OR #19 OR #20 OR #21 OR #22
+#24 #1 AND #11 AND #23
+#25 #24 NOT ([animals]/lim NOT [humans]/lim)
+#26 #25 AND [embase]/lim
+[Embase via OvidSP, verbatim:]
+1-19  [Ovid Embase RCT filter: Randomized controlled trial/; Controlled clinical
+      study/; Random$.ti,ab.; randomization/; intermethod comparison/; placebo.ti,ab.;
+      (compare or compared or comparison).ti.; ((evaluated or evaluate or evaluating
+      or assessed or assess) and (compare or compared or comparing or comparison)).ab.;
+      (open adj label).ti,ab.; ((double or single or doubly or singly) adj (blind or
+      blinded or blindly)).ti,ab.; double blind procedure/; parallel group$1.ti,ab.;
+      (crossover or cross over).ti,ab.; ((assign$ or match or matched or allocation)
+      adj5 (alternate or group$1 or intervention$1 or patient$1 or subject$1 or
+      participant$1)).ti,ab.; (assigned or allocated).ti,ab.; (controlled adj7 (study
+      or design or trial)).ti,ab.; (volunteer or volunteers).ti,ab.; human experiment/;
+      trial.ti.]
+20    or/1-19
+21    exp breast/
+22    exp breast disease/
+23    (21 or 22) and exp neoplasm/
+24    exp breast tumor/
+25    exp breast cancer/
+26    exp breast carcinoma/
+27    (breast$ adj5 (neoplas$ or cancer$ or carcin$ or tumo$ or metasta$
+      or malig$)).ti,ab.
+28    or/21-27
+29    exp yoga/
+30    (yora or yogic or asana or pranayama or dhyana or dharana or meditation).tw.
+31    exp meditation/
+32    29 or 30 or 31
+33    20 and 28 and 32
+34    limit 33 to embase
+("yora" in line 30 is a typo for yoga.)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were the Cochrane Breast Cancer Specialised Register,
+MEDLINE via PubMed (Appendix 1), Embase (Appendix 2), CENTRAL 2016 Issue 1
+(Appendix 3), the WHO ICTRP portal (Appendix 4), ClinicalTrials.gov (Appendix 5) and
+IndMed (Appendix 6), all to 29 January 2016. Web of Science was not used.
+[CENTRAL strategy (Appendix 3), verbatim:
+#1 MeSH descriptor: [Breast Neoplasms] explode all trees
+#2 breast near cancer*
+#3 breast near neoplasm*
+#4 breast near carcinoma*
+#5 breast near tumour*
+#6 breast near tumor*
+#7 #1 or #2 or #3 or #4 or #5 or #6
+#8 MeSH descriptor: [Yoga] explode all trees
+#9 MeSH descriptor: [Meditation] explode all trees
+#10 yoga or yogic or meditation or asana or pranayama or dharana or dhyana
+#11 #8 or #9 or #10
+#12 #7 and #11]</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD010802.pub2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add category 7: patients' symptoms
Reeve 2014 (JNCI) is the paper that defines the 12-symptom core set in the brief;
its own search was two terms. Balitsky 2024 (JAMA Netw Open) has information-
specialist strategies for five databases. Ream 2020 (Cochrane) analyses symptoms
one by one and searches for none of them.

Records the negative finding: no JIF>=5 review enumerates the 12 symptoms as a
search block, and points to the nearest reusable material.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Depression" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Nutritional status" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 HRQOL" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Patients' symptoms" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
@@ -21,6 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 Depression'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5 Nutritional status'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6 HRQOL'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'7 Patients'' symptoms'!$A$2:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3524,4 +3526,433 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>07. Patients' symptoms (fatigue, insomnia, pain, anorexia, dyspnea, cognitive problems, anxiety, nausea, depression, sensory neuropathy, constipation, diarrhea)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1st author / year</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Impact factor</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Purpose of the study</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PICO</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - PubMed / MEDLINE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Embase</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Web of Science</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="241.5" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Recommended patient-reported core set of symptoms to measure in adult cancer treatment trials</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Reeve BB, 2014</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Journal of the National Cancer Institute</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>9.9 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>To derive, by systematic review plus analysis of six large datasets and multistakeholder consensus, a core set of patient-reported symptoms for adult cancer treatment trials. This is the paper that produced the 12 symptoms in the brief - fatigue, insomnia, pain, anorexia (appetite loss), dyspnea, cognitive problems, anxiety (includes worry), nausea, depression (includes sadness), sensory neuropathy, constipation and diarrhea. Included as the anchor reference for the category, and as a caution: the paper that defines the symptom set retrieved its evidence with a two-term search.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>P: Adults (&gt;= 18 years) with cancer, across diverse cancer populations and treatment
+   modalities.
+I: Anticancer treatment (any modality) in clinical trials measuring a patient-reported
+   outcome.
+C: Not applicable - this is a core-outcome-set derivation, not a comparative review.
+O: Which symptoms should form a core set, judged on prevalence across cancer
+   populations, impact on health outcomes and quality of life, and attribution to
+   disease or to anticancer treatment.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>[Reported in full in the Literature Review section, verbatim:]
+"Search terms included 'multiple symptoms' and 'cancer' and was limited to adults
+(aged 18 years or older) and to reports published in English between 2001 and 2011.
+This strategy identified 55 publications..."
+The review itself is reported as "described elsewhere" - in Reilly CM et al.,
+"A literature synthesis of symptom prevalence and severity in persons receiving
+active cancer treatment", Support Care Cancer 2013;21:1525-50 - which extended
+Kim et al.'s earlier synthesis of studies using the Symptom Distress Scale, the
+M.D. Anderson Symptom Inventory and the Memorial Symptom Assessment Scale.
+No database name, interface, field tag or line-numbered strategy is given. The 12
+symptoms are an output of the review; none of them is an input to the search.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Not reported. No database is named in the paper; the search is described only by the
+two terms above, and the underlying review is cited to Reilly 2013.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Not reported. See above.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/jnci/dju129</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="632.5" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Patient-Reported Outcome Measures in Cancer Care: An Updated Systematic Review and Meta-Analysis</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Balitsky AK, 2024</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>JAMA Network Open</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>10.5 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>To determine whether integrating patient-reported outcome measures into cancer care is associated with patient-related, therapy-related and health-care-utilisation outcomes. Included because it is the best-documented symptom-adjacent strategy at this impact level: an information specialist's line-numbered strategies for five databases, run twice (an original search and a 2022 update), with per-database yields reported. The symptom concept is expressed at one level of abstraction - "patient reported outcome(s)" AND (inventory or instrument* or measure* or self-report*) - rather than by naming symptoms.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>P: Adults (&gt;= 18 years) with active cancer receiving anticancer therapy (survivors
+   excluded).
+I: Administration of a patient-reported outcome measure, with results shared with the
+   patient's health care professional.
+C: Standard care without PROM administration.
+O: Patient-related outcomes (HRQOL, symptom control, patient-clinician communication);
+   therapy-related outcomes (treatment adherence, chemotherapy dose modification,
+   survival); health care utilisation (emergency visits, hospital admissions).</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[Not searched as PubMed. Ovid MEDLINE and MEDLINE Epub Ahead of Print, In-Process and
+other non-indexed citations, 1946 to present; searches to 26 September 2022.
+eAppendix in Supplement 1, verbatim (result counts as printed):]
+1  exp Neoplasms/ (3489255)
+2  (cancer* or neoplasm* or carcinoma* or oncol* or malignan* or tumor* or leukemia*
+   or leukaemia* or sarcoma* or lymphoma* or melanoma* or blastoma*
+   or myeloma*).mp. (4606954)
+3  1 or 2 (4799855)
+4  (patient reported outcomes or patient reported outcome or patient based outcome
+   or patient reported outcome measure$).mp. (27045)
+5  (inventory or instrument* or measure* or self-report*).ti,ab. (3825061)
+6  4 and 5 (17872)
+7  3 and 6 (3253)
+8  Epidemiologic Studies/ (8708)
+9  exp Case-Control Studies/ (1189370)
+10 exp Cohort Studies/ (2159240)
+11 Case control.tw. (134508)
+12 (cohort adj (study or studies)).tw. (238711)
+13 Cohort analy$.tw. (9174)
+14 (Follow up adj (study or studies)).tw. (51361)
+15 (observational adj (study or studies)).tw. (123476)
+16 Longitudinal.tw. (268228)
+17 Retrospective.tw. (597112)
+18 Cross sectional.tw. (400545)
+19 Cross-sectional studies/ (372470)
+20 or/8-19 (3264389)
+21 exp animals/ not humans.sh. (4849833)
+22 20 not 21 (3196743)
+23 7 and 22 (1296)
+24 randomized controlled trial.pt. (534665)
+25 controlled clinical trial.pt. (94229)
+26 randomi?ed.ab. (626711)
+27 placebo.ab. (219040)
+28 drug therapy.fs. (2336519)
+29 randomly.ab. (359969)
+30 trial.ab. (556534)
+31 groups.ab. (2209788)
+32 or/24-31 (5054529)
+33 exp animals/ not humans.sh. (4849833)
+34 32 not 33 (4396229)
+35 7 and 34 (1463)
+36 23 or 35 (2191)
+37 limit 36 to yr="2012 -Current" (2030)</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>[Embase via OvidSP, 1974 to 2021 (original search) and 1996 to 23 September 2022
+(update). eAppendix in Supplement 1, verbatim (population and PRO blocks; the
+observational filter is lines 8-23 and the RCT filter lines 25-44):]
+1  exp malignant neoplasm/ (3666710)
+2  (cancer* or neoplasm* or carcinoma* or oncol* or malignan* or tumor* or leukemia*
+   or leukaemia* or sarcoma* or lymphoma* or melanoma* or blastoma*
+   or myeloma*).mp. (6022711)
+3  1 or 2 (6089519)
+4  (patient reported outcomes or patient reported outcome or patient based outcome
+   or patient reported outcome measure$).mp. (49934)
+5  (inventory or instrument* or measure* or self-report*).ti,ab. (4948202)
+6  4 and 5 (31490)
+7  3 and 6 (6768)
+8-23  [observational-study filter: clinical study/; case control study/; family study/;
+      longitudinal study/; retrospective study/; prospective study/ not randomized
+      controlled trials/; cohort analysis/; and .mp. adjacency lines for cohort,
+      case control, follow up, observational, epidemiologic$ and cross sectional
+      "study or studies"]
+24 7 and 23 (2301)
+25-44 [Embase RCT filter: randomized controlled trial/; Controlled clinical study/;
+      random$.ti,ab.; randomization/; intermethod comparison/; placebo.ti,ab.;
+      (compare or compared or comparison).ti.; ((evaluated or evaluate or evaluating
+      or assessed or assess) and (compare or compared or comparing or comparison)).ab.;
+      (open adj label).ti,ab.; ((double or single or doubly or singly) adj (blind or
+      blinded or blindly)).ti,ab.; double blind procedure/; parallel group$1.ti,ab.;
+      (crossover or cross over).ti,ab.; ((assign$ or match or matched or allocation)
+      adj5 (alternate or group$1 or intervention$1 or patient$1 or subject$1 or
+      participant$1)).ti,ab.; (assigned or allocated).ti,ab.; (controlled adj7 (study
+      or design or trial)).ti,ab.; (volunteer or volunteers).ti,ab.; human experiment/;
+      trial.ti.]
+Yields by database for the updated search: MEDLINE, Embase, PsycInfo 605, CENTRAL 3434,
+CINAHL 1866; subtotal 13 857, 3554 after limits, 1049 duplicates removed.</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were MEDLINE and MEDLINE Epub ahead of print
+(OvidSP), Embase (OvidSP), PsycINFO (OvidSP), CENTRAL and CINAHL (EBSCO), from
+1 January 2012 to 26 September 2022, with no language or publication-status
+restriction. The search from the 2014 predecessor review was re-run first
+(eAppendices 1 and 2). Web of Science was not used.
+[The CINAHL translation (EBSCOhost) is given in the same appendix and shows the PRO
+concept in EBSCO syntax:
+S4  (MH "Patient-Reported Outcomes")
+S5  TX patient reported outcome
+S6  TX patient reported outcomes
+S7  TX patient based outcome
+S8  TX patient reported outcome measure*
+S9  S5 OR S6 OR S7 OR S8
+S10 TX inventory or instrument* or measure* or self-report*
+S11 S9 AND S10
+S12 S4 OR S11
+S13 S3 AND S12]</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1001/jamanetworkopen.2024.24793</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="391" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Telephone interventions for symptom management in adults with cancer</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Ream E, 2020</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>To assess the effectiveness of telephone-delivered interventions for reducing symptoms associated with cancer and its treatment, to determine which symptoms are most responsive, and whether intervention configuration and dose modify the effect. Included because the review's own question is explicitly "which symptoms respond" - it analyses anxiety, depression, fatigue, emotional distress, pain and others as separate outcomes - and yet not one symptom term appears in any of the three search strategies. It is the clearest demonstration in this collection that a symptom-focused review can be built entirely on a population-plus-intervention search.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>P: Adults (&gt;= 18 years) with cancer, during or after treatment.
+I: Telephone-delivered interventions for symptom management, alone or with additional
+   face-to-face, printed or electronic support.
+C: Usual care or another intervention.
+O: Individual symptoms - anxiety, depression, fatigue, emotional distress, pain,
+   nausea and others; symptom clusters; quality of life; adverse events.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>[Not searched as PubMed. MEDLINE via Ovid. Appendix 2, verbatim:]
+1  exp Neoplasms/
+2  (neoplasm* or cancer* or carcinoma* or tumour* or adenocarcinoma* or leukemi*
+   or leukaemi* or lymphoma* or tumor* or malignan* or myeloma*).mp.
+3  exp Radiotherapy/
+4  (radiotherap* or radiation or radiochemotherap* or chemoradi* or chemotherap*).mp.
+5  1 or 2 or 3 or 4
+6  exp Telemedicine/
+7  (telemedicine or (tele adj medicine)).mp.
+8  (teleconsultation or (tele adj consultation)).mp.
+9  (remote* adj5 consultation*).mp.
+10 telephone*.mp.
+11 phone*.mp.
+12 cellphone*.mp.
+13 8 or 6 or 11 or 7 or 10 or 9 or 12
+14 "randomized controlled trial".pt.
+15 "controlled clinical trial".pt.
+16 randomized.ab.
+17 randomly.ab.
+18 trial.ab.
+19 groups.ab.
+20 18 or 19 or 16 or 17 or 15 or 14
+21 13 and 20 and 5
+Note that the population block folds treatment modality (radiotherapy, chemotherapy)
+into the cancer concept with OR rather than AND - a useful pattern if you want to
+capture treated populations without requiring the treatment to be indexed. There is
+no symptom block.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>[Embase via Ovid. Appendix 3, verbatim:]
+1  exp Neoplasm/
+2  (neoplasm* or cancer* or carcinoma* or tumour* or adenocarcinoma* or leukemi*
+   or leukaemi* or lymphoma* or tumor* or malignan* or myeloma*).mp.
+3  exp Radiotherapy/
+4  (radiotherap* or radiation or radiochemotherap* or chemoradi* or chemotherap*).mp
+5  1 or 2 or 3 or 4
+6  exp Telemedicine/
+7  (telemedicine or (tele adj medicine)).mp.
+8  (teleconsultation or (tele adj consultation)).mp.
+9  (remote* adj5 consultation*).mp.
+10 telephone*.mp.
+11 phone*.mp.
+12 cellphone*.mp.
+13 8 or 6 or 11 or 7 or 10 or 9 or 12
+14 exp Controlled Clinical Trial/
+15 randomized.ab.
+16 randomly.ab.
+17 trial.ab.
+18 groups.ab.
+19 18 or 16 or 17 or 15 or 14
+20 19 and 13 and 5</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. Databases searched were CENTRAL, MEDLINE (Ovid), Embase (Ovid),
+PsycINFO, CINAHL and British Nursing Index, plus trial registries and reference
+lists. Web of Science was not used.
+[CENTRAL strategy (Appendix 1), verbatim:
+#1 MeSH descriptor Neoplasms explode all trees
+#2 neoplasm* or cancer* or carcinoma* or tumour* or adenocarcinoma* or leukemi*
+   or leukaemi* or lymphoma* or tumor* or malignan* or myeloma*
+#3 MeSH descriptor Radiotherapy explode all trees
+#4 radiotherap* or radiation or radiochemotherap* or chemoradi* or chemotherap*
+#5 (#1 OR #2 OR #3 OR #4)
+#6 MeSH descriptor Telemedicine explode all trees
+#7 telemedicine or (tele next medicine)
+#8 teleconsultation or (tele next consultation)
+#9 telephone*
+#10 phone*
+#11 cellphone*
+#12 remote* near/5 consultation*
+#13 (#6 OR #7 OR #8 OR #9 OR #10 OR #11 OR #12)
+#14 (#5 AND #13)]</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD007568.pub2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add category 8: patients' satisfaction - all 8 sheets now populated
Jacobsen 2018 (JCO) has the only genuine named outcome block in the collection,
pairing "patient satisfaction" free text with "Patient Satisfaction"[Mesh].
Gomes 2013 (Cochrane) names satisfaction in its objectives and searches twelve
databases without a satisfaction term. Shao 2025 (Int J Nurs Stud) searched
Web of Science and treats satisfaction and patient experience as separate
constructs.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Nutritional status" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 HRQOL" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Patients' symptoms" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Patients' satisfaction" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
@@ -23,6 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5 Nutritional status'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6 HRQOL'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'7 Patients'' symptoms'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'8 Patients'' satisfaction'!$A$2:$J$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3955,4 +3957,410 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>08. Patients' satisfaction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1st author / year</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Impact factor</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Purpose of the study</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>PICO</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - PubMed / MEDLINE</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Embase</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Search terms / strings - Web of Science</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="529" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Systematic Review of the Impact of Cancer Survivorship Care Plans on Health Outcomes and Health Care Delivery</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Jacobsen PB, 2018</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Journal of Clinical Oncology</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>42.1 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>To determine what impact providing a survivorship care plan has on health outcomes and health care delivery for people diagnosed with cancer, with satisfaction with care as one of the health-care-experience outcomes. Included because its fourth search set is an explicit patient-centred outcome block - the clearest published example in this collection of retrieving on satisfaction rather than screening for it.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>P: Individuals diagnosed with cancer.
+I: Survivor or care-provider receipt of a survivorship care plan (SCP).
+C: No receipt of an SCP, an alternative method of receiving an SCP, or no comparison
+   (for non-randomised studies).
+O: Patient-reported health outcomes (e.g. quality of life); health care use; health
+   care costs; health outcomes (e.g. quality-adjusted life years); and health care
+   experience (e.g. satisfaction with care).</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>[PubMed/MEDLINE searched natively. Search strategy printed in the Appendix, verbatim -
+four sets combined as 1 AND 2 AND 3 AND 4:]
+1 (Cancer OR Cancers OR Neoplasm OR Neoplasms OR Neoplasia OR "Neoplasms"[Mesh])
+2 (("care planning" OR "care plan*" OR "survivorship care plan*" OR "Follow-up care"
+  OR "follow up care" OR ("follow up" AND care) OR (follow-up AND care)
+  OR "continuity of care" OR "continual care" OR "continuous care"
+  OR "longitudinal care" OR "Patient Care Planning"[Mesh]
+  OR "Continuity of Patient Care"[Mesh]) AND (Survivor* OR Survivorship
+  OR "Survivors"[Mesh])
+3 ("Randomized controlled trial" OR "Non-randomized controlled trial"
+  OR "non-randomized controlled trial" OR "Randomized Controlled Trial"
+  [Publication Type] OR "Non-Randomized Controlled Trials as Topic"[Mesh])
+4 ("patient satisfaction" OR "quality of life" OR QOL OR Distress OR Understanding
+  OR "screening compliance" OR Feasibility OR ("care coordination" AND rating*)
+  OR "disease recurrence" OR "serious clinical event*" OR "social support"
+  OR "survival rate" OR "Treatment Outcome"[Mesh] OR "Patient Outcome
+  Assessment"[Mesh] OR "Patient Satisfaction"[Mesh] OR "Quality of Life"[Mesh]
+  OR "Stress, Psychological"[Mesh] OR "Comprehension"[Mesh]
+  OR "Patient Compliance"[Mesh] OR "Feasibility Studies"[Mesh]
+  OR "Recurrence"[Mesh] OR "Social Support"[Mesh] OR "Survival Rate"[Mesh])
+1 AND 2 AND 3 AND 4
+Set 4 is the reusable part: it pairs each free-text outcome phrase with its MeSH
+equivalent, so "patient satisfaction" and "Patient Satisfaction"[Mesh] both appear.
+Caveat before reuse: bare Understanding, Feasibility and Distress will retrieve very
+widely, and AND-ing an outcome set into the strategy will drop trials whose abstracts
+do not name the outcome.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Not reported. Only a PubMed/MEDLINE strategy is printed. The review states the search
+was supplemented by expert input on relevant publications.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Not reported. See above.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1200/JCO.2018.77.7482</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="760" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Effectiveness and cost-effectiveness of home palliative care services for adults with advanced illness and their caregivers</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Gomes B, 2013</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Cochrane Database of Systematic Reviews</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>8.8 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>To quantify the effect of home palliative care services on dying at home, and to examine their effect on other patient and caregiver outcomes including symptom control, quality of life, caregiver distress and satisfaction with care, together with resource use, costs and cost-effectiveness. Included as the large-scale contrast: satisfaction with care is named in objective 2, twelve databases were searched, and not one of the strategies contains a satisfaction term.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>P: Adults with advanced illness (the majority of included participants had cancer)
+   and their family caregivers.
+I: Home palliative care services - specialist teams providing palliative care at home.
+C: Usual care, or care without a home palliative care service.
+O: Dying at home (primary); symptom burden and control; quality of life; caregiver
+   distress and grief; satisfaction with care; resource use, costs and
+   cost-effectiveness.</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[Not searched as PubMed. MEDLINE via Ovid, 1950 to 21 November 2012; strategies
+refined with the Cochrane PaPaS Trials Search Co-ordinator. Appendix 1, verbatim
+(population/setting blocks in full; design filter summarised):]
+1  exp Palliative Care/
+2  exp Terminal Care/
+3  exp Terminally Ill/
+4  palliat*.mp.
+5  (terminal* and (care or caring or ill*)).mp.
+6  ((advanced or end stage or terminal*) adj4 (disease* or illness* or cancer*
+   or malignan*)).mp.
+7  (last year of life or LYOL or life's end or end of life).mp.
+8  or/1-7
+9  exp Home Care Services/
+10 exp Home Care Agencies/
+11 exp Mobile Health Units/
+12 exp Community Health Nursing/
+13 (home adj4 (hospital or palliat*)).mp.
+14 ((macmillan or marie curie or district) adj nurs*).mp.
+15 ((home or in-home or domicile or outreach or residential or housing or posthospital
+   or post-hospital or communit* or mobile or ambulatory or door to door) adj2
+   (team* or center* or centre* or treat* or care or interven* or therap* or
+   management or model* or program or programs or programme* or service* or base*
+   or nurs*)).mp.
+16 (homecare or home-care or homebased or home-based).mp.
+17 or/9-16
+18 hospice*.mp.
+19 18 or (8 and 17)
+20 (child* or adolescent* or infant* or baby or babies or neonat* or juvenil*
+   or pediatric* or paediatric* or young person* or young people or youth*
+   or young adult* or matern*).ti.
+21 19 not 20
+22-33 [randomised and controlled-trial design filter: clinical trial/ or controlled
+      clinical trial/ or multicenter study/ or randomized controlled trial/; the same
+      as publication types; chi-square distribution/ or chi-square?.ti,ab.;
+      "random*".ab,ti.; controlled.ti.; trial.ti.; Control Groups/; (control* adj2
+      (clinical or group* or trial* or study or studies or design* or method*)).ti,ab.;
+      ((multicent* or multi-cent* or multisite? or multi-site?) adj (study or studies
+      or trial*)).ti,ab.; double-blind method/ or single-blind method/;
+      ((single or double or triple or treble) adj blind*).ti,ab.]
+34-51 [non-randomised design filter: intervention?/pre-post/before-after/
+      quasi-experiment* terms, unioned]
+52 33 or 41 or 51
+53 groups.ab.
+54 52 or 53
+55 humans.sh.
+56 54 and 55
+57 56 and 21
+Line 19 is the useful pattern: hospice* alone, OR (palliative concept AND home
+setting concept) - a "named-entity OR concept-intersection" construction that is
+worth borrowing whenever one word reliably identifies the topic.
+There is no satisfaction, quality-of-life or symptom term anywhere in the strategy.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>[EMBASE, 1980 to 21 November 2012. Appendix 5, verbatim (population/setting blocks;
+design filter from line 25):]
+1  exp palliative therapy/
+2  exp palliative nursing/
+3  exp cancer palliative therapy/
+4  exp terminal care/
+5  exp terminal disease/
+6  exp terminally ill patient/
+7  palliat*.mp
+8  terminal* and (care or caring or ill*).mp
+9  ((advanced or end stage or terminal*) adj4 (disease* or illness* or cancer*
+   or malignan*)).mp
+10 last year of life or LYOL or or end of life.mp
+11 or/1-10
+12 exp home care/
+13 exp home health agency/
+14 exp community care/
+15 exp community health nursing/
+16 home adj4 (hospital or palliat*).mp
+17 (macmillan or marie curie or district) adj nurs*.mp
+18 (home or in-home or domicile or outreach or residential or housing or posthospital
+   or post-hospital or communit* or mobile or ambulatory or door to door) adj2
+   (team* or center* or centre* or treat* or care or interven* or therap* or
+   management or model* or program or programs or programme* or service* or base*
+   or nurs*).mp
+19 homecare or home-care or homebased or home-based.mp
+20 or/12-19
+21 hospice*.mp
+22 21 or (11 and 20)
+23 (child* or adolescent* or infant* or baby or babies or neonat* or juvenil*
+   or pediatric* or paediatric* or young person* or young people or youth*
+   or young adult* or matern*).ti.
+24 22 not 23
+25 onwards [Embase design filter: clinical trial/ or controlled clinical trial/ or
+   multicenter study/ or randomized controlled trial/; chi-square distribution/ or
+   chi-square?.ti,ab.; "random*".ab,ti.; controlled.ti.; and the rest as in MEDLINE]
+(Line 10 is printed with a duplicated "or".)</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Not searched. Twelve databases were searched: CENTRAL (21 November 2012), EMBASE
+(1980 to 21 November 2012), MEDLINE (1950 to 21 November 2012), the Cochrane PaPaS
+Trials Register and EPOC Trials Register (both 11 May 2010), CINAHL (1981 to
+13 April 2010), EURONHEED (1980 to 13 April 2010), PsycINFO (1806 to 13 April 2010),
+CDSR, DARE, the HTA Database and NHS EED (all 7 April 2010). Web of Science was not
+used.
+[The CENTRAL/CDSR/DARE/HTA/NHS EED strategy (Appendix 4) is the same design in
+Cochrane Library proximity syntax, and the shortest usable version of the concept is
+the PaPaS Trials Register line (Appendix 2), verbatim:
+hospice* or ((palliat* or terminal* or "end stage") and (home or community or
+outreach or ambulatory))]</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/14651858.CD007760.pub2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="287.5" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Development and application of patient-reported experience measures for cancer patients: a scoping review</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Shao Q, 2025</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>International Journal of Nursing Studies</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>7.5 (2023 JIF)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>To map the development, content and application of patient-reported experience measures (PREMs) for people with cancer, and to define what a PREM is relative to neighbouring constructs. Included for two reasons: it searched Web of Science, and it makes explicit a vocabulary problem that matters for your review - the authors deliberately excluded studies that measured patient satisfaction, quality of care or attitude scales rather than patient experience, treating satisfaction and experience as distinct constructs with distinct literatures.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>P: Patients with cancer (any type, any stage).
+Concept: Patient-reported experience measures - their development, psychometric
+   evaluation and domains.
+Context: National and international cancer-care initiatives; excluded were studies
+   measuring patient satisfaction, quality of care, attitude scales or PROMs rather
+   than patient experience, studies tied to one specific treatment, and studies where
+   proxies completed the measure.
+O: Number and identity of PREMs; definitions; evaluation status; domains of
+   application.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>[PubMed searched, from database inception to July 2024, using "a combination of
+subject terms and free-text words". The Methods give the concept groups verbatim
+rather than a line-numbered strategy:]
+Group 1 (population): 'cancer, oncology, malignancy, neoplasms'
+Group 2 (concept): 'patient experience, patient-reported experience,
+                    patient-reported experience measure'
+Group 3 (measurement): 'measure, tool, instrument, score, scale, survey,
+                    questionnaire, psychometrics'
+The paper states that the English terms "reported experience measure" and
+"measure, tool, instrument, score, scale, survey, questionnaire, psychometrics" were
+the ones applied in PubMed, Web of Science and MEDLINE. Reference lists of all
+retrieved articles were checked and Google Scholar was hand-searched.
+2216 records were reviewed and 24 included.
+Note there is no satisfaction term: satisfaction was an explicit exclusion criterion,
+not a search concept.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Not searched. The three databases searched were PubMed, Web of Science and MEDLINE.</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Searched. The Web of Science strategy is reproduced in the paper as Figure 1
+("Web of Science search strategies"), which is a bitmap image rather than text, so it
+cannot be transcribed verbatim here. What the Methods state in text is that the same
+three concept groups above were applied in Web of Science using a combination of
+subject terms and free-text words, from database inception to July 2024. Consult
+Figure 1 of the published article for the exact string.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.ijnurstu.2025.105077</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Sheet 2: replace Molenaar 2023 with Neo 2017, recovered via Unpaywall
Unpaywall identified a legal gold-OA copy of Neo 2017 (Cancer Treatment Reviews,
IF 9.6) in the King's College London repository, plus its supplementary Appendix 1
on the Elsevier CDN. That appendix carries the best functional-status block found
anywhere in this exercise: a thirteen-synonym ADL/functional-disability concept
plus the Activities of Daily Living MeSH explosion, with no intervention concept.

This was one of the three reviews previously recorded as unobtainable. Swapping it
in for Molenaar also drops Cochrane from 12/24 to 11/24 and gives sheet 2 a real
outcome block, which it previously lacked entirely.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -1068,142 +1068,115 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="713" customHeight="1">
+    <row r="3" ht="701.5" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prehabilitation versus no prehabilitation to improve functional capacity, reduce postoperative complications and improve quality of life in colorectal cancer surgery</t>
+          <t>Disability in activities of daily living among adults with cancer: a systematic review and meta-analysis</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Molenaar CJ, 2023</t>
+          <t>Neo J, 2017</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Cochrane Database of Systematic Reviews</t>
+          <t>Cancer Treatment Reviews</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>8.4 (2023 JIF, Cochrane Library)</t>
+          <t>9.6 (2023 JIF)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>To determine the effects of multimodal prehabilitation programmes on functional capacity, postoperative complications and quality of life in adults undergoing surgery for colorectal cancer. Functional capacity (6-minute walk test, VO2 peak, handgrip strength) is the lead outcome, yet no functional-capacity terms appear anywhere in the search - the strategy is population AND surgery AND (each of four intervention components), run as four separate intersections.</t>
+          <t>To determine the prevalence of disability in activities of daily living among adults with cancer, which ADL items are most often affected, and which instruments are used to measure it. The best functional-status search block available in this impact band: the review has no intervention concept at all, and instead intersects a two-term cancer population with a thirteen-synonym functional-disability block and an observational-design filter. If you take one outcome block for functional status, take this one.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Adults with non-metastatic colorectal cancer scheduled for surgery.
-I: Multimodal prehabilitation (&gt;= two preoperative components from exercise,
-   nutrition, psychological support, smoking cessation).
-C: No prehabilitation (usual preoperative care).
-O: Functional capacity (6-minute walk test, VO2 peak, handgrip strength);
-   postoperative complications and mortality; health-related quality of life;
-   hospital length of stay.</t>
+          <t>P: Adults with cancer (any type, any stage, any treatment setting).
+I: Nil - the review deliberately has no intervention concept.
+C: Nil.
+O: Disability in activities of daily living (ADL) and instrumental activities of daily
+   living (IADL) - prevalence, affected items, and measurement instruments.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>[MEDLINE searched January 2021, reported in native PubMed syntax.
-Appendix 2, verbatim:]
-#1 Search ((("Colorectal Neoplasms"[Mesh] OR (("Neoplasms"[Mesh] OR carcinoma*[tiab]
-   OR neoplas*[tiab] OR tumour*[tiab] OR tumor*[tiab] OR cancer*[tiab] OR cancer[sb]
-   OR oncolog*[tiab] OR malignan*[tiab] OR carcinogen*[tiab] OR oncogen*[tiab]
-   AND (colorectal*[tiab] OR colon*[tiab] OR rectal*[tiab])))))
-#2 Search "surgery"[Subheading] OR "Surgical Procedures, Operative"[Mesh]
-   OR "Surgeons"[Mesh] OR "Perioperative Period"[Mesh] OR "Perioperative Care"[Mesh]
-   OR "Preoperative Care"[Mesh] OR "Perioperative Care"[Mesh:NoExp] OR surger*[tiab]
-   OR surgical*[tiab] OR surgeon*[tiab] OR operation*[tiab] OR operative*[tiab]
-   OR perioperati*[tiab] OR preoperati*[tiab] OR pre operati*[tiab]
-   OR peri operati*[tiab] OR anesthe*[tiab] OR anaesthe*[tiab] OR incisi*[tiab]
-   OR excisi*[tiab] OR invasive*[tiab] OR Prehab*[tiab]
-#3 Search (#1 AND #2)
-#4 Search "Exercise Therapy"[Mesh] OR "Exercise"[Mesh] OR "Physical Education and
-   Training"[Mesh] OR "Exercise Movement Techniques"[Mesh] OR remedial exercis*[tiab]
-   OR exercise therap*[tiab] OR rehabilitation exercis*[tiab] OR exercis*[tiab]
-   OR physical activit*[tiab] OR physical exercis*[tiab] OR aerobic exercis*[tiab]
-   OR exercise training*[tiab] OR isometric exercis*[tiab]
-   OR (Physical Education*[tiab] AND training) OR exercise movement Techni*[tiab]
-#5 Search (Psychosocial[tiab] OR psychologic*[tiab] OR "Cognitive Behavioral
-   Therapy"[Mesh] OR cognitive behav*[tiab] OR cognitive psychotherap*[tiab]
-   OR (cogniti*[tiab] AND therap*[tiab]) OR psychoeducation[tiab]
-   OR psycho-education[tiab])
-#6 Search "Nutrition Therapy"[Mesh] OR "Nutritional Status"[Mesh]
-   OR medical nutrition therap*[tiab] OR nutrition therap*[tiab] OR nutrition[tiab]
-#7 Search "Smoking Cessation"[Mesh] OR "Smoking"[Mesh] OR "Tobacco Use Cessation"[Mesh]
-   OR stopping smoking[tiab] OR smoking cessation*[tiab] OR giving up smoking*[tiab]
-   OR quitting smoking[tiab] smoking[tiab] OR smoking behav*[tiab]
-   OR smoking habit*[tiab] OR tobacco cessation[tiab]
-#8  Search #3 AND #4
-#9  Search #3 AND #5
-#10 Search #3 AND #6
-#11 Search #3 AND #7
-Note: no functional-capacity, physical-function or activities-of-daily-living terms
-appear in the strategy; the outcome was applied at screening.</t>
+          <t>[Not searched as PubMed. MEDLINE(R) via Ovid, 1946 to June 2016; search alerts run to
+November 2016. Online supplement, Appendix 1, verbatim - the review labels this the
+"example search strategy", adapted for the other 11 databases:]
+1  Cancer*.mp.
+2  exp Carcinoma/
+3  Carcinoma*.mp.
+4  1 or 2 or 3
+5  Function* disabilit*.mp.
+6  Function* outcome*.mp.
+7  Function* impairment*.mp.
+8  Function* status.mp.
+9  Function* performance.mp.
+10 Function* limitation*.mp.
+11 exp "Activities of Daily Living"/
+12 ADL.mp.
+13 (Activit* adj2 daily living).mp.
+14 (Instrumental Activit* adj2 daily living).mp.
+15 IADL.mp.
+16 Activit* limitation*.mp.
+17 Participation restriction*.mp.
+18 5 or 6 or 7 or 8 or 9 or 10 or 11 or 12 or 13 or 14 or 15 or 16 or 17
+19 Epidemiologic studies/
+20 exp case control studies/
+21 exp cohort studies/
+22 Case control.tw.
+23 (Cohort adj (study or studies)).tw.
+24 Cohort analy$.tw.
+25 (Follow up adj (study or studies)).tw.
+26 (Observational adj (study or studies)).tw.
+27 Longitudinal.tw.
+28 Retrospective.tw.
+29 Cross sectional.tw.
+30 Cross-sectional studies/
+31 19 or 20 or 21 or 22 or 23 or 24 or 25 or 26 or 27 or 28 or 29 or 30
+32 4 and 18 and 31
+33 Limit 32 to (English language and humans and "all adult (19 plus years)")
+key: adj = adjacent; exp = explode; mp = title, original title, abstract, subject
+heading, name of substance, and registry word; tw = text word.
+The supplement also gives the concept table the strategy was built from - Population:
+cancer, carcinoma. Intervention: nil. Comparison: nil. Outcome: functional
+disability, functional disabilities, functional outcome, functional impairment,
+functional limitation, functional status, functional performance, activities of daily
+living, ADL, instrumental activities of daily living, IADL, activity limitation,
+participation restriction. Study type: observational/epidemiologic/case-control/
+cohort/cohort analysis/longitudinal/retrospective/cross-sectional/follow-up/
+prospective/correlational studies.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>[Embase via Ovid, 1974 to 2021 week 4. Appendix 3, verbatim:]
-#1  exp colorectal tumor/
-#2  exp neoplasm/
-#3  (carcinoma* or neoplasm* or tumour* or tumor* or cancer* or oncolog* or malignan*
-    or carcinogen* or oncogen*).ab,ti.
-#4  2 or 3
-#5  (colorectal* or colon* or rectal*).ab,ti.
-#6  4 and 5
-#7  1 or 6
-#8  exp surgery/
-#9  exp surgeon/
-#10 exp perioperative period/
-#11 exp preoperative period/
-#12 (surger* or surgical* or surgeon* or operation* or operative* or perioperati*
-    or preoperati* or pre operati* or peri operati* or anesthe* or anaesthe*
-    or incisi* or excisi* or invasive* or Prehab*).ab,ti.
-#13 8 or 9 or 10 or 11 or 12
-#14 (remedial exercis* or exercise therap* or rehabilitation exercis* or exercis*
-    or physical activit* or physical exercis* or aerobic exercis* or exercise training*
-    or isometric exercis* or exercise movement techni*).ab,ti.
-#15 exp kinesiotherapy/
-#16 14 or 15
-#17 7 and 13 and 16
-#18 exp diet therapy/
-#19 exp nutritional status/
-#20 (medical nutrition therap* or nutrition therap* or nutrition).ab,ti.
-#21 18 or 19 or 20
-#22 7 and 13 and 21
-#23 exp cognitive behavioral therapy/
-#24 (Psychosocial or psychologic* or cognitive behav* or cognitive psychotherap*
-    or psychoeducation or psycho-education).ab,ti.
-#25 (cogniti* and therap*).ab,ti.
-#26 23 or 24 or 25
-#27 7 and 13 and 26
-#28 exp smoking cessation/
-#29 exp smoking/
-#30 (stopping smoking or smoking cessation* or giving up smoking* or quitting smoking
-    or smoking or smoking behav* or smoking habit* or tobacco cessation).ab,ti.
-#31 28 or 29 or 30
-#32 7 and 13 and 31</t>
+          <t>Searched, but no Embase-specific string was published. The Methods state that the
+strategy "was developed for MEDLINE and adapted where necessary for all other
+databases", and only the MEDLINE example is reproduced (Appendix 1). Twelve
+databases were searched from inception to June 2016: MEDLINE, EMBASE, CINAHL, ASSIA,
+PsycINFO, Social Policy and Practice, IBSS, ScienceDirect, Social Service Abstracts,
+Sociological Abstracts, Scopus and Web of Science Core Collection.</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Not searched. Databases searched were CENTRAL (Cochrane Library, 2021 week 4),
-MEDLINE (Ovid, 1950 to 2021 week 4), Embase (Ovid, 1974 to 2021 week 4) and PsycINFO
-(EBSCOhost, 1967 to 2021 week 4), plus ClinicalTrials.gov, Google Scholar, the
-Netherlands Trial Register and WHO ICTRP (to March 2021). Web of Science was not used.
-[PsycINFO strategy (Appendix 4) shows the same shape in EBSCOhost syntax:
-S1 DE "Neoplasms"; S2 TI colorectal cancer* OR AB colorectal cancer*; S3 DE "Surgery";
-S4 TI surger* OR AB surger*; S5 S1 OR S2; S6 S3 OR S4; S7 S5 AND S6;
-S8 DE "Psychosocial Rehabilitation"; ... S24 S7 AND S23]</t>
+          <t>Searched (Web of Science Core Collection, and Web of Science Conference Proceedings
+for grey literature), but no Web of Science-specific string was published - only the
+MEDLINE example strategy, adapted. Grey literature was additionally searched in
+OpenGrey, ProQuest Dissertations &amp; Theses, Scopus Conference Proceedings, HMIC and
+Global Health. No date restriction; limited to human studies published in English.
+This is one of only four reviews in the collection that searched Web of Science, and
+one of two that searched it without publishing the string.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1002/14651858.CD013259.pub3</t>
+          <t>https://doi.org/10.1016/j.ctrv.2017.10.006</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add strategies/ with complete unabbreviated search strategies for 7 reviews
The workbook cells condense long design filters and repeated term lists to stay
readable, which cost fidelity for anyone wanting to re-run a strategy rather than
read it. strategies/ now holds the full text for every database searched, for the
seven records where condensing happened, each with a provenance header naming the
appendix or supplement it came from. Published typos are preserved, not silently
fixed. All 21 affected cells now point to their file.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -1256,7 +1256,8 @@
 24 limit 23 to yr="1990 -Current"
 25 24 not 19
 26 19 or 24
-Note: no physical-function terms appear in the strategy.</t>
+Note: no physical-function terms appear in the strategy.
+[Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -1305,7 +1306,8 @@
 50 limit 49 to yr="1990 -Current"
 51 limit 50 to conference abstracts
 52 50 not 51
-53 52 not 45</t>
+53 52 not 45
+[Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -1328,7 +1330,8 @@
    or cancer* or tumor* or tumour* or oncol* or malign* or carcinom* or adenocarcinom*
    or adenoma or metasta*))):ti,ab,kw
 #8 [same term list combined with AND rather than near/3]:ti
-#9 #6 or #7 or #8 with Publication Year from 1990 to 2021, in Trials]</t>
+#9 #6 or #7 or #8 with Publication Year from 1990 to 2021, in Trials]
+[Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -2207,7 +2210,8 @@
 key: mp = title, abstract, original title, name of substance word, subject heading
 word, keyword heading word, protocol supplementary concept, rare disease
 supplementary concept, unique identifier; pt = publication type; ab = abstract;
-sh = subject heading; ti = title.</t>
+sh = subject heading; ti = title.
+[Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -2252,7 +2256,8 @@
 32 (exp animal/ or nonhuman/ or exp animal experiment/) not human/
 33 31 not 32
 Note "choriocrcinoma*" is a typo for choriocarcinoma* in the published Embase and
-CENTRAL appendices; the MEDLINE appendix spells it correctly.</t>
+CENTRAL appendices; the MEDLINE appendix spells it correctly.
+[Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -2275,7 +2280,8 @@
 #9 Any MeSH descriptor with qualifier(s): [Drug therapy - DT]
 #10-#16 [antidepressant class MeSH explosions and the ~70-agent drug-name list]
 #17 #9 or #10 or #11 or #12 or #13 or #14 or #15 or #16
-#18 #3 and #8 and #17]</t>
+#18 #3 and #8 and #17]
+[Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -2284,7 +2290,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="736" customHeight="1">
+    <row r="5" ht="759" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Aerobic Physical Activity and Depression Among Patients With Cancer: A Systematic Review and Meta-Analysis</t>
@@ -2360,7 +2366,8 @@
 31 exp animals/ not humans.sh
 32 30 not 31
 33 4 and 7 and 19 and 32
-   limit 33 to (english language and yr="1980 -Current")</t>
+   limit 33 to (english language and yr="1980 -Current")
+[Complete unabbreviated strategy, all databases: strategies/04_kulchycki2024_aerobic-activity-depression.txt]</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -2390,7 +2397,8 @@
 30 (exp animal/ or nonhuman/) not exp human/
 31 29 not 30
 32 4 and 7 and 19 and 31
-33 limit 32 to (english language and yr="1980 -Current")</t>
+33 limit 32 to (english language and yr="1980 -Current")
+[Complete unabbreviated strategy, all databases: strategies/04_kulchycki2024_aerobic-activity-depression.txt]</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -2419,7 +2427,8 @@
   or resilien*)
 ...
 25 #3 AND #4 AND #15 AND #24
-26 #25 AND PUBYEAR AFT 1979 AND ( LIMIT-TO ( LANGUAGE , "English" ) )]</t>
+26 #25 AND PUBYEAR AFT 1979 AND ( LIMIT-TO ( LANGUAGE , "English" ) )]
+[Complete unabbreviated strategy, all databases: strategies/04_kulchycki2024_aerobic-activity-depression.txt]</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -3107,7 +3116,8 @@
 74-76  Survivors/ ; survivor.mp. ; 74 or 75   [used to exclude survivorship trials,
        which are covered by the companion review]
 Note "qlc-c30" is a transposition of QLQ-C30, and "sta1" of STAI, in the published
-appendix. Repair both before reuse.</t>
+appendix. Repair both before reuse.
+[Complete unabbreviated strategy, all databases: strategies/06_mishra2012_hrqol.txt]</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -3160,7 +3170,8 @@
 72-74  Survivors/; survivor$.mp.; 72 or 73
 75     32 and 65 and 66 and 71
 76     75 not 74
-(Line 69 is printed as ".mp3" - a typo for .mp.; "stal" in line 58 is STAI.)</t>
+(Line 69 is printed as ".mp3" - a typo for .mp.; "stal" in line 58 is STAI.)
+[Complete unabbreviated strategy, all databases: strategies/06_mishra2012_hrqol.txt]</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -3176,7 +3187,8 @@
 language or date restriction. Trial registries (WHO ICTRP, Current Controlled Trials,
 CenterWatch, ClinicalTrials.gov), reference lists and expert contact were also used.
 [The CINAHL version (Appendix 4) is the same HRQoL set in EBSCOhost syntax and
-includes (MH "Functional Status") and (MH "Pain Measurement") as controlled terms.]</t>
+includes (MH "Functional Status") and (MH "Pain Measurement") as controlled terms.]
+[Complete unabbreviated strategy, all databases: strategies/06_mishra2012_hrqol.txt]</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -3185,7 +3197,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="724.5" customHeight="1">
+    <row r="4" ht="747.5" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Health-related quality of life outcomes in randomized controlled trials in metastatic hormone-sensitive prostate cancer: a systematic review</t>
@@ -3260,7 +3272,8 @@
   OR "phase iii"[tw] OR "phase three"[tw] OR "phase 3"[tw] OR "phaseiii"[tw]
   OR "phasethree"[tw] OR "phase3"[tw])
 NOT "review"[pt] AND english[la] AND ("2015/01/01"[PDAT] : "3000/12/31"[PDAT])
-NOT (phase II publication types and title terms, unless also phase III)</t>
+NOT (phase II publication types and title terms, unless also phase III)
+[Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -3279,7 +3292,8 @@
 AND [phase III / randomised design filter] NOT review NOT meeting abstract,
 English, 2015 onwards.
 Note the population block uses ADJ4 in Embase where PubMed used a plain AND, so the
-Embase run is the more specific of the two.</t>
+Embase run is the more specific of the two.
+[Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -3316,7 +3330,8 @@
 This is the most complete Web of Science template in the collection: note TI=/AB=
 used separately where PubMed uses [tw], TS= for the topic block, NEAR/5 replacing
 ADJ4, DT= for document type, la= for language and py= for an explicit year list.
-Google Scholar and the Cochrane Library were also searched.</t>
+Google Scholar and the Cochrane Library were also searched.
+[Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -3653,7 +3668,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="632.5" customHeight="1">
+    <row r="4" ht="655.5" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Patient-Reported Outcome Measures in Cancer Care: An Updated Systematic Review and Meta-Analysis</t>
@@ -3735,7 +3750,8 @@
 34 32 not 33 (4396229)
 35 7 and 34 (1463)
 36 23 or 35 (2191)
-37 limit 36 to yr="2012 -Current" (2030)</t>
+37 limit 36 to yr="2012 -Current" (2030)
+[Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -3771,7 +3787,8 @@
       or design or trial)).ti,ab.; (volunteer or volunteers).ti,ab.; human experiment/;
       trial.ti.]
 Yields by database for the updated search: MEDLINE, Embase, PsycInfo 605, CENTRAL 3434,
-CINAHL 1866; subtotal 13 857, 3554 after limits, 1049 duplicates removed.</t>
+CINAHL 1866; subtotal 13 857, 3554 after limits, 1049 duplicates removed.
+[Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -3792,7 +3809,8 @@
 S10 TX inventory or instrument* or measure* or self-report*
 S11 S9 AND S10
 S12 S4 OR S11
-S13 S3 AND S12]</t>
+S13 S3 AND S12]
+[Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -4185,7 +4203,8 @@
 Line 19 is the useful pattern: hospice* alone, OR (palliative concept AND home
 setting concept) - a "named-entity OR concept-intersection" construction that is
 worth borrowing whenever one word reliably identifies the topic.
-There is no satisfaction, quality-of-life or symptom term anywhere in the strategy.</t>
+There is no satisfaction, quality-of-life or symptom term anywhere in the strategy.
+[Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -4226,7 +4245,8 @@
 25 onwards [Embase design filter: clinical trial/ or controlled clinical trial/ or
    multicenter study/ or randomized controlled trial/; chi-square distribution/ or
    chi-square?.ti,ab.; "random*".ab,ti.; controlled.ti.; and the rest as in MEDLINE]
-(Line 10 is printed with a duplicated "or".)</t>
+(Line 10 is printed with a duplicated "or".)
+[Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -4241,7 +4261,8 @@
 Cochrane Library proximity syntax, and the shortest usable version of the concept is
 the PaPaS Trials Register line (Appendix 2), verbatim:
 hospice* or ((palliat* or terminal* or "end stage") and (home or community or
-outreach or ambulatory))]</t>
+outreach or ambulatory))]
+[Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add annex sheet 9: the ten reviews the IF>=5 rule excluded
Six are ovarian or gynaecological cancer specific and two are restricted to older
adults, so several are closer to the target population than records that made the
main sheets. Martin 2020 (older women, gynaecological cancer surgery, functional
recovery) is the best population-and-outcome match in the entire candidate pool and
fails only on impact factor.

All ten verified against PubMed for author, year, journal and DOI. build.py now
supports a per-category column set so the annex renders as a candidate list rather
than forcing empty strategy cells.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 HRQOL" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Patients' symptoms" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Patients' satisfaction" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Annex - excluded by IF rule" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
@@ -25,6 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6 HRQOL'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'7 Patients'' symptoms'!$A$2:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'8 Patients'' satisfaction'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'9 Annex - excluded by IF rule'!$A$2:$G$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4373,4 +4375,445 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>09. Annex: reviews excluded by the JIF &gt;= 5 rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1st author / year</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Impact factor</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Why it is relevant to this review</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Why it was excluded</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="57.5" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>A Systematic Review of Health-Related Quality of Life Reporting in Ovarian Cancer Phase III Clinical Trials</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Wilson MK, 2018</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>The Oncologist</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>~4.8</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>The single closest miss in the whole exercise. Ovarian cancer specific, HRQOL specific, and about phase III treatment trials - it maps onto category 6 and onto your review's population simultaneously. Would have replaced a breast or prostate cancer record on the HRQOL sheet.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>JIF ~4.8, just below the 5 threshold</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1634/theoncologist.2017-0297</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Nutritional Interventions to Improve Clinical Outcomes in Ovarian Cancer: A Systematic Review of Randomized Controlled Trials</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Rinninella E, 2019</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Nutrients</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>~4.8</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Ovarian cancer specific and nutrition specific. Would have given category 5 a second ovarian record alongside Billson 2013, and a more recent one.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>JIF ~4.8, just below the 5 threshold</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/nu11061404</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Depression and anxiety in ovarian cancer: a systematic review and meta-analysis of prevalence rates</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Watts S, 2015</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>BMJ Open</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>~2.4</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>The only ovarian-cancer-specific depression review found. A prevalence review, so depression is necessarily a search concept rather than a screening criterion - which is exactly the structure category 4 is about.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>JIF ~2.4</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1136/bmjopen-2015-007618</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Functional recovery in older women undergoing surgery for gynaecological malignancies: A systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Martin FE, 2020</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Geriatric Oncology</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>~3.0</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Older women, gynaecological cancer, surgical treatment, functional status. On paper this is the single best population-and-outcome match to your review in the entire candidate pool - it fails only on impact factor.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>JIF ~3.0</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jgo.2020.06.006</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Quality of life outcomes following surgery for advanced ovarian cancer: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Kumar S, 2019</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>International Journal of Gynecological Cancer</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>~4.1</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Ovarian cancer, surgical treatment, HRQOL outcome - the exact intersection of category 1 and category 6.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>JIF ~4.1</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1136/ijgc-2018-000125</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Ovarian cancer survivors' quality of life: a systematic review</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Ahmed-Lecheheb D, 2016</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Cancer Survivorship</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>~3.4</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Ovarian cancer specific HRQOL review covering the survivorship phase, which the records on sheet 6 do not.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>JIF ~3.4</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s11764-016-0525-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>A systematic review of patient values, preferences and expectations for the treatment of recurrent ovarian cancer</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>PEBC's Ovarian Oncology Guidelines Group, 2017</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Gynecologic Oncology</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>~4.5</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Ovarian cancer, treatment, and a patient-centred construct (values, preferences, expectations) adjacent to satisfaction. Relevant to categories 1 and 8 together, and to any patient-centred framing of a treatment review.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>JIF ~4.5</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.ygyno.2017.05.039</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Psychosocial interventions and quality of life in gynaecological cancer patients: a systematic review</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Hersch J, 2009</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Psycho-Oncology</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>~3.3</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Gynaecological cancer with HRQOL and psychological outcomes - closer in population to your review than the breast and prostate cancer records that occupy sheet 6.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>JIF ~3.3</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pon.1443</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Patient-Reported Physical Function Measures in Cancer Clinical Trials</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Atkinson TM, 2017</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Epidemiologic Reviews</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>~3.4-4.1</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>A five-component search built around physical function and PRO measurement properties, in native PubMed syntax. Would have strengthened category 2, though only the measurement-properties component is printed verbatim in the paper.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>JIF below 5; sources give ~3.4 (2024) to ~4.1 (2023)</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/epirev/mxx008</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Effects of patient navigation on satisfaction with cancer care: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Wells KJ, 2018</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Supportive Care in Cancer</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>~2.8</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>The most on-topic satisfaction review found anywhere - satisfaction with cancer care is the outcome, not a secondary endpoint. Directly relevant to category 8.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>JIF ~2.8</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s00520-018-4108-2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:G12"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Excel row-height ceiling, refresh all docs for the changes made
Excel's hard maximum row height is 409.5pt, so the previous 760pt setting was
silently clamped and 18 of 24 rows were visually truncated with no indication.
Rows are now capped at the real maximum and each sheet states which rows overflow
and where to read the full text.

Docs brought up to date: methods.md gains the Unpaywall retrieval route, the
verification section (CrossRef + executable checks, including the claim the PubMed
run disproved), and an explicit statement of the collection's biases. impact_factors.md
corrects the Cochrane record count, adds Cancer Treatment Reviews, and documents the
IJNS / IJNS Advances confusion as the failure mode the table exists to prevent.
README rewritten around the two deliverables.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -35,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +61,12 @@
     <font>
       <name val="Consolas"/>
       <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -107,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,6 +129,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -490,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -564,7 +573,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="471.5" customHeight="1">
+    <row r="3" ht="409" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Neoadjuvant chemotherapy before surgery versus surgery followed by chemotherapy for initial treatment in advanced epithelial ovarian cancer</t>
@@ -701,7 +710,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="506" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Interventions for the treatment of borderline ovarian tumours</t>
@@ -843,7 +852,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="414" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Optimal primary surgical treatment for advanced epithelial ovarian cancer</t>
@@ -981,9 +990,17 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rows 3, 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:J5"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -996,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1070,7 +1087,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="701.5" customHeight="1">
+    <row r="3" ht="409" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Disability in activities of daily living among adults with cancer: a systematic review and meta-analysis</t>
@@ -1182,7 +1199,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="760" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Physical function endpoints in cancer cachexia clinical trials: Systematic Review 1 of the cachexia endpoints series</t>
@@ -1422,9 +1439,17 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rows 3, 4: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:J5"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1437,7 +1462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1511,7 +1536,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="760" customHeight="1">
+    <row r="3" ht="409" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Non-pharmacological interventions for cognitive impairment due to systemic cancer treatment</t>
@@ -1687,7 +1712,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="655.5" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Long-term neurocognitive and other side effects of radiotherapy, with or without chemotherapy, for glioma</t>
@@ -1939,9 +1964,17 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rows 3, 4: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:J5"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1954,7 +1987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2121,7 +2154,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="760" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Antidepressants for the treatment of depression in people with cancer</t>
@@ -2292,7 +2325,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="759" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Aerobic Physical Activity and Depression Among Patients With Cancer: A Systematic Review and Meta-Analysis</t>
@@ -2439,9 +2472,17 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rows 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:J5"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2454,7 +2495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2528,7 +2569,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="736" customHeight="1">
+    <row r="3" ht="409" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Perioperative nutrition interventions for women with ovarian cancer</t>
@@ -2727,7 +2768,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="494.5" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Prevalence of and Survival with Cachexia among Patients with Cancer: A Systematic Review and Meta-Analysis</t>
@@ -2830,7 +2871,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="760" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Nutritional status, body composition and chemotherapy dosing in children and young people with cancer: a systematic review</t>
@@ -2941,9 +2982,17 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rows 3, 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:J5"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2956,7 +3005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3030,7 +3079,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="760" customHeight="1">
+    <row r="3" ht="409" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Exercise interventions on health-related quality of life for people with cancer during active treatment</t>
@@ -3199,7 +3248,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="747.5" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Health-related quality of life outcomes in randomized controlled trials in metastatic hormone-sensitive prostate cancer: a systematic review</t>
@@ -3342,7 +3391,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="760" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Yoga for improving health-related quality of life, mental health and cancer-related symptoms in women diagnosed with breast cancer</t>
@@ -3511,9 +3560,17 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rows 3, 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:J5"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3526,7 +3583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3670,7 +3727,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="655.5" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Patient-Reported Outcome Measures in Cancer Care: An Updated Systematic Review and Meta-Analysis</t>
@@ -3943,9 +4000,17 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rows 4: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:J5"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3958,7 +4023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4032,7 +4097,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="598" customHeight="1">
+    <row r="3" ht="409" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Systematic Review of the Impact of Cancer Survivorship Care Plans on Health Outcomes and Health Care Delivery</t>
@@ -4119,7 +4184,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="760" customHeight="1">
+    <row r="4" ht="409" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Effectiveness and cost-effectiveness of home palliative care services for adults with advanced illness and their caregivers</t>
@@ -4368,9 +4433,17 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rows 3, 4: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:J5"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Set the whole workbook to Arial 11
Changed in scripts/build.py rather than in the .xlsx, so it survives the next
rebuild. Header, body, sheet title and the overflow note now all use one
typeface; the Consolas monospace styling on the three search-string columns is
gone, along with the MONO_FONT/MONO_KEYS split that only existed to support it.

Row height now scales from FONT_SIZE rather than a hard-coded 11.5, so 11pt text
is not sitting in rows measured for 9pt.

Verified: all 414 non-empty cells across the nine sheets report Arial 11.0pt and
nothing else.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -35,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,29 +44,25 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <sz val="9"/>
+      <name val="Arial"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Consolas"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="007F7F7F"/>
-      <sz val="9"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -113,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -122,16 +118,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -608,7 +598,7 @@
    surgical morbidity/mortality.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE was searched via Silver Platter/Ovid,
 1966 to October week 1 2020; searches run 9 October 2020. Appendix 2, verbatim:]
@@ -643,7 +633,7 @@
 or investigation*) and (advanced or stage III or stage IV)]</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to 2020 week 40; searches run 9 October 2020.
 Appendix 1, verbatim:]
@@ -682,7 +672,7 @@
 or investigation*) and (advanced or stage III or stage IV)]</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL (2020, Issue 10), Embase via Ovid,
 MEDLINE (Silver Platter/Ovid), PDQ and MetaRegister; reference lists and trial
@@ -711,32 +701,32 @@
       </c>
     </row>
     <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Interventions for the treatment of borderline ovarian tumours</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Faluyi O, 2010</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Cochrane Database of Systematic Reviews</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>8.4 (2023 JIF, Cochrane Library)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>To evaluate the benefits and harms of different interventions (surgery, chemotherapy, radiotherapy, observation) in women with borderline ovarian tumours. Included as an exemplar of the broadest possible treatment concept: the review has no drug- or procedure-named intervention block at all. Instead, treatment is captured through floating subheadings (drug therapy, surgery, therapy, radiotherapy) folded into the study-design block, so that any treatment is retrievable.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>P: Women with borderline (low malignant potential) ovarian tumours.
 I: Any intervention for treatment - surgery (including fertility-sparing and
@@ -746,7 +736,7 @@
    adverse events; quality of life.</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1950 to week 3 2009. Appendix 1, verbatim:]
 1  exp Ovarian Neoplasms/
@@ -785,7 +775,7 @@
 word; ab = abstract; fs = floating subheading.</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to 2009 week 2. Appendix 2, verbatim:]
 1  Ovary Tumor/
@@ -826,7 +816,7 @@
 dt (drug therapy), su (surgery), th (therapy) and rt (radiotherapy).</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were the Cochrane Gynaecological Cancer Group
 Trials Register, CENTRAL, MEDLINE and EMBASE, plus reference lists and trial
@@ -846,7 +836,7 @@
 #12 (#10 OR #11)]</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD007696.pub2</t>
         </is>
@@ -889,7 +879,7 @@
 O: Overall survival; progression-free survival; adverse events; quality of life.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1950 to July week 3 2010
 (databases searched to August 2010). Appendix 1, verbatim:]
@@ -927,7 +917,7 @@
 word; fs = floating subheading; pt = publication type.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to week 30 2010. Appendix 2, verbatim:]
 1  exp Ovary Tumor/
@@ -959,7 +949,7 @@
 title, device manufacturer, drug manufacturer name; fs = floating subheading.</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were the Cochrane Gynaecological Cancer
 Collaborative Review Group Trials Register, CENTRAL (The Cochrane Library 2010,
@@ -991,7 +981,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Rows 3, 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
         </is>
@@ -1122,7 +1112,7 @@
    living (IADL) - prevalence, affected items, and measurement instruments.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE(R) via Ovid, 1946 to June 2016; search alerts run to
 November 2016. Online supplement, Appendix 1, verbatim - the review labels this the
@@ -1172,7 +1162,7 @@
 prospective/correlational studies.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Searched, but no Embase-specific string was published. The Methods state that the
 strategy "was developed for MEDLINE and adapted where necessary for all other
@@ -1182,7 +1172,7 @@
 Sociological Abstracts, Scopus and Web of Science Core Collection.</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Searched (Web of Science Core Collection, and Web of Science Conference Proceedings
 for grey literature), but no Web of Science-specific string was published - only the
@@ -1200,32 +1190,32 @@
       </c>
     </row>
     <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Physical function endpoints in cancer cachexia clinical trials: Systematic Review 1 of the cachexia endpoints series</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>McDonald J, 2023</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Journal of Cachexia, Sarcopenia and Muscle</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>9.4 (2023 JIF)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>To assess the frequency and diversity of physical function endpoints used in cancer cachexia clinical trials, and how often they change with intervention. Included as an exemplar of a librarian-built Ovid strategy in which physical function is the whole point of the review yet appears nowhere in the search: retrieval is population (cancer) AND condition (cachexia) AND study design, with physical function applied as an eligibility criterion.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>P: Adults (&gt;= 18 years) with cancer cachexia.
 I: Any cachexia intervention lasting more than 14 days (nutritional, pharmacological,
@@ -1235,7 +1225,7 @@
    up-and-go, physical activity, patient-reported physical function.</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. Ovid MEDLINE(R) ALL 1946 to 1 July 2021; search run
 2 June 2021 by a research librarian, University of Oslo. Appendix S1, verbatim:]
@@ -1279,7 +1269,7 @@
 [Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>[Embase Classic+Embase 1947 to 1 July 2021 via Ovid; run 2 June 2021.
 Appendix S1, verbatim (population/condition block; the design block is a long
@@ -1329,7 +1319,7 @@
 [Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were MEDLINE (Ovid), Embase (Ovid) and the Cochrane
 Central Register of Controlled Trials, 1990 to 2 June 2021. Web of Science was not used.
@@ -1353,13 +1343,13 @@
 [Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/jcsm.13321</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="368" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Geriatric assessment in older patients with a hematologic malignancy: a systematic review</t>
@@ -1397,7 +1387,7 @@
    life; mortality.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>[MEDLINE, searched 4 March 2019 and updated 20 January 2020; results limited to
 studies published after 1 January 2013. Reported in native PubMed syntax as a single
@@ -1418,7 +1408,7 @@
 frail*/vulnerabl*; there are no ADL, IADL or physical-function terms.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Searched, but no separate Embase string was published. The Methods state that "the
 following search was performed ... in both MEDLINE and EMBASE" and then give one
@@ -1426,7 +1416,7 @@
 by database (832 citations from MEDLINE, 3797 from EMBASE, 4629 total).</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were MEDLINE and EMBASE only, supplemented by
 cross-referencing the reference lists of included studies and by carrying forward
@@ -1440,9 +1430,9 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Rows 3, 4: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Rows 3, 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1565,7 @@
    adverse events.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>[PubMed searched natively (via NCBI); 1980 to 29 September 2015. Appendix 6, verbatim:]
 #1  neoplasm*[MeSH Terms]
@@ -1646,7 +1636,7 @@
 23 21 not 22]</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>[Embase via OvidSP, 1980 to 29 September 2015. Appendix 3, verbatim:]
 1  exp neoplasm/
@@ -1683,7 +1673,7 @@
 title, device manufacturer, drug manufacturer, device trade name, keyword.</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL, MEDLINE (OvidSP), Embase (OvidSP),
 PsycINFO (OvidSP), CINAHL (EBSCO) and PubMed, 1980 to 29 September 2015, plus trial
@@ -1713,32 +1703,32 @@
       </c>
     </row>
     <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Long-term neurocognitive and other side effects of radiotherapy, with or without chemotherapy, for glioma</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Lawrie TA, 2019</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Cochrane Database of Systematic Reviews</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>8.4 (2023 JIF, Cochrane Library)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>To evaluate the long-term (at least two years after diagnosis) neurocognitive and other side effects of radiotherapy, with or without chemotherapy, in people with glioma, and to write a brief economic commentary. Included as an exemplar of the alternative structure: rather than a stand-alone cognition block, cognit* is one term inside a generic late-effects adjacency, so cognition is retrieved as a species of treatment harm.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>P: People with glioma (any grade), followed at least two years from diagnosis.
 I: Radiotherapy, with or without chemotherapy.
@@ -1747,7 +1737,7 @@
    life; survival; costs (brief economic commentary).</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1946 to October week 5 2018; searched
 16 February 2018 and updated 14 November 2018. Appendix 1, verbatim:]
@@ -1797,7 +1787,7 @@
 filter for the economic commentary.]</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to 2018 week 46. Appendix 1, verbatim:]
 1  exp Glioma/
@@ -1844,7 +1834,7 @@
 [A parallel Embase run substituted a health-economics filter for lines 21-37.]</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL (2018, Issue 11), MEDLINE via Ovid and
 Embase via Ovid, plus ClinicalTrials.gov and the WHO ICTRP for ongoing trials.
@@ -1877,13 +1867,13 @@
 #22 #14 AND #21]</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD013047.pub2</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="264.5" customHeight="1">
+    <row r="5" ht="333.96" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Meta-analysis of cognitive functioning in breast cancer survivors previously treated with standard-dose chemotherapy</t>
@@ -1920,7 +1910,7 @@
    ability, memory, executive function, processing speed, attention, visuospatial).</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>[PubMed searched natively; studies published 1937 to June 2011; English only.
 Seven search-term sets, verbatim from the Methods:]
@@ -1939,7 +1929,7 @@
 exactly as published.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were PubMed, PsycINFO, CINAHL and the Cochrane
 Library.
@@ -1952,7 +1942,7 @@
 a different spelling variant.]</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were PubMed, PsycINFO, CINAHL and the Cochrane
 Library only.</t>
@@ -1965,7 +1955,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Rows 3, 4: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
         </is>
@@ -2061,7 +2051,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="322" customHeight="1">
+    <row r="3" ht="406.5600000000001" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Exercise Interventions for Depression, Anxiety, and Quality of Life in Older Adults With Cancer: A Systematic Review and Meta-Analysis</t>
@@ -2096,7 +2086,7 @@
 O: Depression severity; anxiety severity; health-related quality of life (HRQOL).</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>[PubMed searched natively, database inception to 5 November 2024.
 eTable 1 in Supplement 1, verbatim:]
@@ -2112,7 +2102,7 @@
 quotes are replaced with straight double quotes.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>[Embase, database inception to 5 November 2024. eTable 1, verbatim:]
 #1 'geriatrics'/exp OR 'aged'/exp OR 'aging'/exp OR 'senescence'/exp
@@ -2127,7 +2117,7 @@
 before reuse.</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were PubMed, Embase, PsycINFO and the Cochrane
 Library, from inception to 5 November 2024.
@@ -2155,32 +2145,32 @@
       </c>
     </row>
     <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Antidepressants for the treatment of depression in people with cancer</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Vita G, 2023</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Cochrane Database of Systematic Reviews</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>8.4 (2023 JIF, Cochrane Library)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>To evaluate the efficacy, tolerability and acceptability of antidepressants for treating depressive symptoms in adults (18 years or older) with cancer of any site and stage. Included as the reference-standard structure for this outcome: population AND depression AND antidepressant, where the depression block pairs three MeSH terms with one adjacency that catches adjustment, reactive and dysthymic disorders, and the drug block names roughly 70 individual agents alongside five exploded drug classes.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>P: Adults (&gt;= 18 years) with any primary cancer diagnosis and depression (major
    depressive disorder, adjustment disorder, dysthymic disorder, or depressive
@@ -2192,7 +2182,7 @@
    reason).</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1946 to November 2022; latest search date
 24 November 2022. Appendix 2, verbatim:]
@@ -2249,7 +2239,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to November 2022. Appendix 3, verbatim:]
 1  exp neoplasm/
@@ -2295,7 +2285,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL (2022, Issue 11), MEDLINE Ovid,
 Embase Ovid and PsycINFO Ovid, all to November 2022, supplemented by handsearching
@@ -2319,7 +2309,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD011006.pub4</t>
         </is>
@@ -2361,7 +2351,7 @@
    others), short- and long-term.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. Ovid MEDLINE, publications 1 January 1980 to 5 July 2023;
 strategy built by a research librarian. eTable 1 in Supplement 1, verbatim
@@ -2405,7 +2395,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_kulchycki2024_aerobic-activity-depression.txt]</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1 January 1980 to 5 July 2023. eTable 1, verbatim (population and
 depression blocks; exercise block lines 8-19, design filter lines 20-29):]
@@ -2436,7 +2426,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_kulchycki2024_aerobic-activity-depression.txt]</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Web of Science was not searched. Scopus was used as the citation-index equivalent,
 alongside MEDLINE, Embase, CENTRAL, CINAHL and PsycINFO (1 January 1980 to
@@ -2473,7 +2463,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Rows 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
         </is>
@@ -2605,7 +2595,7 @@
    status; quality of life; gastrointestinal function; mortality.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. Medline via Ovid, 1946 to July week 4 2012.
 Appendix 2, verbatim:]
@@ -2662,7 +2652,7 @@
 (Line 38 is printed as "7 and 25 and 29 and 37~" with a stray tilde.)</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to 2012 week 31. Appendix 3, verbatim:]
 1  perioperative period/
@@ -2717,7 +2707,7 @@
 44 42 not 43</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were the Cochrane Gynaecological Cancer Group
 Specialised Register, CENTRAL (2012, Issue 7), Medline (1946 to July week 4 2012),
@@ -2769,32 +2759,32 @@
       </c>
     </row>
     <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Prevalence of and Survival with Cachexia among Patients with Cancer: A Systematic Review and Meta-Analysis</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Takaoka T, 2024</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Advances in Nutrition</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>8.0 (2023 JIF)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>To quantify how the reported prevalence of cachexia in patients with cancer varies by diagnostic criterion, and to estimate the association between cachexia and overall survival. Included because it is the only review in this collection that publishes a complete Web of Science strategy, set out side by side with the PubMed version so the MeSH-to-TS= translation is visible line for line.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>P: Patients with cancer (any type, any stage).
 I/E: Presence of cachexia, diagnosed by any published definitive criterion
@@ -2803,7 +2793,7 @@
 O: Prevalence of cachexia by diagnostic criterion; overall survival.</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>[PubMed searched natively, inception to 31 July 2023. Supplemental Table 2, verbatim
 (result counts as printed):]
@@ -2829,13 +2819,13 @@
 truncation on Cancer/Tumor. Sensitivity was traded for a manageable yield.</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Only PubMed and Web of Science were searched, from inception to
 31 July 2023, by a single researcher.</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>[Web of Science searched, inception to 31 July 2023. Supplemental Table 2, verbatim
 (result counts as printed):]
@@ -2865,7 +2855,7 @@
 "epidemiologic(al)" must both be entered.</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.advnut.2024.100282</t>
         </is>
@@ -2910,7 +2900,7 @@
    reactions; survival (overall, disease-free, progression-free).</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>[MEDLINE (PubMed) searched to 30 September 2024; strategy developed with a library
 specialist and set out by PICO element. Supplementary 1, verbatim:]
@@ -2960,7 +2950,7 @@
 translated, not a runnable line-numbered strategy.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Searched, but no Embase-specific string was published. The Methods state that
 "Medical Subject Headings, major topics, and multi-purpose terms were developed" and
@@ -2968,7 +2958,7 @@
 (Supplementary 1).</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Searched (Web of Science Core Collection), but no Web of Science-specific string was
 published. Databases searched were MEDLINE (PubMed), EMBASE, Web of Science Core
@@ -2983,7 +2973,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Rows 3, 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
         </is>
@@ -3116,7 +3106,7 @@
    well-being, pain, fatigue, sleep, body image, vitality; adverse events.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>[MEDLINE searched via PubMed, inception to May 2010 (430 hits) and January 2010 to
 November 2011 (190 hits). Appendix 1, verbatim - lines 32-58 are the HRQoL block:]
@@ -3171,7 +3161,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_mishra2012_hrqol.txt]</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>[Embase, inception to May 2010 (713 hits) and January 2010 to November 2011 (349 hits).
 Appendix 3, verbatim - lines 33-58 are the HRQoL block:]
@@ -3225,7 +3215,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_mishra2012_hrqol.txt]</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Web of Science was used, but for citation searching of key authors rather than with a
 subject strategy, so no Web of Science string exists. As reported: "We also searched
@@ -3249,32 +3239,32 @@
       </c>
     </row>
     <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Health-related quality of life outcomes in randomized controlled trials in metastatic hormone-sensitive prostate cancer: a systematic review</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Osanto S, 2024</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>eClinicalMedicine</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>9.6 (2023 JIF)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>To review how HRQoL was assessed and reported in phase III randomised trials comparing treatment arms in metastatic hormone-sensitive prostate cancer. Included for two reasons: it is one of only two records in this collection with a published Web of Science strategy, and its HRQoL/PRO block is the broadest - it treats anxiety, depression, functional status, fatigue, pain, symptom burden, sexual and social functioning as facets of the same concept, which is exactly the union your review needs across categories 2, 3, 4, 6 and 7.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>P: Patients with metastatic hormone-sensitive prostate cancer (mHSPC).
 I: Systemic treatment arms of phase III RCTs (androgen deprivation therapy alone or
@@ -3286,7 +3276,7 @@
    between-arm difference.</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>[PubMed searched natively; restricted to publications from 1 January 2015.
 Supplementary Table 2, verbatim - the HRQoL/PRO block reproduced in full, the
@@ -3327,7 +3317,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>[Embase (OVID version), same date limits. Supplementary Table 2, verbatim - structure
 reproduced, population block abbreviated:]
@@ -3347,7 +3337,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>[Web of Science searched. Supplementary Table 2, verbatim - the topic block
 reproduced in full, population block abbreviated:]
@@ -3385,7 +3375,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.eclinm.2024.102914</t>
         </is>
@@ -3427,7 +3417,7 @@
    symptoms (fatigue, sleep disturbance); adverse events.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>[MEDLINE searched via PubMed on 29 January 2016. Appendix 1, verbatim:]
 #1  yoga [mh]
@@ -3469,7 +3459,7 @@
 There is no HRQoL, mental-health or symptom block.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>[Embase searched 29 January 2016. Appendix 2 gives two versions.
 Embase.com syntax, verbatim:]
@@ -3533,7 +3523,7 @@
 ("yora" in line 30 is a typo for yoga.)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were the Cochrane Breast Cancer Specialised Register,
 MEDLINE via PubMed (Appendix 1), Embase (Appendix 2), CENTRAL 2016 Issue 1
@@ -3561,7 +3551,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Rows 3, 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
         </is>
@@ -3657,7 +3647,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="241.5" customHeight="1">
+    <row r="3" ht="304.92" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Recommended patient-reported core set of symptoms to measure in adult cancer treatment trials</t>
@@ -3695,7 +3685,7 @@
    disease or to anticancer treatment.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>[Reported in full in the Literature Review section, verbatim:]
 "Search terms included 'multiple symptoms' and 'cancer' and was limited to adults
@@ -3710,13 +3700,13 @@
 symptoms are an output of the review; none of them is an input to the search.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Not reported. No database is named in the paper; the search is described only by the
 two terms above, and the underlying review is cited to Reilly 2013.</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not reported. See above.</t>
         </is>
@@ -3728,32 +3718,32 @@
       </c>
     </row>
     <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Patient-Reported Outcome Measures in Cancer Care: An Updated Systematic Review and Meta-Analysis</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Balitsky AK, 2024</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>JAMA Network Open</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>10.5 (2023 JIF)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>To determine whether integrating patient-reported outcome measures into cancer care is associated with patient-related, therapy-related and health-care-utilisation outcomes. Included because it is the best-documented symptom-adjacent strategy at this impact level: an information specialist's line-numbered strategies for five databases, run twice (an original search and a 2022 update), with per-database yields reported. The symptom concept is expressed at one level of abstraction - "patient reported outcome(s)" AND (inventory or instrument* or measure* or self-report*) - rather than by naming symptoms.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>P: Adults (&gt;= 18 years) with active cancer receiving anticancer therapy (survivors
    excluded).
@@ -3765,7 +3755,7 @@
    survival); health care utilisation (emergency visits, hospital admissions).</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. Ovid MEDLINE and MEDLINE Epub Ahead of Print, In-Process and
 other non-indexed citations, 1946 to present; searches to 26 September 2022.
@@ -3813,7 +3803,7 @@
 [Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>[Embase via OvidSP, 1974 to 2021 (original search) and 1996 to 23 September 2022
 (update). eAppendix in Supplement 1, verbatim (population and PRO blocks; the
@@ -3850,7 +3840,7 @@
 [Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were MEDLINE and MEDLINE Epub ahead of print
 (OvidSP), Embase (OvidSP), PsycINFO (OvidSP), CENTRAL and CINAHL (EBSCO), from
@@ -3872,13 +3862,13 @@
 [Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1001/jamanetworkopen.2024.24793</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="391" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Telephone interventions for symptom management in adults with cancer</t>
@@ -3914,7 +3904,7 @@
    nausea and others; symptom clusters; quality of life; adverse events.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid. Appendix 2, verbatim:]
 1  exp Neoplasms/
@@ -3945,7 +3935,7 @@
 no symptom block.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid. Appendix 3, verbatim:]
 1  exp Neoplasm/
@@ -3971,7 +3961,7 @@
 20 19 and 13 and 5</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL, MEDLINE (Ovid), Embase (Ovid),
 PsycINFO, CINAHL and British Nursing Index, plus trial registries and reference
@@ -4001,9 +3991,9 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Rows 4: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Rows 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4124,7 @@
    experience (e.g. satisfaction with care).</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>[PubMed/MEDLINE searched natively. Search strategy printed in the Appendix, verbatim -
 four sets combined as 1 AND 2 AND 3 AND 4:]
@@ -4167,13 +4157,13 @@
 The full four-set strategy returns 846 records.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Not reported. Only a PubMed/MEDLINE strategy is printed. The review states the search
 was supplemented by expert input on relevant publications.</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Not reported. See above.</t>
         </is>
@@ -4185,32 +4175,32 @@
       </c>
     </row>
     <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Effectiveness and cost-effectiveness of home palliative care services for adults with advanced illness and their caregivers</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Gomes B, 2013</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Cochrane Database of Systematic Reviews</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>8.4 (2023 JIF, Cochrane Library)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>To quantify the effect of home palliative care services on dying at home, and to examine their effect on other patient and caregiver outcomes including symptom control, quality of life, caregiver distress and satisfaction with care, together with resource use, costs and cost-effectiveness. Included as the large-scale contrast: satisfaction with care is named in objective 2, twelve databases were searched, and not one of the strategies contains a satisfaction term.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>P: Adults with advanced illness (the majority of included participants had cancer)
    and their family caregivers.
@@ -4221,7 +4211,7 @@
    cost-effectiveness.</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1950 to 21 November 2012; strategies
 refined with the Cochrane PaPaS Trials Search Co-ordinator. Appendix 1, verbatim
@@ -4277,7 +4267,7 @@
 [Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>[EMBASE, 1980 to 21 November 2012. Appendix 5, verbatim (population/setting blocks;
 design filter from line 25):]
@@ -4319,7 +4309,7 @@
 [Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Twelve databases were searched: CENTRAL (21 November 2012), EMBASE
 (1980 to 21 November 2012), MEDLINE (1950 to 21 November 2012), the Cochrane PaPaS
@@ -4335,13 +4325,13 @@
 [Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD007760.pub2</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="379.5" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Factors influencing cancer patients' experiences of care in the USA, United Kingdom and Canada: A systematic review</t>
@@ -4381,7 +4371,7 @@
    Survey (AOPSS).</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>[PubMed searched, no year restriction, English only; last search 27 February 2022.
 Table 1, verbatim - three parallel searches, one per survey instrument:]
@@ -4400,12 +4390,12 @@
 parenthesise if you port it.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Only PubMed, Web of Science and Google Scholar were used.</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>[Web of Science searched, all years, English. Table 1, verbatim - three parallel
 searches, one per survey instrument:]
@@ -4434,9 +4424,9 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Rows 3, 4: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Rows 3, 4, 5: some cells are longer than Excel's maximum row height (409.5 pt) allows it to display. The cell content is complete - click the cell and read the formula bar, or use docs/tables/*.md and strategies/*.txt for the full text.</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4502,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="57.5" customHeight="1">
+    <row r="3" ht="72.60000000000001" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>A Systematic Review of Health-Related Quality of Life Reporting in Ovarian Cancer Phase III Clinical Trials</t>
@@ -4549,44 +4539,44 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="46" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="4" ht="58.08000000000001" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Nutritional Interventions to Improve Clinical Outcomes in Ovarian Cancer: A Systematic Review of Randomized Controlled Trials</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Rinninella E, 2019</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Nutrients</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>~4.8</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Ovarian cancer specific and nutrition specific. Would have given category 5 a second ovarian record alongside Billson 2013, and a more recent one.</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>JIF ~4.8, just below the 5 threshold</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/nu11061404</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1">
+    <row r="5" ht="58.08000000000001" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Depression and anxiety in ovarian cancer: a systematic review and meta-analysis of prevalence rates</t>
@@ -4623,44 +4613,44 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="6" ht="58.08000000000001" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Functional recovery in older women undergoing surgery for gynaecological malignancies: A systematic review and meta-analysis</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Martin FE, 2020</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Journal of Geriatric Oncology</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>~3.0</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Older women, gynaecological cancer, surgical treatment, functional status. On paper this is the single best population-and-outcome match to your review in the entire candidate pool - it fails only on impact factor.</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>JIF ~3.0</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.jgo.2020.06.006</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="46" customHeight="1">
+    <row r="7" ht="58.08000000000001" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Quality of life outcomes following surgery for advanced ovarian cancer: a systematic review and meta-analysis</t>
@@ -4697,44 +4687,44 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="8" ht="58.08000000000001" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Ovarian cancer survivors' quality of life: a systematic review</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Ahmed-Lecheheb D, 2016</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Journal of Cancer Survivorship</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>~3.4</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Ovarian cancer specific HRQOL review covering the survivorship phase, which the records on sheet 6 do not.</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>JIF ~3.4</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s11764-016-0525-8</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1">
+    <row r="9" ht="58.08000000000001" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>A systematic review of patient values, preferences and expectations for the treatment of recurrent ovarian cancer</t>
@@ -4771,44 +4761,44 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="10" ht="58.08000000000001" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Psychosocial interventions and quality of life in gynaecological cancer patients: a systematic review</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Hersch J, 2009</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Psycho-Oncology</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>~3.3</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Gynaecological cancer with HRQOL and psychological outcomes - closer in population to your review than the breast and prostate cancer records that occupy sheet 6.</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>JIF ~3.3</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/pon.1443</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
+    <row r="11" ht="58.08000000000001" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Patient-Reported Physical Function Measures in Cancer Clinical Trials</t>
@@ -4845,38 +4835,38 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="12" ht="58.08000000000001" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Effects of patient navigation on satisfaction with cancer care: a systematic review and meta-analysis</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Wells KJ, 2018</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Supportive Care in Cancer</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>~2.8</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>The most on-topic satisfaction review found anywhere - satisfaction with cancer care is the outcome, not a secondary endpoint. Directly relevant to category 8.</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>JIF ~2.8</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1007/s00520-018-4108-2</t>
         </is>

</xml_diff>

<commit_message>
Split PICO into four columns: Population, Intervention/exposure, Comparison, Outcome
Done as a data migration in data/NN_*.yml rather than a parse at render time, so
the four elements are now first-class fields (pico_p, pico_i, pico_c, pico_o) and
the single combined pico field is gone.

All 24 records used exactly P / I / C / O in order - three with I/E for
intervention-or-exposure, which is why the column is headed 'I - Intervention /
exposure'. Verified word for word against the pre-migration copies in git: the
round-trip is identical for all 24 records, nothing lost or reordered.

The workbook now has 13 columns; the Markdown tables render PICO as a small
labelled table per record. Fonts unchanged at Arial 11 across all 510 cells.
</commit_message>
<xml_diff>
--- a/output/search_strategies.xlsx
+++ b/output/search_strategies.xlsx
@@ -18,14 +18,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Annex - excluded by IF rule" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Functional status'!$A$2:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 Cognition'!$A$2:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 Depression'!$A$2:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5 Nutritional status'!$A$2:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6 HRQOL'!$A$2:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'7 Patients'' symptoms'!$A$2:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'8 Patients'' satisfaction'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 OC treatment (general)'!$A$2:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Functional status'!$A$2:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 Cognition'!$A$2:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 Depression'!$A$2:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'5 Nutritional status'!$A$2:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'6 HRQOL'!$A$2:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'7 Patients'' symptoms'!$A$2:$M$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'8 Patients'' satisfaction'!$A$2:$M$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'9 Annex - excluded by IF rule'!$A$2:$G$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -497,11 +497,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -539,25 +542,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PICO</t>
+          <t>P - Population</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>I - Intervention / exposure</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C - Comparison</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>O - Outcome</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Search terms / strings - PubMed / MEDLINE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Embase</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Web of Science</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -591,14 +609,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Women with advanced (FIGO stage III/IV) epithelial ovarian cancer.
-I: Platinum-based chemotherapy before cytoreductive surgery (neoadjuvant chemotherapy).
-C: Platinum-based chemotherapy following cytoreductive surgery (primary debulking surgery).
-O: Overall survival; progression-free survival; adverse events; quality of life;
-   surgical morbidity/mortality.</t>
+          <t>Women with advanced (FIGO stage III/IV) epithelial ovarian cancer.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Platinum-based chemotherapy before cytoreductive surgery (neoadjuvant chemotherapy).</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Platinum-based chemotherapy following cytoreductive surgery (primary debulking surgery).</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Overall survival; progression-free survival; adverse events; quality of life; surgical morbidity/mortality.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE was searched via Silver Platter/Ovid,
 1966 to October week 1 2020; searches run 9 October 2020. Appendix 2, verbatim:]
@@ -633,7 +662,7 @@
 or investigation*) and (advanced or stage III or stage IV)]</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to 2020 week 40; searches run 9 October 2020.
 Appendix 1, verbatim:]
@@ -672,7 +701,7 @@
 or investigation*) and (advanced or stage III or stage IV)]</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL (2020, Issue 10), Embase via Ovid,
 MEDLINE (Silver Platter/Ovid), PDQ and MetaRegister; reference lists and trial
@@ -694,7 +723,7 @@
 #14 (#3 AND #9 AND #13)]</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD005343.pub6</t>
         </is>
@@ -728,15 +757,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>P: Women with borderline (low malignant potential) ovarian tumours.
-I: Any intervention for treatment - surgery (including fertility-sparing and
-   radical), chemotherapy, radiotherapy.
-C: An alternative intervention, or observation/no further treatment.
-O: Overall survival; recurrence/disease-free survival; fertility outcomes;
-   adverse events; quality of life.</t>
+          <t>Women with borderline (low malignant potential) ovarian tumours.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Any intervention for treatment - surgery (including fertility-sparing and radical), chemotherapy, radiotherapy.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>An alternative intervention, or observation/no further treatment.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Overall survival; recurrence/disease-free survival; fertility outcomes; adverse events; quality of life.</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1950 to week 3 2009. Appendix 1, verbatim:]
 1  exp Ovarian Neoplasms/
@@ -775,7 +814,7 @@
 word; ab = abstract; fs = floating subheading.</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to 2009 week 2. Appendix 2, verbatim:]
 1  Ovary Tumor/
@@ -816,7 +855,7 @@
 dt (drug therapy), su (surgery), th (therapy) and rt (radiotherapy).</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were the Cochrane Gynaecological Cancer Group
 Trials Register, CENTRAL, MEDLINE and EMBASE, plus reference lists and trial
@@ -836,7 +875,7 @@
 #12 (#10 OR #11)]</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD007696.pub2</t>
         </is>
@@ -870,16 +909,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P: Women with advanced (FIGO stage III/IV) epithelial ovarian cancer undergoing
-   primary cytoreductive surgery.
-I: Primary cytoreductive surgery achieving a given level of residual disease
-   (e.g. microscopic / &lt; 1 cm / optimal).
-C: Primary cytoreductive surgery achieving a greater level of residual disease
-   (e.g. suboptimal, &gt; 1 cm).
-O: Overall survival; progression-free survival; adverse events; quality of life.</t>
+          <t>Women with advanced (FIGO stage III/IV) epithelial ovarian cancer undergoing primary cytoreductive surgery.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Primary cytoreductive surgery achieving a given level of residual disease (e.g. microscopic / &lt; 1 cm / optimal).</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Primary cytoreductive surgery achieving a greater level of residual disease (e.g. suboptimal, &gt; 1 cm).</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Overall survival; progression-free survival; adverse events; quality of life.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1950 to July week 3 2010
 (databases searched to August 2010). Appendix 1, verbatim:]
@@ -917,7 +965,7 @@
 word; fs = floating subheading; pt = publication type.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to week 30 2010. Appendix 2, verbatim:]
 1  exp Ovary Tumor/
@@ -949,7 +997,7 @@
 title, device manufacturer, drug manufacturer name; fs = floating subheading.</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were the Cochrane Gynaecological Cancer
 Collaborative Review Group Trials Register, CENTRAL (The Cochrane Library 2010,
@@ -974,7 +1022,7 @@
 #16 (#8 AND #12 AND #15)]</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD007565.pub2</t>
         </is>
@@ -988,10 +1036,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:M5"/>
   <mergeCells count="2">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1003,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1011,11 +1059,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1053,25 +1104,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PICO</t>
+          <t>P - Population</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>I - Intervention / exposure</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C - Comparison</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>O - Outcome</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Search terms / strings - PubMed / MEDLINE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Embase</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Web of Science</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -1105,14 +1171,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Adults with cancer (any type, any stage, any treatment setting).
-I: Nil - the review deliberately has no intervention concept.
-C: Nil.
-O: Disability in activities of daily living (ADL) and instrumental activities of daily
-   living (IADL) - prevalence, affected items, and measurement instruments.</t>
+          <t>Adults with cancer (any type, any stage, any treatment setting).</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Nil - the review deliberately has no intervention concept.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Nil.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Disability in activities of daily living (ADL) and instrumental activities of daily living (IADL) - prevalence, affected items, and measurement instruments.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE(R) via Ovid, 1946 to June 2016; search alerts run to
 November 2016. Online supplement, Appendix 1, verbatim - the review labels this the
@@ -1162,7 +1239,7 @@
 prospective/correlational studies.</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Searched, but no Embase-specific string was published. The Methods state that the
 strategy "was developed for MEDLINE and adapted where necessary for all other
@@ -1172,7 +1249,7 @@
 Sociological Abstracts, Scopus and Web of Science Core Collection.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Searched (Web of Science Core Collection, and Web of Science Conference Proceedings
 for grey literature), but no Web of Science-specific string was published - only the
@@ -1183,7 +1260,7 @@
 one of two that searched it without publishing the string.</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.ctrv.2017.10.006</t>
         </is>
@@ -1217,15 +1294,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>P: Adults (&gt;= 18 years) with cancer cachexia.
-I: Any cachexia intervention lasting more than 14 days (nutritional, pharmacological,
-   exercise, multimodal), in controlled trials with more than 40 participants.
-C: Control arm as defined by each trial.
-O: Physical function endpoints - handgrip strength, 6-minute walk test, timed
-   up-and-go, physical activity, patient-reported physical function.</t>
+          <t>Adults (&gt;= 18 years) with cancer cachexia.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Any cachexia intervention lasting more than 14 days (nutritional, pharmacological, exercise, multimodal), in controlled trials with more than 40 participants.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Control arm as defined by each trial.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Physical function endpoints - handgrip strength, 6-minute walk test, timed up-and-go, physical activity, patient-reported physical function.</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. Ovid MEDLINE(R) ALL 1946 to 1 July 2021; search run
 2 June 2021 by a research librarian, University of Oslo. Appendix S1, verbatim:]
@@ -1269,7 +1356,7 @@
 [Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>[Embase Classic+Embase 1947 to 1 July 2021 via Ovid; run 2 June 2021.
 Appendix S1, verbatim (population/condition block; the design block is a long
@@ -1319,7 +1406,7 @@
 [Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were MEDLINE (Ovid), Embase (Ovid) and the Cochrane
 Central Register of Controlled Trials, 1990 to 2 June 2021. Web of Science was not used.
@@ -1343,7 +1430,7 @@
 [Complete unabbreviated strategy, all databases: strategies/02_mcdonald2023_cachexia-physical-function.txt]</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/jcsm.13321</t>
         </is>
@@ -1377,17 +1464,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P: Older patients with a haematologic malignancy (leukaemia, lymphoma, multiple
-   myeloma, myelodysplastic syndrome, myeloproliferative neoplasms).
-I: Geriatric assessment (any validated multidomain instrument), applied before or
-   during antineoplastic treatment.
-C: No geriatric assessment, or patients without the impairment identified.
-O: Prevalence of geriatric impairments; treatment decision-making; chemotherapy
-   toxicity; healthcare utilisation; physical functioning after treatment; quality of
-   life; mortality.</t>
+          <t>Older patients with a haematologic malignancy (leukaemia, lymphoma, multiple myeloma, myelodysplastic syndrome, myeloproliferative neoplasms).</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Geriatric assessment (any validated multidomain instrument), applied before or during antineoplastic treatment.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>No geriatric assessment, or patients without the impairment identified.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Prevalence of geriatric impairments; treatment decision-making; chemotherapy toxicity; healthcare utilisation; physical functioning after treatment; quality of life; mortality.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>[MEDLINE, searched 4 March 2019 and updated 20 January 2020; results limited to
 studies published after 1 January 2013. Reported in native PubMed syntax as a single
@@ -1408,7 +1503,7 @@
 frail*/vulnerabl*; there are no ADL, IADL or physical-function terms.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Searched, but no separate Embase string was published. The Methods state that "the
 following search was performed ... in both MEDLINE and EMBASE" and then give one
@@ -1416,14 +1511,14 @@
 by database (832 citations from MEDLINE, 3797 from EMBASE, 4629 total).</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were MEDLINE and EMBASE only, supplemented by
 cross-referencing the reference lists of included studies and by carrying forward
 eligible studies from the earlier 2013 review by Hamaker et al.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.3324/haematol.2019.245803</t>
         </is>
@@ -1437,10 +1532,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:M5"/>
   <mergeCells count="2">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1452,7 +1547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1460,11 +1555,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -1502,25 +1600,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PICO</t>
+          <t>P - Population</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>I - Intervention / exposure</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C - Comparison</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>O - Outcome</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Search terms / strings - PubMed / MEDLINE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Embase</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Web of Science</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -1554,18 +1667,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Adults with cancer receiving or having received systemic cancer treatment
-   (chemotherapy or hormonal therapy, alone or with other treatments).
-I: Non-pharmacological interventions targeting cognitive function (compensatory
-   strategy training, cognitive rehabilitation/training, exercise, mind-body).
-C: Wait-list, usual care, attention control or an alternative non-pharmacological
-   intervention.
-O: Objective and subjective cognitive function; non-cognitive effects (quality of
-   life, physical and psychological well-being, fatigue, mood); duration of effect;
-   adverse events.</t>
+          <t>Adults with cancer receiving or having received systemic cancer treatment (chemotherapy or hormonal therapy, alone or with other treatments).</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Non-pharmacological interventions targeting cognitive function (compensatory strategy training, cognitive rehabilitation/training, exercise, mind-body).</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Wait-list, usual care, attention control or an alternative non-pharmacological intervention.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Objective and subjective cognitive function; non-cognitive effects (quality of life, physical and psychological well-being, fatigue, mood); duration of effect; adverse events.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>[PubMed searched natively (via NCBI); 1980 to 29 September 2015. Appendix 6, verbatim:]
 #1  neoplasm*[MeSH Terms]
@@ -1636,7 +1756,7 @@
 23 21 not 22]</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>[Embase via OvidSP, 1980 to 29 September 2015. Appendix 3, verbatim:]
 1  exp neoplasm/
@@ -1673,7 +1793,7 @@
 title, device manufacturer, drug manufacturer, device trade name, keyword.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL, MEDLINE (OvidSP), Embase (OvidSP),
 PsycINFO (OvidSP), CINAHL (EBSCO) and PubMed, 1980 to 29 September 2015, plus trial
@@ -1696,7 +1816,7 @@
 S50 (S47 or S48 or S49) S51 (S44 and S50)]</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD011325.pub2</t>
         </is>
@@ -1730,14 +1850,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>P: People with glioma (any grade), followed at least two years from diagnosis.
-I: Radiotherapy, with or without chemotherapy.
-C: No radiotherapy, or a different type/dose/schedule of radiotherapy.
-O: Long-term neurocognitive function (primary); other late side effects; quality of
-   life; survival; costs (brief economic commentary).</t>
+          <t>People with glioma (any grade), followed at least two years from diagnosis.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Radiotherapy, with or without chemotherapy.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>No radiotherapy, or a different type/dose/schedule of radiotherapy.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Long-term neurocognitive function (primary); other late side effects; quality of life; survival; costs (brief economic commentary).</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1946 to October week 5 2018; searched
 16 February 2018 and updated 14 November 2018. Appendix 1, verbatim:]
@@ -1787,7 +1918,7 @@
 filter for the economic commentary.]</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to 2018 week 46. Appendix 1, verbatim:]
 1  exp Glioma/
@@ -1834,7 +1965,7 @@
 [A parallel Embase run substituted a health-economics filter for lines 21-37.]</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL (2018, Issue 11), MEDLINE via Ovid and
 Embase via Ovid, plus ClinicalTrials.gov and the WHO ICTRP for ongoing trials.
@@ -1867,7 +1998,7 @@
 #22 #14 AND #21]</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD013047.pub2</t>
         </is>
@@ -1901,16 +2032,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P: Women who had completed standard-dose chemotherapy for breast cancer at least
-   six months previously.
-I: Standard-dose chemotherapy (past exposure).
-C: Healthy controls, patients not treated with chemotherapy, or the patient's own
-   pre-treatment/normative scores.
-O: Objective neuropsychological test performance across cognitive domains (verbal
-   ability, memory, executive function, processing speed, attention, visuospatial).</t>
+          <t>Women who had completed standard-dose chemotherapy for breast cancer at least six months previously.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Standard-dose chemotherapy (past exposure).</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Healthy controls, patients not treated with chemotherapy, or the patient's own pre-treatment/normative scores.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Objective neuropsychological test performance across cognitive domains (verbal ability, memory, executive function, processing speed, attention, visuospatial).</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>[PubMed searched natively; studies published 1937 to June 2011; English only.
 Seven search-term sets, verbatim from the Methods:]
@@ -1929,7 +2069,7 @@
 exactly as published.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were PubMed, PsycINFO, CINAHL and the Cochrane
 Library.
@@ -1942,13 +2082,13 @@
 a different spelling variant.]</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were PubMed, PsycINFO, CINAHL and the Cochrane
 Library only.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1200/JCO.2011.39.5640</t>
         </is>
@@ -1962,10 +2102,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:M5"/>
   <mergeCells count="2">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1977,7 +2117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1985,11 +2125,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2027,25 +2170,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PICO</t>
+          <t>P - Population</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>I - Intervention / exposure</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C - Comparison</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>O - Outcome</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Search terms / strings - PubMed / MEDLINE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Embase</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Web of Science</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -2079,14 +2237,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Older adults with cancer (mean age &gt;= 60 years), any cancer type, any comorbidity.
-I: Exercise interventions - aerobic, resistance and strength training, or mind-body
-   exercise (qigong, yoga, tai chi).
-C: Usual care.
-O: Depression severity; anxiety severity; health-related quality of life (HRQOL).</t>
+          <t>Older adults with cancer (mean age &gt;= 60 years), any cancer type, any comorbidity.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Exercise interventions - aerobic, resistance and strength training, or mind-body exercise (qigong, yoga, tai chi).</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Usual care.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Depression severity; anxiety severity; health-related quality of life (HRQOL).</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>[PubMed searched natively, database inception to 5 November 2024.
 eTable 1 in Supplement 1, verbatim:]
@@ -2102,7 +2271,7 @@
 quotes are replaced with straight double quotes.</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>[Embase, database inception to 5 November 2024. eTable 1, verbatim:]
 #1 'geriatrics'/exp OR 'aged'/exp OR 'aging'/exp OR 'senescence'/exp
@@ -2117,7 +2286,7 @@
 before reuse.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were PubMed, Embase, PsycINFO and the Cochrane
 Library, from inception to 5 November 2024.
@@ -2138,7 +2307,7 @@
 #4 (depress* OR anxi* OR burden* OR stress* OR 'quality of life').ti,ab.]</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1001/jamanetworkopen.2024.57859</t>
         </is>
@@ -2172,17 +2341,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>P: Adults (&gt;= 18 years) with any primary cancer diagnosis and depression (major
-   depressive disorder, adjustment disorder, dysthymic disorder, or depressive
-   symptoms measured on a validated scale).
-I: Any antidepressant.
-C: Placebo, or another antidepressant.
-O: Efficacy (change in depressive symptoms, response, remission); tolerability
-   (adverse events, dropouts due to adverse events); acceptability (dropouts for any
-   reason).</t>
+          <t>Adults (&gt;= 18 years) with any primary cancer diagnosis and depression (major depressive disorder, adjustment disorder, dysthymic disorder, or depressive symptoms measured on a validated scale).</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Any antidepressant.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Placebo, or another antidepressant.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Efficacy (change in depressive symptoms, response, remission); tolerability (adverse events, dropouts due to adverse events); acceptability (dropouts for any reason).</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1946 to November 2022; latest search date
 24 November 2022. Appendix 2, verbatim:]
@@ -2239,7 +2416,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to November 2022. Appendix 3, verbatim:]
 1  exp neoplasm/
@@ -2285,7 +2462,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL (2022, Issue 11), MEDLINE Ovid,
 Embase Ovid and PsycINFO Ovid, all to November 2022, supplemented by handsearching
@@ -2309,7 +2486,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_vita2023_antidepressants.txt]</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD011006.pub4</t>
         </is>
@@ -2343,15 +2520,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P: Patients with any cancer diagnosis, including haematopoietic stem cell transplant
-   recipients.
-I: Aerobic physical activity interventions (randomised controlled trials).
-C: Usual care or non-aerobic control.
-O: Severity of depression on validated self-reported scales (CES-D, HADS, BDI and
-   others), short- and long-term.</t>
+          <t>Patients with any cancer diagnosis, including haematopoietic stem cell transplant recipients.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Aerobic physical activity interventions (randomised controlled trials).</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Usual care or non-aerobic control.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Severity of depression on validated self-reported scales (CES-D, HADS, BDI and others), short- and long-term.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. Ovid MEDLINE, publications 1 January 1980 to 5 July 2023;
 strategy built by a research librarian. eTable 1 in Supplement 1, verbatim
@@ -2395,7 +2582,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_kulchycki2024_aerobic-activity-depression.txt]</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1 January 1980 to 5 July 2023. eTable 1, verbatim (population and
 depression blocks; exercise block lines 8-19, design filter lines 20-29):]
@@ -2426,7 +2613,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_kulchycki2024_aerobic-activity-depression.txt]</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Web of Science was not searched. Scopus was used as the citation-index equivalent,
 alongside MEDLINE, Embase, CENTRAL, CINAHL and PsycINFO (1 January 1980 to
@@ -2456,7 +2643,7 @@
 [Complete unabbreviated strategy, all databases: strategies/04_kulchycki2024_aerobic-activity-depression.txt]</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1001/jamanetworkopen.2024.37964</t>
         </is>
@@ -2470,10 +2657,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:M5"/>
   <mergeCells count="2">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2485,7 +2672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2493,11 +2680,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -2535,25 +2725,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PICO</t>
+          <t>P - Population</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>I - Intervention / exposure</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C - Comparison</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>O - Outcome</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Search terms / strings - PubMed / MEDLINE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Embase</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Web of Science</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -2587,15 +2792,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Women with ovarian cancer undergoing surgery (perioperative period).
-I: Any nutrition intervention - enteral or parenteral nutrition, oral supplements,
-   immunonutrition, early feeding, dietary advice.
-C: Standard perioperative care or an alternative nutrition intervention.
-O: Postoperative complications and infection; length of hospital stay; nutritional
-   status; quality of life; gastrointestinal function; mortality.</t>
+          <t>Women with ovarian cancer undergoing surgery (perioperative period).</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Any nutrition intervention - enteral or parenteral nutrition, oral supplements, immunonutrition, early feeding, dietary advice.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Standard perioperative care or an alternative nutrition intervention.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Postoperative complications and infection; length of hospital stay; nutritional status; quality of life; gastrointestinal function; mortality.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. Medline via Ovid, 1946 to July week 4 2012.
 Appendix 2, verbatim:]
@@ -2652,7 +2867,7 @@
 (Line 38 is printed as "7 and 25 and 29 and 37~" with a stray tilde.)</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid, 1980 to 2012 week 31. Appendix 3, verbatim:]
 1  perioperative period/
@@ -2707,7 +2922,7 @@
 44 42 not 43</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were the Cochrane Gynaecological Cancer Group
 Specialised Register, CENTRAL (2012, Issue 7), Medline (1946 to July week 4 2012),
@@ -2752,7 +2967,7 @@
 Line #24 is printed with "of PN" where "or PN" is meant.]</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD009884.pub2</t>
         </is>
@@ -2786,14 +3001,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>P: Patients with cancer (any type, any stage).
-I/E: Presence of cachexia, diagnosed by any published definitive criterion
-   (Fearon, EPCRC, ASPEN/AND, Evans, GLIM and others).
-C: Patients with cancer without cachexia.
-O: Prevalence of cachexia by diagnostic criterion; overall survival.</t>
+          <t>Patients with cancer (any type, any stage).</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Presence of cachexia, diagnosed by any published definitive criterion (Fearon, EPCRC, ASPEN/AND, Evans, GLIM and others).</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Patients with cancer without cachexia.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Prevalence of cachexia by diagnostic criterion; overall survival.</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>[PubMed searched natively, inception to 31 July 2023. Supplemental Table 2, verbatim
 (result counts as printed):]
@@ -2819,13 +3045,13 @@
 truncation on Cancer/Tumor. Sensitivity was traded for a manageable yield.</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Only PubMed and Web of Science were searched, from inception to
 31 July 2023, by a single researcher.</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>[Web of Science searched, inception to 31 July 2023. Supplemental Table 2, verbatim
 (result counts as printed):]
@@ -2855,7 +3081,7 @@
 "epidemiologic(al)" must both be entered.</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.advnut.2024.100282</t>
         </is>
@@ -2889,18 +3115,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P: Children and young people (&lt; 21 years) with cancer receiving antineoplastic
-   therapy.
-I/E: Antineoplastic drug therapy (chemotherapy, alkylating agents, combination
-   protocols).
-C: Nutritional status groups - undernutrition/sarcopenia versus normal nutrition
-   versus overweight/obesity/sarcopenic obesity, defined by body composition, BMI
-   or nutritional status measures.
-O: Pharmacokinetic and pharmacodynamic parameters; drug toxicity and adverse
-   reactions; survival (overall, disease-free, progression-free).</t>
+          <t>Children and young people (&lt; 21 years) with cancer receiving antineoplastic therapy.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Antineoplastic drug therapy (chemotherapy, alkylating agents, combination protocols).</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Nutritional status groups - undernutrition/sarcopenia versus normal nutrition versus overweight/obesity/sarcopenic obesity, defined by body composition, BMI or nutritional status measures.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Pharmacokinetic and pharmacodynamic parameters; drug toxicity and adverse reactions; survival (overall, disease-free, progression-free).</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>[MEDLINE (PubMed) searched to 30 September 2024; strategy developed with a library
 specialist and set out by PICO element. Supplementary 1, verbatim:]
@@ -2950,7 +3183,7 @@
 translated, not a runnable line-numbered strategy.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Searched, but no Embase-specific string was published. The Methods state that
 "Medical Subject Headings, major topics, and multi-purpose terms were developed" and
@@ -2958,7 +3191,7 @@
 (Supplementary 1).</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Searched (Web of Science Core Collection), but no Web of Science-specific string was
 published. Databases searched were MEDLINE (PubMed), EMBASE, Web of Science Core
@@ -2966,7 +3199,7 @@
 30 September 2024. Only the MEDLINE term list is reproduced.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1038/s41416-025-03023-3</t>
         </is>
@@ -2980,10 +3213,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:M5"/>
   <mergeCells count="2">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2995,7 +3228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3003,11 +3236,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -3045,25 +3281,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PICO</t>
+          <t>P - Population</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>I - Intervention / exposure</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C - Comparison</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>O - Outcome</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Search terms / strings - PubMed / MEDLINE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Embase</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Web of Science</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -3097,16 +3348,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Adults with any cancer, during active treatment (surgery, chemotherapy,
-   radiotherapy, hormonal therapy).
-I: Exercise interventions (aerobic, resistance, combination, mind-body including
-   yoga, tai chi, qigong, hydrotherapy).
-C: Usual care, no exercise, or an alternative non-exercise intervention.
-O: Overall HRQoL and HRQoL domains - physical, psychological, social, spiritual
-   well-being, pain, fatigue, sleep, body image, vitality; adverse events.</t>
+          <t>Adults with any cancer, during active treatment (surgery, chemotherapy, radiotherapy, hormonal therapy).</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Exercise interventions (aerobic, resistance, combination, mind-body including yoga, tai chi, qigong, hydrotherapy).</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Usual care, no exercise, or an alternative non-exercise intervention.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Overall HRQoL and HRQoL domains - physical, psychological, social, spiritual well-being, pain, fatigue, sleep, body image, vitality; adverse events.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>[MEDLINE searched via PubMed, inception to May 2010 (430 hits) and January 2010 to
 November 2011 (190 hits). Appendix 1, verbatim - lines 32-58 are the HRQoL block:]
@@ -3161,7 +3421,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_mishra2012_hrqol.txt]</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>[Embase, inception to May 2010 (713 hits) and January 2010 to November 2011 (349 hits).
 Appendix 3, verbatim - lines 33-58 are the HRQoL block:]
@@ -3215,7 +3475,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_mishra2012_hrqol.txt]</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Web of Science was used, but for citation searching of key authors rather than with a
 subject strategy, so no Web of Science string exists. As reported: "We also searched
@@ -3232,7 +3492,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_mishra2012_hrqol.txt]</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD008465.pub2</t>
         </is>
@@ -3266,17 +3526,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>P: Patients with metastatic hormone-sensitive prostate cancer (mHSPC).
-I: Systemic treatment arms of phase III RCTs (androgen deprivation therapy alone or
-   in combination with docetaxel, abiraterone, apalutamide, enzalutamide, darolutamide
-   or radiotherapy).
-C: The comparator arm of each trial (usually ADT alone).
-O: Health-related quality of life and patient-reported outcomes - instrument used,
-   domains, timing, compliance, statistical handling, and the direction of any
-   between-arm difference.</t>
+          <t>Patients with metastatic hormone-sensitive prostate cancer (mHSPC).</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Systemic treatment arms of phase III RCTs (androgen deprivation therapy alone or in combination with docetaxel, abiraterone, apalutamide, enzalutamide, darolutamide or radiotherapy).</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>The comparator arm of each trial (usually ADT alone).</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Health-related quality of life and patient-reported outcomes - instrument used, domains, timing, compliance, statistical handling, and the direction of any between-arm difference.</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>[PubMed searched natively; restricted to publications from 1 January 2015.
 Supplementary Table 2, verbatim - the HRQoL/PRO block reproduced in full, the
@@ -3317,7 +3585,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>[Embase (OVID version), same date limits. Supplementary Table 2, verbatim - structure
 reproduced, population block abbreviated:]
@@ -3337,7 +3605,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>[Web of Science searched. Supplementary Table 2, verbatim - the topic block
 reproduced in full, population block abbreviated:]
@@ -3375,7 +3643,7 @@
 [Complete unabbreviated strategy, all databases: strategies/06_osanto2024_hrqol-mhspc.txt]</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.eclinm.2024.102914</t>
         </is>
@@ -3409,15 +3677,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P: Women with a diagnosis of breast cancer, receiving active treatment or having
-   completed treatment.
-I: Yoga (including asana, pranayama, dhyana, dharana, meditation).
-C: No therapy, or another active intervention (psychosocial/educational, exercise).
-O: Health-related quality of life; mental health (depression, anxiety); cancer-related
-   symptoms (fatigue, sleep disturbance); adverse events.</t>
+          <t>Women with a diagnosis of breast cancer, receiving active treatment or having completed treatment.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Yoga (including asana, pranayama, dhyana, dharana, meditation).</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>No therapy, or another active intervention (psychosocial/educational, exercise).</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Health-related quality of life; mental health (depression, anxiety); cancer-related symptoms (fatigue, sleep disturbance); adverse events.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>[MEDLINE searched via PubMed on 29 January 2016. Appendix 1, verbatim:]
 #1  yoga [mh]
@@ -3459,7 +3737,7 @@
 There is no HRQoL, mental-health or symptom block.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>[Embase searched 29 January 2016. Appendix 2 gives two versions.
 Embase.com syntax, verbatim:]
@@ -3523,7 +3801,7 @@
 ("yora" in line 30 is a typo for yoga.)</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were the Cochrane Breast Cancer Specialised Register,
 MEDLINE via PubMed (Appendix 1), Embase (Appendix 2), CENTRAL 2016 Issue 1
@@ -3544,7 +3822,7 @@
 #12 #7 and #11]</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD010802.pub2</t>
         </is>
@@ -3558,10 +3836,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:M5"/>
   <mergeCells count="2">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3573,7 +3851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3581,11 +3859,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -3623,25 +3904,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PICO</t>
+          <t>P - Population</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>I - Intervention / exposure</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C - Comparison</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>O - Outcome</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Search terms / strings - PubMed / MEDLINE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Embase</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Web of Science</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -3675,17 +3971,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Adults (&gt;= 18 years) with cancer, across diverse cancer populations and treatment
-   modalities.
-I: Anticancer treatment (any modality) in clinical trials measuring a patient-reported
-   outcome.
-C: Not applicable - this is a core-outcome-set derivation, not a comparative review.
-O: Which symptoms should form a core set, judged on prevalence across cancer
-   populations, impact on health outcomes and quality of life, and attribution to
-   disease or to anticancer treatment.</t>
+          <t>Adults (&gt;= 18 years) with cancer, across diverse cancer populations and treatment modalities.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Anticancer treatment (any modality) in clinical trials measuring a patient-reported outcome.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable - this is a core-outcome-set derivation, not a comparative review.</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Which symptoms should form a core set, judged on prevalence across cancer populations, impact on health outcomes and quality of life, and attribution to disease or to anticancer treatment.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>[Reported in full in the Literature Review section, verbatim:]
 "Search terms included 'multiple symptoms' and 'cancer' and was limited to adults
@@ -3700,18 +4004,18 @@
 symptoms are an output of the review; none of them is an input to the search.</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Not reported. No database is named in the paper; the search is described only by the
 two terms above, and the underlying review is cited to Reilly 2013.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Not reported. See above.</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1093/jnci/dju129</t>
         </is>
@@ -3745,17 +4049,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>P: Adults (&gt;= 18 years) with active cancer receiving anticancer therapy (survivors
-   excluded).
-I: Administration of a patient-reported outcome measure, with results shared with the
-   patient's health care professional.
-C: Standard care without PROM administration.
-O: Patient-related outcomes (HRQOL, symptom control, patient-clinician communication);
-   therapy-related outcomes (treatment adherence, chemotherapy dose modification,
-   survival); health care utilisation (emergency visits, hospital admissions).</t>
+          <t>Adults (&gt;= 18 years) with active cancer receiving anticancer therapy (survivors excluded).</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Administration of a patient-reported outcome measure, with results shared with the patient's health care professional.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Standard care without PROM administration.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Patient-related outcomes (HRQOL, symptom control, patient-clinician communication); therapy-related outcomes (treatment adherence, chemotherapy dose modification, survival); health care utilisation (emergency visits, hospital admissions).</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. Ovid MEDLINE and MEDLINE Epub Ahead of Print, In-Process and
 other non-indexed citations, 1946 to present; searches to 26 September 2022.
@@ -3803,7 +4115,7 @@
 [Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>[Embase via OvidSP, 1974 to 2021 (original search) and 1996 to 23 September 2022
 (update). eAppendix in Supplement 1, verbatim (population and PRO blocks; the
@@ -3840,7 +4152,7 @@
 [Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were MEDLINE and MEDLINE Epub ahead of print
 (OvidSP), Embase (OvidSP), PsycINFO (OvidSP), CENTRAL and CINAHL (EBSCO), from
@@ -3862,7 +4174,7 @@
 [Complete unabbreviated strategy, all databases: strategies/07_balitsky2024_proms.txt]</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1001/jamanetworkopen.2024.24793</t>
         </is>
@@ -3896,15 +4208,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P: Adults (&gt;= 18 years) with cancer, during or after treatment.
-I: Telephone-delivered interventions for symptom management, alone or with additional
-   face-to-face, printed or electronic support.
-C: Usual care or another intervention.
-O: Individual symptoms - anxiety, depression, fatigue, emotional distress, pain,
-   nausea and others; symptom clusters; quality of life; adverse events.</t>
+          <t>Adults (&gt;= 18 years) with cancer, during or after treatment.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Telephone-delivered interventions for symptom management, alone or with additional face-to-face, printed or electronic support.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Usual care or another intervention.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Individual symptoms - anxiety, depression, fatigue, emotional distress, pain, nausea and others; symptom clusters; quality of life; adverse events.</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid. Appendix 2, verbatim:]
 1  exp Neoplasms/
@@ -3935,7 +4257,7 @@
 no symptom block.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>[Embase via Ovid. Appendix 3, verbatim:]
 1  exp Neoplasm/
@@ -3961,7 +4283,7 @@
 20 19 and 13 and 5</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Databases searched were CENTRAL, MEDLINE (Ovid), Embase (Ovid),
 PsycINFO, CINAHL and British Nursing Index, plus trial registries and reference
@@ -3984,7 +4306,7 @@
 #14 (#5 AND #13)]</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD007568.pub2</t>
         </is>
@@ -3998,10 +4320,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:M5"/>
   <mergeCells count="2">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4013,7 +4335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4021,11 +4343,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="62" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -4063,25 +4388,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PICO</t>
+          <t>P - Population</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>I - Intervention / exposure</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C - Comparison</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>O - Outcome</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Search terms / strings - PubMed / MEDLINE</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Embase</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Search terms / strings - Web of Science</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -4115,16 +4455,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>P: Individuals diagnosed with cancer.
-I: Survivor or care-provider receipt of a survivorship care plan (SCP).
-C: No receipt of an SCP, an alternative method of receiving an SCP, or no comparison
-   (for non-randomised studies).
-O: Patient-reported health outcomes (e.g. quality of life); health care use; health
-   care costs; health outcomes (e.g. quality-adjusted life years); and health care
-   experience (e.g. satisfaction with care).</t>
+          <t>Individuals diagnosed with cancer.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Survivor or care-provider receipt of a survivorship care plan (SCP).</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>No receipt of an SCP, an alternative method of receiving an SCP, or no comparison (for non-randomised studies).</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Patient-reported health outcomes (e.g. quality of life); health care use; health care costs; health outcomes (e.g. quality-adjusted life years); and health care experience (e.g. satisfaction with care).</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>[PubMed/MEDLINE searched natively. Search strategy printed in the Appendix, verbatim -
 four sets combined as 1 AND 2 AND 3 AND 4:]
@@ -4157,18 +4506,18 @@
 The full four-set strategy returns 846 records.</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Not reported. Only a PubMed/MEDLINE strategy is printed. The review states the search
 was supplemented by expert input on relevant publications.</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Not reported. See above.</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1200/JCO.2018.77.7482</t>
         </is>
@@ -4202,16 +4551,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>P: Adults with advanced illness (the majority of included participants had cancer)
-   and their family caregivers.
-I: Home palliative care services - specialist teams providing palliative care at home.
-C: Usual care, or care without a home palliative care service.
-O: Dying at home (primary); symptom burden and control; quality of life; caregiver
-   distress and grief; satisfaction with care; resource use, costs and
-   cost-effectiveness.</t>
+          <t>Adults with advanced illness (the majority of included participants had cancer) and their family caregivers.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Home palliative care services - specialist teams providing palliative care at home.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Usual care, or care without a home palliative care service.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Dying at home (primary); symptom burden and control; quality of life; caregiver distress and grief; satisfaction with care; resource use, costs and cost-effectiveness.</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>[Not searched as PubMed. MEDLINE via Ovid, 1950 to 21 November 2012; strategies
 refined with the Cochrane PaPaS Trials Search Co-ordinator. Appendix 1, verbatim
@@ -4267,7 +4625,7 @@
 [Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>[EMBASE, 1980 to 21 November 2012. Appendix 5, verbatim (population/setting blocks;
 design filter from line 25):]
@@ -4309,7 +4667,7 @@
 [Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Not searched. Twelve databases were searched: CENTRAL (21 November 2012), EMBASE
 (1980 to 21 November 2012), MEDLINE (1950 to 21 November 2012), the Cochrane PaPaS
@@ -4325,7 +4683,7 @@
 [Complete unabbreviated strategy, all databases: strategies/08_gomes2013_home-palliative-care.txt]</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1002/14651858.CD007760.pub2</t>
         </is>
@@ -4359,19 +4717,25 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>P: Adults with cancer responding to a national patient-experience survey in the USA,
-   United Kingdom or Canada.
-I/E: Patient, clinical and health-system characteristics (age, sex, ethnicity,
-   socioeconomic position, cancer type and stage, comorbidity, provider and
-   hospital factors).
-C: Patients with the contrasting characteristic within the same survey.
-O: Reported experience of cancer care, as measured by the National Cancer Patient
-   Experience Survey (CPES), the Consumer Assessment of Healthcare Providers and
-   Systems (CAHPS/SEER-CAHPS) or the Ambulatory Oncology Patient Satisfaction
-   Survey (AOPSS).</t>
+          <t>Adults with cancer responding to a national patient-experience survey in the USA, United Kingdom or Canada.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Patient, clinical and health-system characteristics (age, sex, ethnicity, socioeconomic position, cancer type and stage, comorbidity, provider and hospital factors).</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Patients with the contrasting characteristic within the same survey.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Reported experience of cancer care, as measured by the National Cancer Patient Experience Survey (CPES), the Consumer Assessment of Healthcare Providers and Systems (CAHPS/SEER-CAHPS) or the Ambulatory Oncology Patient Satisfaction Survey (AOPSS).</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>[PubMed searched, no year restriction, English only; last search 27 February 2022.
 Table 1, verbatim - three parallel searches, one per survey instrument:]
@@ -4390,12 +4754,12 @@
 parenthesise if you port it.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Not searched. Only PubMed, Web of Science and Google Scholar were used.</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>[Web of Science searched, all years, English. Table 1, verbatim - three parallel
 searches, one per survey instrument:]
@@ -4417,7 +4781,7 @@
 your review needs both, search both vocabularies.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.eclinm.2022.101405</t>
         </is>
@@ -4431,10 +4795,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:M5"/>
   <mergeCells count="2">
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>